<commit_message>
12# X pixel size param
</commit_message>
<xml_diff>
--- a/Sources/Cuga-Calibration-Solution/Assets/Data/InitData.xlsx
+++ b/Sources/Cuga-Calibration-Solution/Assets/Data/InitData.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1714" uniqueCount="406">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1718" uniqueCount="408">
   <si>
     <t>Id</t>
   </si>
@@ -1088,6 +1088,12 @@
   </si>
   <si>
     <t>CugaCalibration.ViewModels.Laser.LaserRtfcCalibrationViewModel</t>
+  </si>
+  <si>
+    <t>Pmt Agc Delay</t>
+  </si>
+  <si>
+    <t>CugaCalibration.ViewModels.Laser.LaserPmtAgcDelayCalibrationViewModel</t>
   </si>
   <si>
     <t>Title</t>
@@ -16748,7 +16754,30 @@
       </c>
       <c r="J315" s="6"/>
     </row>
-    <row r="316" spans="10:10">
+    <row r="316" ht="20.1" customHeight="1" spans="1:10">
+      <c r="A316" s="5">
+        <v>1608</v>
+      </c>
+      <c r="B316" s="6" t="s">
+        <v>351</v>
+      </c>
+      <c r="C316" s="5">
+        <v>16</v>
+      </c>
+      <c r="D316" s="5">
+        <v>1608</v>
+      </c>
+      <c r="E316" s="5"/>
+      <c r="F316" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="G316" s="6" t="s">
+        <v>352</v>
+      </c>
+      <c r="H316" s="6"/>
+      <c r="I316" s="6" t="s">
+        <v>351</v>
+      </c>
       <c r="J316" s="6"/>
     </row>
     <row r="317" ht="20.1" customHeight="1" spans="1:10">
@@ -16756,7 +16785,7 @@
         <v>2</v>
       </c>
       <c r="B317" s="6" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="C317" s="5">
         <v>-1</v>
@@ -16771,7 +16800,7 @@
       <c r="G317" s="6"/>
       <c r="H317" s="6"/>
       <c r="I317" s="6" t="s">
-        <v>351</v>
+        <v>353</v>
       </c>
       <c r="J317" s="6"/>
     </row>
@@ -16780,7 +16809,7 @@
         <v>21</v>
       </c>
       <c r="B318" s="6" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="C318" s="5">
         <v>2</v>
@@ -16795,7 +16824,7 @@
       <c r="G318" s="6"/>
       <c r="H318" s="6"/>
       <c r="I318" s="6" t="s">
-        <v>352</v>
+        <v>354</v>
       </c>
       <c r="J318" s="6"/>
     </row>
@@ -16804,7 +16833,7 @@
         <v>2110</v>
       </c>
       <c r="B319" s="6" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="C319" s="5">
         <v>21</v>
@@ -16817,11 +16846,11 @@
         <v>55</v>
       </c>
       <c r="G319" s="6" t="s">
-        <v>354</v>
+        <v>356</v>
       </c>
       <c r="H319" s="6"/>
       <c r="I319" s="6" t="s">
-        <v>353</v>
+        <v>355</v>
       </c>
       <c r="J319" s="6"/>
     </row>
@@ -16830,7 +16859,7 @@
         <v>2111</v>
       </c>
       <c r="B320" s="6" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="C320" s="5">
         <v>21</v>
@@ -16843,11 +16872,11 @@
         <v>55</v>
       </c>
       <c r="G320" s="6" t="s">
-        <v>356</v>
+        <v>358</v>
       </c>
       <c r="H320" s="6"/>
       <c r="I320" s="6" t="s">
-        <v>355</v>
+        <v>357</v>
       </c>
       <c r="J320" s="6"/>
     </row>
@@ -16856,7 +16885,7 @@
         <v>22</v>
       </c>
       <c r="B321" s="6" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="C321" s="5">
         <v>2</v>
@@ -16871,7 +16900,7 @@
       <c r="G321" s="6"/>
       <c r="H321" s="6"/>
       <c r="I321" s="6" t="s">
-        <v>357</v>
+        <v>359</v>
       </c>
       <c r="J321" s="6"/>
     </row>
@@ -16880,7 +16909,7 @@
         <v>2201</v>
       </c>
       <c r="B322" s="6" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="C322" s="5">
         <v>22</v>
@@ -16893,11 +16922,11 @@
         <v>55</v>
       </c>
       <c r="G322" s="6" t="s">
-        <v>359</v>
+        <v>361</v>
       </c>
       <c r="H322" s="6"/>
       <c r="I322" s="6" t="s">
-        <v>358</v>
+        <v>360</v>
       </c>
       <c r="J322" s="6"/>
     </row>
@@ -16906,7 +16935,7 @@
         <v>2202</v>
       </c>
       <c r="B323" s="6" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="C323" s="5">
         <v>22</v>
@@ -16919,11 +16948,11 @@
         <v>55</v>
       </c>
       <c r="G323" s="6" t="s">
-        <v>361</v>
+        <v>363</v>
       </c>
       <c r="H323" s="6"/>
       <c r="I323" s="6" t="s">
-        <v>360</v>
+        <v>362</v>
       </c>
       <c r="J323" s="6"/>
     </row>
@@ -16932,7 +16961,7 @@
         <v>2203</v>
       </c>
       <c r="B324" s="6" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="C324" s="5">
         <v>22</v>
@@ -16945,11 +16974,11 @@
         <v>55</v>
       </c>
       <c r="G324" s="6" t="s">
-        <v>363</v>
+        <v>365</v>
       </c>
       <c r="H324" s="6"/>
       <c r="I324" s="6" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="J324" s="6"/>
     </row>
@@ -16958,7 +16987,7 @@
         <v>23</v>
       </c>
       <c r="B325" s="6" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="C325" s="5">
         <v>2</v>
@@ -16973,7 +17002,7 @@
       <c r="G325" s="6"/>
       <c r="H325" s="6"/>
       <c r="I325" s="6" t="s">
-        <v>364</v>
+        <v>366</v>
       </c>
       <c r="J325" s="6"/>
     </row>
@@ -16982,7 +17011,7 @@
         <v>2301</v>
       </c>
       <c r="B326" s="6" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="C326" s="5">
         <v>23</v>
@@ -16995,11 +17024,11 @@
         <v>55</v>
       </c>
       <c r="G326" s="6" t="s">
-        <v>366</v>
+        <v>368</v>
       </c>
       <c r="H326" s="6"/>
       <c r="I326" s="6" t="s">
-        <v>365</v>
+        <v>367</v>
       </c>
       <c r="J326" s="6"/>
     </row>
@@ -17008,7 +17037,7 @@
         <v>2302</v>
       </c>
       <c r="B327" s="15" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="C327" s="5">
         <v>23</v>
@@ -17023,7 +17052,7 @@
       <c r="G327" s="15"/>
       <c r="H327" s="6"/>
       <c r="I327" s="6" t="s">
-        <v>367</v>
+        <v>369</v>
       </c>
       <c r="J327" s="6"/>
     </row>
@@ -17032,7 +17061,7 @@
         <v>23021</v>
       </c>
       <c r="B328" s="15" t="s">
-        <v>368</v>
+        <v>370</v>
       </c>
       <c r="C328" s="5">
         <v>2302</v>
@@ -17045,11 +17074,11 @@
         <v>55</v>
       </c>
       <c r="G328" s="15" t="s">
-        <v>369</v>
+        <v>371</v>
       </c>
       <c r="H328" s="6"/>
       <c r="I328" s="6" t="s">
-        <v>370</v>
+        <v>372</v>
       </c>
       <c r="J328" s="6"/>
     </row>
@@ -17058,7 +17087,7 @@
         <v>23022</v>
       </c>
       <c r="B329" s="15" t="s">
-        <v>371</v>
+        <v>373</v>
       </c>
       <c r="C329" s="5">
         <v>2302</v>
@@ -17071,11 +17100,11 @@
         <v>55</v>
       </c>
       <c r="G329" s="15" t="s">
-        <v>372</v>
+        <v>374</v>
       </c>
       <c r="H329" s="6"/>
       <c r="I329" s="6" t="s">
-        <v>373</v>
+        <v>375</v>
       </c>
       <c r="J329" s="6"/>
     </row>
@@ -17108,7 +17137,7 @@
         <v>23031</v>
       </c>
       <c r="B331" s="6" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="C331" s="5">
         <v>2303</v>
@@ -17121,11 +17150,11 @@
         <v>55</v>
       </c>
       <c r="G331" s="6" t="s">
-        <v>375</v>
+        <v>377</v>
       </c>
       <c r="H331" s="6"/>
       <c r="I331" s="6" t="s">
-        <v>374</v>
+        <v>376</v>
       </c>
       <c r="J331" s="6"/>
     </row>
@@ -17134,7 +17163,7 @@
         <v>23032</v>
       </c>
       <c r="B332" s="6" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="C332" s="5">
         <v>2303</v>
@@ -17147,11 +17176,11 @@
         <v>55</v>
       </c>
       <c r="G332" s="6" t="s">
-        <v>377</v>
+        <v>379</v>
       </c>
       <c r="H332" s="6"/>
       <c r="I332" s="6" t="s">
-        <v>376</v>
+        <v>378</v>
       </c>
       <c r="J332" s="6"/>
     </row>
@@ -17160,7 +17189,7 @@
         <v>23033</v>
       </c>
       <c r="B333" s="6" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="C333" s="5">
         <v>2303</v>
@@ -17173,11 +17202,11 @@
         <v>55</v>
       </c>
       <c r="G333" s="6" t="s">
-        <v>379</v>
+        <v>381</v>
       </c>
       <c r="H333" s="6"/>
       <c r="I333" s="6" t="s">
-        <v>378</v>
+        <v>380</v>
       </c>
       <c r="J333" s="6"/>
     </row>
@@ -17186,7 +17215,7 @@
         <v>23034</v>
       </c>
       <c r="B334" s="6" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="C334" s="5">
         <v>2303</v>
@@ -17199,11 +17228,11 @@
         <v>55</v>
       </c>
       <c r="G334" s="6" t="s">
-        <v>381</v>
+        <v>383</v>
       </c>
       <c r="H334" s="6"/>
       <c r="I334" s="6" t="s">
-        <v>380</v>
+        <v>382</v>
       </c>
       <c r="J334" s="6"/>
     </row>
@@ -17212,7 +17241,7 @@
         <v>2304</v>
       </c>
       <c r="B335" s="6" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="C335" s="5">
         <v>23</v>
@@ -17227,7 +17256,7 @@
       <c r="G335" s="6"/>
       <c r="H335" s="6"/>
       <c r="I335" s="6" t="s">
-        <v>382</v>
+        <v>384</v>
       </c>
       <c r="J335" s="6"/>
     </row>
@@ -17236,7 +17265,7 @@
         <v>23041</v>
       </c>
       <c r="B336" s="6" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="C336" s="5">
         <v>2304</v>
@@ -17249,11 +17278,11 @@
         <v>55</v>
       </c>
       <c r="G336" s="6" t="s">
-        <v>384</v>
+        <v>386</v>
       </c>
       <c r="H336" s="6"/>
       <c r="I336" s="6" t="s">
-        <v>383</v>
+        <v>385</v>
       </c>
       <c r="J336" s="6"/>
     </row>
@@ -17262,7 +17291,7 @@
         <v>23042</v>
       </c>
       <c r="B337" s="6" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="C337" s="5">
         <v>2304</v>
@@ -17275,11 +17304,11 @@
         <v>55</v>
       </c>
       <c r="G337" s="6" t="s">
-        <v>386</v>
+        <v>388</v>
       </c>
       <c r="H337" s="6"/>
       <c r="I337" s="6" t="s">
-        <v>385</v>
+        <v>387</v>
       </c>
       <c r="J337" s="6"/>
     </row>
@@ -17288,7 +17317,7 @@
         <v>23043</v>
       </c>
       <c r="B338" s="6" t="s">
-        <v>387</v>
+        <v>389</v>
       </c>
       <c r="C338" s="5">
         <v>2304</v>
@@ -17301,11 +17330,11 @@
         <v>55</v>
       </c>
       <c r="G338" s="6" t="s">
-        <v>388</v>
+        <v>390</v>
       </c>
       <c r="H338" s="6"/>
       <c r="I338" s="6" t="s">
-        <v>389</v>
+        <v>391</v>
       </c>
       <c r="J338" s="6"/>
     </row>
@@ -17314,7 +17343,7 @@
         <v>23044</v>
       </c>
       <c r="B339" s="6" t="s">
-        <v>390</v>
+        <v>392</v>
       </c>
       <c r="C339" s="5">
         <v>2304</v>
@@ -17327,11 +17356,11 @@
         <v>55</v>
       </c>
       <c r="G339" s="6" t="s">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="H339" s="6"/>
       <c r="I339" s="6" t="s">
-        <v>392</v>
+        <v>394</v>
       </c>
       <c r="J339" s="6"/>
     </row>
@@ -17340,7 +17369,7 @@
         <v>2305</v>
       </c>
       <c r="B340" s="6" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="C340" s="5">
         <v>23</v>
@@ -17355,7 +17384,7 @@
       <c r="G340" s="5"/>
       <c r="H340" s="5"/>
       <c r="I340" s="6" t="s">
-        <v>393</v>
+        <v>395</v>
       </c>
       <c r="J340" s="6"/>
     </row>
@@ -17364,7 +17393,7 @@
         <v>23051</v>
       </c>
       <c r="B341" s="6" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="C341" s="5">
         <v>2305</v>
@@ -17377,11 +17406,11 @@
         <v>55</v>
       </c>
       <c r="G341" s="6" t="s">
-        <v>395</v>
+        <v>397</v>
       </c>
       <c r="H341" s="5"/>
       <c r="I341" s="6" t="s">
-        <v>394</v>
+        <v>396</v>
       </c>
       <c r="J341" s="6"/>
     </row>
@@ -17390,7 +17419,7 @@
         <v>23052</v>
       </c>
       <c r="B342" s="6" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="C342" s="5">
         <v>2305</v>
@@ -17403,11 +17432,11 @@
         <v>55</v>
       </c>
       <c r="G342" s="6" t="s">
-        <v>397</v>
+        <v>399</v>
       </c>
       <c r="H342" s="6"/>
       <c r="I342" s="6" t="s">
-        <v>396</v>
+        <v>398</v>
       </c>
       <c r="J342" s="6"/>
     </row>
@@ -17416,7 +17445,7 @@
         <v>24</v>
       </c>
       <c r="B343" s="6" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="C343" s="5">
         <v>2</v>
@@ -17431,7 +17460,7 @@
       <c r="G343" s="6"/>
       <c r="H343" s="6"/>
       <c r="I343" s="6" t="s">
-        <v>398</v>
+        <v>400</v>
       </c>
       <c r="J343" s="6"/>
     </row>
@@ -17440,7 +17469,7 @@
         <v>25</v>
       </c>
       <c r="B344" s="6" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="C344" s="5">
         <v>2</v>
@@ -17455,7 +17484,7 @@
       <c r="G344" s="6"/>
       <c r="H344" s="6"/>
       <c r="I344" s="6" t="s">
-        <v>399</v>
+        <v>401</v>
       </c>
       <c r="J344" s="6"/>
     </row>
@@ -17464,7 +17493,7 @@
         <v>2501</v>
       </c>
       <c r="B345" s="6" t="s">
-        <v>400</v>
+        <v>402</v>
       </c>
       <c r="C345" s="5">
         <v>25</v>
@@ -17477,11 +17506,11 @@
         <v>55</v>
       </c>
       <c r="G345" s="6" t="s">
-        <v>401</v>
+        <v>403</v>
       </c>
       <c r="H345" s="6"/>
       <c r="I345" s="6" t="s">
-        <v>402</v>
+        <v>404</v>
       </c>
       <c r="J345" s="6"/>
     </row>
@@ -17490,7 +17519,7 @@
         <v>2502</v>
       </c>
       <c r="B346" s="6" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="C346" s="5">
         <v>25</v>
@@ -17503,11 +17532,11 @@
         <v>55</v>
       </c>
       <c r="G346" s="6" t="s">
-        <v>404</v>
+        <v>406</v>
       </c>
       <c r="H346" s="5"/>
       <c r="I346" s="6" t="s">
-        <v>403</v>
+        <v>405</v>
       </c>
       <c r="J346" s="6"/>
     </row>
@@ -17516,7 +17545,7 @@
         <v>2503</v>
       </c>
       <c r="B347" s="6" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="C347" s="5">
         <v>25</v>
@@ -17530,7 +17559,7 @@
       </c>
       <c r="G347" s="6"/>
       <c r="I347" s="2" t="s">
-        <v>405</v>
+        <v>407</v>
       </c>
       <c r="J347" s="2" t="b">
         <v>1</v>

</xml_diff>

<commit_message>
#80 AOD Alignment 产率架构
</commit_message>
<xml_diff>
--- a/Sources/Cuga-Calibration-Solution/Assets/Data/InitData.xlsx
+++ b/Sources/Cuga-Calibration-Solution/Assets/Data/InitData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\RiderProjects\semix\kaizhi.xuan\netcore_semix_cuga_calibration\Sources\Cuga-Calibration-Solution\Assets\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41666820-1823-471A-9A6C-A960EEE2BE4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66C5F378-1409-453B-BCAA-9308093ACBD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" firstSheet="1" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" firstSheet="1" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SysUser" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1497" uniqueCount="383">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1497" uniqueCount="382">
   <si>
     <t>Id</t>
   </si>
@@ -868,9 +868,6 @@
     <t>AOD</t>
   </si>
   <si>
-    <t>Aod Alignment</t>
-  </si>
-  <si>
     <t>XY Astigmatism</t>
   </si>
   <si>
@@ -878,9 +875,6 @@
   </si>
   <si>
     <t>Illumination Profile</t>
-  </si>
-  <si>
-    <t>CugaCalibration.ViewModels.Laser.LaserIlluminationProfileCalibrationViewModel</t>
   </si>
   <si>
     <t>CIB</t>
@@ -1225,10 +1219,6 @@
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
   <si>
-    <t>CugaCalibration.ViewModels.Laser.LaserPrescanChirpAodAlignmentCalibrationViewModel</t>
-    <phoneticPr fontId="7" type="noConversion"/>
-  </si>
-  <si>
     <t>CugaCalibration.ViewModels.AOD.AODDelayViewModel</t>
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
@@ -1254,6 +1244,14 @@
   </si>
   <si>
     <t>Objective Y Angle</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>CugaCalibration.ViewModels.Laser.LaserIlluminationProfileCalibrationViewModel</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>CugaCalibration.ViewModels.AOD.AODAlignmentViewModel</t>
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
 </sst>
@@ -1419,7 +1417,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1475,6 +1473,9 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -13743,7 +13744,7 @@
         <v>55</v>
       </c>
       <c r="G229" s="18" t="s">
-        <v>374</v>
+        <v>372</v>
       </c>
       <c r="H229" s="5"/>
       <c r="I229" s="5" t="s">
@@ -13769,7 +13770,7 @@
         <v>55</v>
       </c>
       <c r="G230" s="18" t="s">
-        <v>373</v>
+        <v>371</v>
       </c>
       <c r="H230" s="5"/>
       <c r="I230" s="5" t="s">
@@ -13806,7 +13807,7 @@
         <v>15</v>
       </c>
       <c r="B232" s="18" t="s">
-        <v>370</v>
+        <v>368</v>
       </c>
       <c r="C232" s="4">
         <v>1</v>
@@ -13830,7 +13831,7 @@
         <v>1501</v>
       </c>
       <c r="B233" s="18" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="C233" s="4">
         <v>15</v>
@@ -13843,11 +13844,11 @@
         <v>55</v>
       </c>
       <c r="G233" s="18" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="H233" s="5"/>
       <c r="I233" s="18" t="s">
-        <v>371</v>
+        <v>369</v>
       </c>
       <c r="J233" s="5"/>
     </row>
@@ -13856,7 +13857,7 @@
         <v>1502</v>
       </c>
       <c r="B234" s="18" t="s">
-        <v>372</v>
+        <v>370</v>
       </c>
       <c r="C234" s="4">
         <v>15</v>
@@ -13869,11 +13870,11 @@
         <v>55</v>
       </c>
       <c r="G234" s="18" t="s">
-        <v>375</v>
+        <v>381</v>
       </c>
       <c r="H234" s="5"/>
-      <c r="I234" s="5" t="s">
-        <v>275</v>
+      <c r="I234" s="18" t="s">
+        <v>370</v>
       </c>
       <c r="J234" s="5"/>
     </row>
@@ -13882,7 +13883,7 @@
         <v>1503</v>
       </c>
       <c r="B235" s="5" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="C235" s="4">
         <v>15</v>
@@ -13895,11 +13896,11 @@
         <v>55</v>
       </c>
       <c r="G235" s="5" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="H235" s="5"/>
       <c r="I235" s="5" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="J235" s="5"/>
     </row>
@@ -13908,7 +13909,7 @@
         <v>1504</v>
       </c>
       <c r="B236" s="7" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C236" s="6">
         <v>15</v>
@@ -13920,12 +13921,12 @@
       <c r="F236" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="G236" s="7" t="s">
-        <v>279</v>
+      <c r="G236" s="19" t="s">
+        <v>380</v>
       </c>
       <c r="H236" s="7"/>
       <c r="I236" s="7" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="J236" s="5"/>
     </row>
@@ -13934,7 +13935,7 @@
         <v>16</v>
       </c>
       <c r="B237" s="9" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C237" s="8">
         <v>1</v>
@@ -13949,7 +13950,7 @@
       <c r="G237" s="9"/>
       <c r="H237" s="9"/>
       <c r="I237" s="9" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="J237" s="5"/>
     </row>
@@ -13958,7 +13959,7 @@
         <v>1601</v>
       </c>
       <c r="B238" s="5" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C238" s="4">
         <v>16</v>
@@ -13971,11 +13972,11 @@
         <v>55</v>
       </c>
       <c r="G238" s="5" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="H238" s="5"/>
       <c r="I238" s="5" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="J238" s="5"/>
     </row>
@@ -13997,7 +13998,7 @@
         <v>55</v>
       </c>
       <c r="G239" s="5" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="H239" s="5"/>
       <c r="I239" s="5" t="s">
@@ -14023,7 +14024,7 @@
         <v>58</v>
       </c>
       <c r="G240" s="5" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="H240" s="5" t="s">
         <v>60</v>
@@ -14051,7 +14052,7 @@
         <v>58</v>
       </c>
       <c r="G241" s="5" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="H241" s="5" t="s">
         <v>61</v>
@@ -14079,13 +14080,13 @@
         <v>68</v>
       </c>
       <c r="G242" s="5" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="H242" s="5" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="I242" s="5" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="J242" s="5"/>
     </row>
@@ -14107,7 +14108,7 @@
         <v>58</v>
       </c>
       <c r="G243" s="5" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="H243" s="5" t="s">
         <v>64</v>
@@ -14135,7 +14136,7 @@
         <v>58</v>
       </c>
       <c r="G244" s="5" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="H244" s="5" t="s">
         <v>65</v>
@@ -14163,7 +14164,7 @@
         <v>68</v>
       </c>
       <c r="G245" s="5" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="H245" s="5" t="s">
         <v>69</v>
@@ -14191,7 +14192,7 @@
         <v>58</v>
       </c>
       <c r="G246" s="5" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="H246" s="5" t="s">
         <v>64</v>
@@ -14219,7 +14220,7 @@
         <v>58</v>
       </c>
       <c r="G247" s="5" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="H247" s="5" t="s">
         <v>65</v>
@@ -14234,7 +14235,7 @@
         <v>1603</v>
       </c>
       <c r="B248" s="5" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C248" s="4">
         <v>16</v>
@@ -14247,11 +14248,11 @@
         <v>55</v>
       </c>
       <c r="G248" s="5" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="H248" s="5"/>
       <c r="I248" s="5" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="J248" s="5"/>
     </row>
@@ -14260,7 +14261,7 @@
         <v>160301</v>
       </c>
       <c r="B249" s="5" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C249" s="4">
         <v>1603</v>
@@ -14273,7 +14274,7 @@
         <v>58</v>
       </c>
       <c r="G249" s="5" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="H249" s="5" t="s">
         <v>156</v>
@@ -14288,7 +14289,7 @@
         <v>160302</v>
       </c>
       <c r="B250" s="5" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C250" s="4">
         <v>1603</v>
@@ -14301,7 +14302,7 @@
         <v>58</v>
       </c>
       <c r="G250" s="5" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="H250" s="5" t="s">
         <v>60</v>
@@ -14316,7 +14317,7 @@
         <v>160303</v>
       </c>
       <c r="B251" s="5" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C251" s="4">
         <v>1603</v>
@@ -14329,7 +14330,7 @@
         <v>58</v>
       </c>
       <c r="G251" s="5" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="H251" s="5" t="s">
         <v>61</v>
@@ -14344,7 +14345,7 @@
         <v>160304</v>
       </c>
       <c r="B252" s="5" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C252" s="4">
         <v>1603</v>
@@ -14357,13 +14358,13 @@
         <v>58</v>
       </c>
       <c r="G252" s="5" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="H252" s="5" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="I252" s="5" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="J252" s="5"/>
     </row>
@@ -14372,7 +14373,7 @@
         <v>160305</v>
       </c>
       <c r="B253" s="5" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C253" s="4">
         <v>1603</v>
@@ -14385,13 +14386,13 @@
         <v>58</v>
       </c>
       <c r="G253" s="5" t="s">
+        <v>291</v>
+      </c>
+      <c r="H253" s="5" t="s">
         <v>293</v>
       </c>
-      <c r="H253" s="5" t="s">
-        <v>295</v>
-      </c>
       <c r="I253" s="5" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="J253" s="5"/>
     </row>
@@ -14400,7 +14401,7 @@
         <v>160306</v>
       </c>
       <c r="B254" s="5" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C254" s="4">
         <v>1603</v>
@@ -14413,7 +14414,7 @@
         <v>58</v>
       </c>
       <c r="G254" s="5" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="H254" s="5" t="s">
         <v>64</v>
@@ -14428,7 +14429,7 @@
         <v>160307</v>
       </c>
       <c r="B255" s="5" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C255" s="4">
         <v>1603</v>
@@ -14441,7 +14442,7 @@
         <v>58</v>
       </c>
       <c r="G255" s="5" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="H255" s="5" t="s">
         <v>65</v>
@@ -14456,7 +14457,7 @@
         <v>160308</v>
       </c>
       <c r="B256" s="5" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C256" s="4">
         <v>1603</v>
@@ -14469,7 +14470,7 @@
         <v>68</v>
       </c>
       <c r="G256" s="5" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="H256" s="5" t="s">
         <v>161</v>
@@ -14484,7 +14485,7 @@
         <v>160309</v>
       </c>
       <c r="B257" s="5" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C257" s="4">
         <v>1603</v>
@@ -14497,7 +14498,7 @@
         <v>58</v>
       </c>
       <c r="G257" s="5" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="H257" s="5" t="s">
         <v>64</v>
@@ -14512,7 +14513,7 @@
         <v>160310</v>
       </c>
       <c r="B258" s="5" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C258" s="4">
         <v>1603</v>
@@ -14525,7 +14526,7 @@
         <v>58</v>
       </c>
       <c r="G258" s="5" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="H258" s="5" t="s">
         <v>65</v>
@@ -14540,7 +14541,7 @@
         <v>1604</v>
       </c>
       <c r="B259" s="5" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C259" s="4">
         <v>16</v>
@@ -14553,11 +14554,11 @@
         <v>55</v>
       </c>
       <c r="G259" s="5" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="H259" s="5"/>
       <c r="I259" s="5" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="J259" s="5"/>
     </row>
@@ -14566,7 +14567,7 @@
         <v>1608</v>
       </c>
       <c r="B260" s="5" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C260" s="4">
         <v>16</v>
@@ -14579,11 +14580,11 @@
         <v>55</v>
       </c>
       <c r="G260" s="5" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="H260" s="5"/>
       <c r="I260" s="5" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="J260" s="5"/>
     </row>
@@ -14592,7 +14593,7 @@
         <v>1604</v>
       </c>
       <c r="B261" s="7" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C261" s="6">
         <v>16</v>
@@ -14605,11 +14606,11 @@
         <v>55</v>
       </c>
       <c r="G261" s="7" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="H261" s="7"/>
       <c r="I261" s="7" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="J261" s="5"/>
     </row>
@@ -14618,7 +14619,7 @@
         <v>1605</v>
       </c>
       <c r="B262" s="1" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C262" s="4">
         <v>16</v>
@@ -14631,10 +14632,10 @@
         <v>55</v>
       </c>
       <c r="G262" s="5" t="s">
-        <v>305</v>
+        <v>303</v>
       </c>
       <c r="I262" s="1" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="J262" s="5"/>
     </row>
@@ -14643,7 +14644,7 @@
         <v>1606</v>
       </c>
       <c r="B263" s="1" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="C263" s="4">
         <v>16</v>
@@ -14656,11 +14657,11 @@
         <v>55</v>
       </c>
       <c r="G263" s="1" t="s">
-        <v>307</v>
+        <v>305</v>
       </c>
       <c r="H263" s="1"/>
       <c r="I263" s="1" t="s">
-        <v>306</v>
+        <v>304</v>
       </c>
       <c r="J263" s="5"/>
     </row>
@@ -14669,7 +14670,7 @@
         <v>1607</v>
       </c>
       <c r="B264" s="1" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="C264" s="4">
         <v>16</v>
@@ -14682,11 +14683,11 @@
         <v>55</v>
       </c>
       <c r="G264" s="1" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="H264" s="1"/>
       <c r="I264" s="1" t="s">
-        <v>308</v>
+        <v>306</v>
       </c>
       <c r="J264" s="5"/>
     </row>
@@ -14695,7 +14696,7 @@
         <v>2</v>
       </c>
       <c r="B265" s="5" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="C265" s="4">
         <v>-1</v>
@@ -14710,7 +14711,7 @@
       <c r="G265" s="5"/>
       <c r="H265" s="5"/>
       <c r="I265" s="5" t="s">
-        <v>310</v>
+        <v>308</v>
       </c>
       <c r="J265" s="5"/>
     </row>
@@ -14719,7 +14720,7 @@
         <v>21</v>
       </c>
       <c r="B266" s="5" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="C266" s="4">
         <v>2</v>
@@ -14734,7 +14735,7 @@
       <c r="G266" s="5"/>
       <c r="H266" s="5"/>
       <c r="I266" s="5" t="s">
-        <v>311</v>
+        <v>309</v>
       </c>
       <c r="J266" s="5"/>
     </row>
@@ -14743,7 +14744,7 @@
         <v>2110</v>
       </c>
       <c r="B267" s="5" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="C267" s="4">
         <v>21</v>
@@ -14756,11 +14757,11 @@
         <v>55</v>
       </c>
       <c r="G267" s="5" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="H267" s="5"/>
       <c r="I267" s="5" t="s">
-        <v>312</v>
+        <v>310</v>
       </c>
       <c r="J267" s="5"/>
     </row>
@@ -14769,7 +14770,7 @@
         <v>2111</v>
       </c>
       <c r="B268" s="5" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="C268" s="4">
         <v>21</v>
@@ -14782,11 +14783,11 @@
         <v>55</v>
       </c>
       <c r="G268" s="5" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="H268" s="5"/>
       <c r="I268" s="5" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="J268" s="5"/>
     </row>
@@ -14795,7 +14796,7 @@
         <v>22</v>
       </c>
       <c r="B269" s="5" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="C269" s="4">
         <v>2</v>
@@ -14810,7 +14811,7 @@
       <c r="G269" s="5"/>
       <c r="H269" s="5"/>
       <c r="I269" s="5" t="s">
-        <v>316</v>
+        <v>314</v>
       </c>
       <c r="J269" s="5"/>
     </row>
@@ -14819,7 +14820,7 @@
         <v>2201</v>
       </c>
       <c r="B270" s="5" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="C270" s="4">
         <v>22</v>
@@ -14832,11 +14833,11 @@
         <v>55</v>
       </c>
       <c r="G270" s="5" t="s">
-        <v>318</v>
+        <v>316</v>
       </c>
       <c r="H270" s="5"/>
       <c r="I270" s="5" t="s">
-        <v>317</v>
+        <v>315</v>
       </c>
       <c r="J270" s="5"/>
     </row>
@@ -14845,7 +14846,7 @@
         <v>2202</v>
       </c>
       <c r="B271" s="5" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="C271" s="4">
         <v>22</v>
@@ -14858,11 +14859,11 @@
         <v>55</v>
       </c>
       <c r="G271" s="5" t="s">
-        <v>320</v>
+        <v>318</v>
       </c>
       <c r="H271" s="5"/>
       <c r="I271" s="5" t="s">
-        <v>319</v>
+        <v>317</v>
       </c>
       <c r="J271" s="5"/>
     </row>
@@ -14871,7 +14872,7 @@
         <v>2203</v>
       </c>
       <c r="B272" s="5" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="C272" s="4">
         <v>22</v>
@@ -14884,11 +14885,11 @@
         <v>55</v>
       </c>
       <c r="G272" s="5" t="s">
-        <v>322</v>
+        <v>320</v>
       </c>
       <c r="H272" s="5"/>
       <c r="I272" s="5" t="s">
-        <v>321</v>
+        <v>319</v>
       </c>
       <c r="J272" s="5"/>
     </row>
@@ -14897,7 +14898,7 @@
         <v>23</v>
       </c>
       <c r="B273" s="5" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="C273" s="4">
         <v>2</v>
@@ -14912,7 +14913,7 @@
       <c r="G273" s="5"/>
       <c r="H273" s="5"/>
       <c r="I273" s="5" t="s">
-        <v>323</v>
+        <v>321</v>
       </c>
       <c r="J273" s="5"/>
     </row>
@@ -14921,7 +14922,7 @@
         <v>2301</v>
       </c>
       <c r="B274" s="5" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="C274" s="4">
         <v>23</v>
@@ -14934,11 +14935,11 @@
         <v>55</v>
       </c>
       <c r="G274" s="5" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="H274" s="5"/>
       <c r="I274" s="5" t="s">
-        <v>324</v>
+        <v>322</v>
       </c>
       <c r="J274" s="5"/>
     </row>
@@ -14947,7 +14948,7 @@
         <v>2302</v>
       </c>
       <c r="B275" s="5" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="C275" s="4">
         <v>23</v>
@@ -14962,7 +14963,7 @@
       <c r="G275" s="5"/>
       <c r="H275" s="5"/>
       <c r="I275" s="5" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="J275" s="5"/>
     </row>
@@ -14971,7 +14972,7 @@
         <v>23021</v>
       </c>
       <c r="B276" s="5" t="s">
-        <v>327</v>
+        <v>325</v>
       </c>
       <c r="C276" s="4">
         <v>2302</v>
@@ -14984,11 +14985,11 @@
         <v>55</v>
       </c>
       <c r="G276" s="5" t="s">
-        <v>328</v>
+        <v>326</v>
       </c>
       <c r="H276" s="5"/>
       <c r="I276" s="5" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="J276" s="5"/>
     </row>
@@ -14997,7 +14998,7 @@
         <v>23022</v>
       </c>
       <c r="B277" s="5" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C277" s="4">
         <v>2302</v>
@@ -15010,11 +15011,11 @@
         <v>55</v>
       </c>
       <c r="G277" s="5" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="H277" s="5"/>
       <c r="I277" s="5" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="J277" s="5"/>
     </row>
@@ -15047,7 +15048,7 @@
         <v>23031</v>
       </c>
       <c r="B279" s="10" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="C279" s="4">
         <v>2303</v>
@@ -15060,11 +15061,11 @@
         <v>55</v>
       </c>
       <c r="G279" s="10" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="H279" s="5"/>
       <c r="I279" s="10" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="J279" s="5"/>
     </row>
@@ -15073,7 +15074,7 @@
         <v>23032</v>
       </c>
       <c r="B280" s="10" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="C280" s="4">
         <v>2303</v>
@@ -15086,11 +15087,11 @@
         <v>55</v>
       </c>
       <c r="G280" s="10" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="H280" s="5"/>
       <c r="I280" s="10" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="J280" s="5"/>
     </row>
@@ -15099,7 +15100,7 @@
         <v>23033</v>
       </c>
       <c r="B281" s="10" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="C281" s="4">
         <v>2303</v>
@@ -15112,11 +15113,11 @@
         <v>55</v>
       </c>
       <c r="G281" s="10" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="H281" s="5"/>
       <c r="I281" s="10" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="J281" s="5"/>
     </row>
@@ -15125,7 +15126,7 @@
         <v>23034</v>
       </c>
       <c r="B282" s="10" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="C282" s="4">
         <v>2303</v>
@@ -15138,11 +15139,11 @@
         <v>55</v>
       </c>
       <c r="G282" s="10" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="H282" s="5"/>
       <c r="I282" s="10" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="J282" s="5"/>
     </row>
@@ -15151,7 +15152,7 @@
         <v>23035</v>
       </c>
       <c r="B283" s="10" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="C283" s="4">
         <v>2303</v>
@@ -15164,11 +15165,11 @@
         <v>55</v>
       </c>
       <c r="G283" s="10" t="s">
-        <v>342</v>
+        <v>340</v>
       </c>
       <c r="H283" s="5"/>
       <c r="I283" s="10" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="J283" s="5"/>
     </row>
@@ -15177,7 +15178,7 @@
         <v>23036</v>
       </c>
       <c r="B284" s="10" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="C284" s="4">
         <v>2303</v>
@@ -15190,11 +15191,11 @@
         <v>55</v>
       </c>
       <c r="G284" s="10" t="s">
-        <v>344</v>
+        <v>342</v>
       </c>
       <c r="H284" s="5"/>
       <c r="I284" s="10" t="s">
-        <v>343</v>
+        <v>341</v>
       </c>
       <c r="J284" s="5"/>
     </row>
@@ -15203,7 +15204,7 @@
         <v>2304</v>
       </c>
       <c r="B285" s="10" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="C285" s="4">
         <v>23</v>
@@ -15218,7 +15219,7 @@
       <c r="G285" s="5"/>
       <c r="H285" s="5"/>
       <c r="I285" s="10" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="J285" s="5"/>
     </row>
@@ -15227,7 +15228,7 @@
         <v>23041</v>
       </c>
       <c r="B286" s="10" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="C286" s="4">
         <v>2304</v>
@@ -15240,11 +15241,11 @@
         <v>55</v>
       </c>
       <c r="G286" s="10" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="H286" s="5"/>
       <c r="I286" s="10" t="s">
-        <v>346</v>
+        <v>344</v>
       </c>
       <c r="J286" s="5"/>
     </row>
@@ -15253,7 +15254,7 @@
         <v>2305</v>
       </c>
       <c r="B287" s="18" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="C287" s="4">
         <v>23</v>
@@ -15268,7 +15269,7 @@
       <c r="G287" s="5"/>
       <c r="H287" s="5"/>
       <c r="I287" s="18" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="J287" s="5"/>
     </row>
@@ -15277,7 +15278,7 @@
         <v>23051</v>
       </c>
       <c r="B288" s="18" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="C288" s="4">
         <v>2305</v>
@@ -15290,11 +15291,11 @@
         <v>55</v>
       </c>
       <c r="G288" s="18" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="H288" s="5"/>
       <c r="I288" s="18" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="J288" s="5"/>
     </row>
@@ -15303,7 +15304,7 @@
         <v>2306</v>
       </c>
       <c r="B289" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="C289" s="4">
         <v>23</v>
@@ -15318,7 +15319,7 @@
       <c r="G289" s="5"/>
       <c r="H289" s="5"/>
       <c r="I289" s="5" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="J289" s="5"/>
     </row>
@@ -15327,7 +15328,7 @@
         <v>23061</v>
       </c>
       <c r="B290" s="5" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="C290" s="4">
         <v>2306</v>
@@ -15340,11 +15341,11 @@
         <v>55</v>
       </c>
       <c r="G290" s="5" t="s">
-        <v>350</v>
+        <v>348</v>
       </c>
       <c r="H290" s="5"/>
       <c r="I290" s="5" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="J290" s="5"/>
     </row>
@@ -15353,7 +15354,7 @@
         <v>23062</v>
       </c>
       <c r="B291" s="5" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="C291" s="4">
         <v>2306</v>
@@ -15366,11 +15367,11 @@
         <v>55</v>
       </c>
       <c r="G291" s="5" t="s">
-        <v>352</v>
+        <v>350</v>
       </c>
       <c r="H291" s="5"/>
       <c r="I291" s="5" t="s">
-        <v>351</v>
+        <v>349</v>
       </c>
       <c r="J291" s="5"/>
     </row>
@@ -15379,7 +15380,7 @@
         <v>23063</v>
       </c>
       <c r="B292" s="5" t="s">
-        <v>353</v>
+        <v>351</v>
       </c>
       <c r="C292" s="4">
         <v>2306</v>
@@ -15392,11 +15393,11 @@
         <v>55</v>
       </c>
       <c r="G292" s="5" t="s">
-        <v>354</v>
+        <v>352</v>
       </c>
       <c r="H292" s="5"/>
       <c r="I292" s="5" t="s">
-        <v>355</v>
+        <v>353</v>
       </c>
       <c r="J292" s="5"/>
     </row>
@@ -15405,7 +15406,7 @@
         <v>2307</v>
       </c>
       <c r="B293" s="5" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="C293" s="4">
         <v>23</v>
@@ -15420,7 +15421,7 @@
       <c r="G293" s="4"/>
       <c r="H293" s="4"/>
       <c r="I293" s="5" t="s">
-        <v>356</v>
+        <v>354</v>
       </c>
       <c r="J293" s="5"/>
     </row>
@@ -15429,7 +15430,7 @@
         <v>23071</v>
       </c>
       <c r="B294" s="5" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="C294" s="4">
         <v>2307</v>
@@ -15442,11 +15443,11 @@
         <v>55</v>
       </c>
       <c r="G294" s="18" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="H294" s="4"/>
       <c r="I294" s="5" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="J294" s="5"/>
     </row>
@@ -15455,7 +15456,7 @@
         <v>23072</v>
       </c>
       <c r="B295" s="5" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="C295" s="4">
         <v>2307</v>
@@ -15468,11 +15469,11 @@
         <v>55</v>
       </c>
       <c r="G295" s="5" t="s">
-        <v>359</v>
+        <v>357</v>
       </c>
       <c r="H295" s="5"/>
       <c r="I295" s="5" t="s">
-        <v>358</v>
+        <v>356</v>
       </c>
       <c r="J295" s="5"/>
     </row>
@@ -15481,7 +15482,7 @@
         <v>23073</v>
       </c>
       <c r="B296" s="18" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="C296" s="4">
         <v>2307</v>
@@ -15494,11 +15495,11 @@
         <v>55</v>
       </c>
       <c r="G296" s="18" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="H296" s="5"/>
       <c r="I296" s="18" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="J296" s="5"/>
     </row>
@@ -15507,7 +15508,7 @@
         <v>24</v>
       </c>
       <c r="B297" s="5" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="C297" s="4">
         <v>2</v>
@@ -15522,7 +15523,7 @@
       <c r="G297" s="5"/>
       <c r="H297" s="5"/>
       <c r="I297" s="5" t="s">
-        <v>360</v>
+        <v>358</v>
       </c>
       <c r="J297" s="5"/>
     </row>
@@ -15531,7 +15532,7 @@
         <v>2401</v>
       </c>
       <c r="B298" s="5" t="s">
-        <v>361</v>
+        <v>359</v>
       </c>
       <c r="C298" s="4">
         <v>24</v>
@@ -15544,11 +15545,11 @@
         <v>55</v>
       </c>
       <c r="G298" s="5" t="s">
-        <v>362</v>
+        <v>360</v>
       </c>
       <c r="H298" s="5"/>
       <c r="I298" s="5" t="s">
-        <v>363</v>
+        <v>361</v>
       </c>
       <c r="J298" s="5"/>
     </row>
@@ -15557,7 +15558,7 @@
         <v>2402</v>
       </c>
       <c r="B299" s="5" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="C299" s="4">
         <v>24</v>
@@ -15570,11 +15571,11 @@
         <v>55</v>
       </c>
       <c r="G299" s="5" t="s">
-        <v>365</v>
+        <v>363</v>
       </c>
       <c r="H299" s="4"/>
       <c r="I299" s="5" t="s">
-        <v>364</v>
+        <v>362</v>
       </c>
       <c r="J299" s="5"/>
     </row>
@@ -15583,7 +15584,7 @@
         <v>2403</v>
       </c>
       <c r="B300" s="5" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="C300" s="4">
         <v>24</v>
@@ -15597,7 +15598,7 @@
       </c>
       <c r="G300" s="5"/>
       <c r="I300" s="1" t="s">
-        <v>366</v>
+        <v>364</v>
       </c>
       <c r="J300" s="1" t="b">
         <v>1</v>
@@ -15624,7 +15625,7 @@
         <v>25</v>
       </c>
       <c r="B301" s="5" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="C301" s="4">
         <v>2</v>
@@ -15639,7 +15640,7 @@
       <c r="G301" s="5"/>
       <c r="H301" s="5"/>
       <c r="I301" s="5" t="s">
-        <v>367</v>
+        <v>365</v>
       </c>
       <c r="J301" s="5"/>
     </row>
@@ -15648,7 +15649,7 @@
         <v>2501</v>
       </c>
       <c r="B302" s="5" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="C302" s="4">
         <v>25</v>
@@ -15661,11 +15662,11 @@
         <v>55</v>
       </c>
       <c r="G302" s="5" t="s">
-        <v>369</v>
+        <v>367</v>
       </c>
       <c r="H302" s="5"/>
       <c r="I302" s="5" t="s">
-        <v>368</v>
+        <v>366</v>
       </c>
       <c r="J302" s="5"/>
     </row>

</xml_diff>

<commit_message>
#84 remove chuck auto focus
</commit_message>
<xml_diff>
--- a/Sources/Cuga-Calibration-Solution/Assets/Data/InitData.xlsx
+++ b/Sources/Cuga-Calibration-Solution/Assets/Data/InitData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\RiderProjects\semix\kaizhi.xuan\netcore_semix_cuga_calibration\Sources\Cuga-Calibration-Solution\Assets\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF7FCA20-B239-4E45-97DF-59511898C34C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEBCFBDF-83BB-4B51-AFE0-FAB6142E625E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" firstSheet="1" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" firstSheet="1" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SysUser" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1395" uniqueCount="365">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1391" uniqueCount="363">
   <si>
     <t>Id</t>
   </si>
@@ -767,12 +767,6 @@
   </si>
   <si>
     <t>CugaCalibration.ViewModels.Chuck.ChuckRotateScaleCalibrationViewModel</t>
-  </si>
-  <si>
-    <t>Chuck Auto Focus</t>
-  </si>
-  <si>
-    <t>CugaCalibration.ViewModels.Chuck.ChuckAutoFocusCalibrationViewModel</t>
   </si>
   <si>
     <t>Stage Map</t>
@@ -7344,7 +7338,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:Z281"/>
+  <dimension ref="A1:Z280"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.625" style="2" customWidth="1"/>
@@ -12977,139 +12971,141 @@
       </c>
       <c r="J202" s="5"/>
     </row>
-    <row r="203" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A203" s="4">
-        <v>1308</v>
-      </c>
-      <c r="B203" s="5" t="s">
+        <v>1309</v>
+      </c>
+      <c r="B203" s="1" t="s">
         <v>242</v>
       </c>
       <c r="C203" s="4">
         <v>13</v>
       </c>
       <c r="D203" s="4">
-        <v>1308</v>
+        <v>1309</v>
       </c>
       <c r="E203" s="4"/>
       <c r="F203" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="G203" s="5" t="s">
+      <c r="G203" s="1" t="s">
         <v>243</v>
       </c>
-      <c r="H203" s="5"/>
-      <c r="I203" s="5" t="s">
+      <c r="H203" s="1"/>
+      <c r="I203" s="1" t="s">
         <v>242</v>
       </c>
       <c r="J203" s="5"/>
     </row>
-    <row r="204" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A204" s="4">
-        <v>1309</v>
-      </c>
-      <c r="B204" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="B204" s="5" t="s">
         <v>244</v>
       </c>
       <c r="C204" s="4">
-        <v>13</v>
+        <v>1</v>
       </c>
       <c r="D204" s="4">
-        <v>1309</v>
+        <v>14</v>
       </c>
       <c r="E204" s="4"/>
       <c r="F204" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G204" s="1" t="s">
-        <v>245</v>
-      </c>
-      <c r="H204" s="1"/>
-      <c r="I204" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="G204" s="5"/>
+      <c r="H204" s="5"/>
+      <c r="I204" s="5" t="s">
         <v>244</v>
       </c>
       <c r="J204" s="5"/>
     </row>
     <row r="205" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A205" s="4">
+        <v>1401</v>
+      </c>
+      <c r="B205" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="C205" s="4">
         <v>14</v>
       </c>
-      <c r="B205" s="5" t="s">
-        <v>246</v>
-      </c>
-      <c r="C205" s="4">
-        <v>1</v>
-      </c>
       <c r="D205" s="4">
-        <v>14</v>
+        <v>1401</v>
       </c>
       <c r="E205" s="4"/>
       <c r="F205" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G205" s="5"/>
+        <v>55</v>
+      </c>
+      <c r="G205" s="5" t="s">
+        <v>246</v>
+      </c>
       <c r="H205" s="5"/>
       <c r="I205" s="5" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="J205" s="5"/>
     </row>
     <row r="206" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A206" s="4">
-        <v>1401</v>
+        <v>140101</v>
       </c>
       <c r="B206" s="5" t="s">
         <v>247</v>
       </c>
       <c r="C206" s="4">
-        <v>14</v>
+        <v>1401</v>
       </c>
       <c r="D206" s="4">
-        <v>1401</v>
+        <v>140101</v>
       </c>
       <c r="E206" s="4"/>
       <c r="F206" s="4" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="G206" s="5" t="s">
         <v>248</v>
       </c>
-      <c r="H206" s="5"/>
+      <c r="H206" s="5" t="s">
+        <v>60</v>
+      </c>
       <c r="I206" s="5" t="s">
-        <v>247</v>
+        <v>60</v>
       </c>
       <c r="J206" s="5"/>
     </row>
     <row r="207" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A207" s="4">
-        <v>140101</v>
+        <v>140102</v>
       </c>
       <c r="B207" s="5" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="C207" s="4">
         <v>1401</v>
       </c>
       <c r="D207" s="4">
-        <v>140101</v>
+        <v>140102</v>
       </c>
       <c r="E207" s="4"/>
       <c r="F207" s="4" t="s">
         <v>58</v>
       </c>
       <c r="G207" s="5" t="s">
-        <v>250</v>
+        <v>248</v>
       </c>
       <c r="H207" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="I207" s="5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="J207" s="5"/>
     </row>
     <row r="208" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A208" s="4">
-        <v>140102</v>
+        <v>140103</v>
       </c>
       <c r="B208" s="5" t="s">
         <v>249</v>
@@ -13118,360 +13114,360 @@
         <v>1401</v>
       </c>
       <c r="D208" s="4">
-        <v>140102</v>
+        <v>140103</v>
       </c>
       <c r="E208" s="4"/>
       <c r="F208" s="4" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="G208" s="5" t="s">
         <v>250</v>
       </c>
       <c r="H208" s="5" t="s">
-        <v>61</v>
+        <v>251</v>
       </c>
       <c r="I208" s="5" t="s">
-        <v>61</v>
+        <v>251</v>
       </c>
       <c r="J208" s="5"/>
     </row>
     <row r="209" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A209" s="4">
-        <v>140103</v>
+        <v>140104</v>
       </c>
       <c r="B209" s="5" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C209" s="4">
         <v>1401</v>
       </c>
       <c r="D209" s="4">
-        <v>140103</v>
+        <v>140104</v>
       </c>
       <c r="E209" s="4"/>
       <c r="F209" s="4" t="s">
         <v>68</v>
       </c>
       <c r="G209" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="H209" s="5" t="s">
         <v>252</v>
       </c>
-      <c r="H209" s="5" t="s">
-        <v>253</v>
-      </c>
       <c r="I209" s="5" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="J209" s="5"/>
     </row>
     <row r="210" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A210" s="4">
-        <v>140104</v>
+        <v>140105</v>
       </c>
       <c r="B210" s="5" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C210" s="4">
         <v>1401</v>
       </c>
       <c r="D210" s="4">
-        <v>140104</v>
+        <v>140105</v>
       </c>
       <c r="E210" s="4"/>
       <c r="F210" s="4" t="s">
         <v>68</v>
       </c>
       <c r="G210" s="5" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="H210" s="5" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="I210" s="5" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="J210" s="5"/>
     </row>
     <row r="211" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A211" s="4">
-        <v>140105</v>
+        <v>140106</v>
       </c>
       <c r="B211" s="5" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C211" s="4">
         <v>1401</v>
       </c>
       <c r="D211" s="4">
-        <v>140105</v>
+        <v>140106</v>
       </c>
       <c r="E211" s="4"/>
       <c r="F211" s="4" t="s">
         <v>68</v>
       </c>
       <c r="G211" s="5" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="H211" s="5" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="I211" s="5" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="J211" s="5"/>
     </row>
     <row r="212" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A212" s="4">
-        <v>140106</v>
+        <v>140107</v>
       </c>
       <c r="B212" s="5" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C212" s="4">
         <v>1401</v>
       </c>
       <c r="D212" s="4">
-        <v>140106</v>
+        <v>140107</v>
       </c>
       <c r="E212" s="4"/>
       <c r="F212" s="4" t="s">
         <v>68</v>
       </c>
       <c r="G212" s="5" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="H212" s="5" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="I212" s="5" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="J212" s="5"/>
     </row>
     <row r="213" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A213" s="4">
-        <v>140107</v>
+        <v>140108</v>
       </c>
       <c r="B213" s="5" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C213" s="4">
         <v>1401</v>
       </c>
       <c r="D213" s="4">
-        <v>140107</v>
+        <v>140108</v>
       </c>
       <c r="E213" s="4"/>
       <c r="F213" s="4" t="s">
         <v>68</v>
       </c>
       <c r="G213" s="5" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="H213" s="5" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="I213" s="5" t="s">
-        <v>257</v>
+        <v>256</v>
       </c>
       <c r="J213" s="5"/>
     </row>
     <row r="214" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A214" s="4">
-        <v>140108</v>
+        <v>140109</v>
       </c>
       <c r="B214" s="5" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C214" s="4">
         <v>1401</v>
       </c>
       <c r="D214" s="4">
-        <v>140108</v>
+        <v>140109</v>
       </c>
       <c r="E214" s="4"/>
       <c r="F214" s="4" t="s">
         <v>68</v>
       </c>
       <c r="G214" s="5" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="H214" s="5" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="I214" s="5" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="J214" s="5"/>
     </row>
     <row r="215" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A215" s="4">
-        <v>140109</v>
+        <v>140110</v>
       </c>
       <c r="B215" s="5" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C215" s="4">
         <v>1401</v>
       </c>
       <c r="D215" s="4">
-        <v>140109</v>
+        <v>140110</v>
       </c>
       <c r="E215" s="4"/>
       <c r="F215" s="4" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="G215" s="5" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="H215" s="5" t="s">
-        <v>259</v>
+        <v>64</v>
       </c>
       <c r="I215" s="5" t="s">
-        <v>259</v>
+        <v>64</v>
       </c>
       <c r="J215" s="5"/>
     </row>
     <row r="216" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A216" s="4">
-        <v>140110</v>
+        <v>140111</v>
       </c>
       <c r="B216" s="5" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="C216" s="4">
         <v>1401</v>
       </c>
       <c r="D216" s="4">
-        <v>140110</v>
+        <v>140111</v>
       </c>
       <c r="E216" s="4"/>
       <c r="F216" s="4" t="s">
         <v>58</v>
       </c>
       <c r="G216" s="5" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="H216" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="I216" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J216" s="5"/>
     </row>
     <row r="217" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A217" s="4">
-        <v>140111</v>
+        <v>140112</v>
       </c>
       <c r="B217" s="5" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="C217" s="4">
         <v>1401</v>
       </c>
       <c r="D217" s="4">
-        <v>140111</v>
+        <v>140112</v>
       </c>
       <c r="E217" s="4"/>
       <c r="F217" s="4" t="s">
         <v>58</v>
       </c>
       <c r="G217" s="5" t="s">
-        <v>252</v>
+        <v>259</v>
       </c>
       <c r="H217" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="I217" s="5" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="J217" s="5"/>
     </row>
     <row r="218" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A218" s="4">
-        <v>140112</v>
+        <v>140113</v>
       </c>
       <c r="B218" s="5" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C218" s="4">
         <v>1401</v>
       </c>
       <c r="D218" s="4">
-        <v>140112</v>
+        <v>140113</v>
       </c>
       <c r="E218" s="4"/>
       <c r="F218" s="4" t="s">
         <v>58</v>
       </c>
       <c r="G218" s="5" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="H218" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="I218" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J218" s="5"/>
     </row>
     <row r="219" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A219" s="4">
-        <v>140113</v>
+        <v>1402</v>
       </c>
       <c r="B219" s="5" t="s">
         <v>260</v>
       </c>
       <c r="C219" s="4">
-        <v>1401</v>
+        <v>14</v>
       </c>
       <c r="D219" s="4">
-        <v>140113</v>
+        <v>1402</v>
       </c>
       <c r="E219" s="4"/>
       <c r="F219" s="4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G219" s="5" t="s">
         <v>261</v>
       </c>
-      <c r="H219" s="5" t="s">
-        <v>65</v>
-      </c>
+      <c r="H219" s="5"/>
       <c r="I219" s="5" t="s">
-        <v>65</v>
+        <v>260</v>
       </c>
       <c r="J219" s="5"/>
     </row>
     <row r="220" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A220" s="4">
-        <v>1402</v>
+        <v>140201</v>
       </c>
       <c r="B220" s="5" t="s">
         <v>262</v>
       </c>
       <c r="C220" s="4">
-        <v>14</v>
+        <v>1402</v>
       </c>
       <c r="D220" s="4">
-        <v>1402</v>
+        <v>140201</v>
       </c>
       <c r="E220" s="4"/>
       <c r="F220" s="4" t="s">
-        <v>55</v>
+        <v>68</v>
       </c>
       <c r="G220" s="5" t="s">
         <v>263</v>
       </c>
-      <c r="H220" s="5"/>
+      <c r="H220" s="5" t="s">
+        <v>90</v>
+      </c>
       <c r="I220" s="5" t="s">
-        <v>262</v>
+        <v>90</v>
       </c>
       <c r="J220" s="5"/>
     </row>
     <row r="221" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A221" s="4">
-        <v>140201</v>
+        <v>140202</v>
       </c>
       <c r="B221" s="5" t="s">
         <v>264</v>
@@ -13480,7 +13476,7 @@
         <v>1402</v>
       </c>
       <c r="D221" s="4">
-        <v>140201</v>
+        <v>140202</v>
       </c>
       <c r="E221" s="4"/>
       <c r="F221" s="4" t="s">
@@ -13490,72 +13486,72 @@
         <v>265</v>
       </c>
       <c r="H221" s="5" t="s">
-        <v>90</v>
+        <v>69</v>
       </c>
       <c r="I221" s="5" t="s">
-        <v>90</v>
+        <v>69</v>
       </c>
       <c r="J221" s="5"/>
     </row>
     <row r="222" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A222" s="4">
-        <v>140202</v>
+        <v>140203</v>
       </c>
       <c r="B222" s="5" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="C222" s="4">
         <v>1402</v>
       </c>
       <c r="D222" s="4">
-        <v>140202</v>
+        <v>140203</v>
       </c>
       <c r="E222" s="4"/>
       <c r="F222" s="4" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="G222" s="5" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="H222" s="5" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="I222" s="5" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="J222" s="5"/>
     </row>
     <row r="223" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A223" s="4">
-        <v>140203</v>
+        <v>140204</v>
       </c>
       <c r="B223" s="5" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="C223" s="4">
         <v>1402</v>
       </c>
       <c r="D223" s="4">
-        <v>140203</v>
+        <v>140204</v>
       </c>
       <c r="E223" s="4"/>
       <c r="F223" s="4" t="s">
         <v>58</v>
       </c>
       <c r="G223" s="5" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="H223" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="I223" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J223" s="5"/>
     </row>
     <row r="224" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A224" s="4">
-        <v>140204</v>
+        <v>140205</v>
       </c>
       <c r="B224" s="5" t="s">
         <v>266</v>
@@ -13564,417 +13560,415 @@
         <v>1402</v>
       </c>
       <c r="D224" s="4">
-        <v>140204</v>
+        <v>140205</v>
       </c>
       <c r="E224" s="4"/>
       <c r="F224" s="4" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="G224" s="5" t="s">
         <v>267</v>
       </c>
       <c r="H224" s="5" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="I224" s="5" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="J224" s="5"/>
     </row>
     <row r="225" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A225" s="4">
-        <v>140205</v>
+        <v>140206</v>
       </c>
       <c r="B225" s="5" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C225" s="4">
         <v>1402</v>
       </c>
       <c r="D225" s="4">
-        <v>140205</v>
+        <v>140206</v>
       </c>
       <c r="E225" s="4"/>
       <c r="F225" s="4" t="s">
         <v>68</v>
       </c>
       <c r="G225" s="5" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="H225" s="5" t="s">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="I225" s="5" t="s">
-        <v>69</v>
+        <v>90</v>
       </c>
       <c r="J225" s="5"/>
     </row>
     <row r="226" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A226" s="4">
-        <v>140206</v>
+        <v>140207</v>
       </c>
       <c r="B226" s="5" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C226" s="4">
         <v>1402</v>
       </c>
       <c r="D226" s="4">
-        <v>140206</v>
+        <v>140207</v>
       </c>
       <c r="E226" s="4"/>
       <c r="F226" s="4" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="G226" s="5" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="H226" s="5" t="s">
-        <v>90</v>
+        <v>64</v>
       </c>
       <c r="I226" s="5" t="s">
-        <v>90</v>
+        <v>64</v>
       </c>
       <c r="J226" s="5"/>
     </row>
     <row r="227" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A227" s="4">
-        <v>140207</v>
+        <v>140208</v>
       </c>
       <c r="B227" s="5" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C227" s="4">
         <v>1402</v>
       </c>
       <c r="D227" s="4">
-        <v>140207</v>
+        <v>140208</v>
       </c>
       <c r="E227" s="4"/>
       <c r="F227" s="4" t="s">
         <v>58</v>
       </c>
       <c r="G227" s="5" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="H227" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="I227" s="5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="J227" s="5"/>
     </row>
     <row r="228" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A228" s="4">
-        <v>140208</v>
+        <v>1403</v>
       </c>
       <c r="B228" s="5" t="s">
         <v>268</v>
       </c>
       <c r="C228" s="4">
-        <v>1402</v>
+        <v>14</v>
       </c>
       <c r="D228" s="4">
-        <v>140208</v>
+        <v>1403</v>
       </c>
       <c r="E228" s="4"/>
       <c r="F228" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="G228" s="5" t="s">
-        <v>269</v>
-      </c>
-      <c r="H228" s="5" t="s">
-        <v>65</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="G228" s="18" t="s">
+        <v>350</v>
+      </c>
+      <c r="H228" s="5"/>
       <c r="I228" s="5" t="s">
-        <v>65</v>
+        <v>268</v>
       </c>
       <c r="J228" s="5"/>
     </row>
     <row r="229" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A229" s="4">
-        <v>1403</v>
+        <v>1404</v>
       </c>
       <c r="B229" s="5" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C229" s="4">
         <v>14</v>
       </c>
       <c r="D229" s="4">
-        <v>1403</v>
+        <v>1404</v>
       </c>
       <c r="E229" s="4"/>
       <c r="F229" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G229" s="18" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="H229" s="5"/>
       <c r="I229" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="J229" s="5"/>
+    </row>
+    <row r="230" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A230" s="4">
+        <v>1405</v>
+      </c>
+      <c r="B230" s="1" t="s">
         <v>270</v>
-      </c>
-      <c r="J229" s="5"/>
-    </row>
-    <row r="230" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A230" s="4">
-        <v>1404</v>
-      </c>
-      <c r="B230" s="5" t="s">
-        <v>271</v>
       </c>
       <c r="C230" s="4">
         <v>14</v>
       </c>
       <c r="D230" s="4">
-        <v>1404</v>
+        <v>1405</v>
       </c>
       <c r="E230" s="4"/>
       <c r="F230" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="G230" s="18" t="s">
-        <v>351</v>
-      </c>
-      <c r="H230" s="5"/>
-      <c r="I230" s="5" t="s">
+      <c r="G230" s="1" t="s">
         <v>271</v>
       </c>
+      <c r="H230" s="1"/>
+      <c r="I230" s="1"/>
       <c r="J230" s="5"/>
     </row>
-    <row r="231" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A231" s="4">
-        <v>1405</v>
-      </c>
-      <c r="B231" s="1" t="s">
-        <v>272</v>
+        <v>15</v>
+      </c>
+      <c r="B231" s="18" t="s">
+        <v>346</v>
       </c>
       <c r="C231" s="4">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="D231" s="4">
-        <v>1405</v>
+        <v>15</v>
       </c>
       <c r="E231" s="4"/>
       <c r="F231" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G231" s="1" t="s">
-        <v>273</v>
-      </c>
-      <c r="H231" s="1"/>
-      <c r="I231" s="1"/>
+        <v>52</v>
+      </c>
+      <c r="G231" s="5"/>
+      <c r="H231" s="5"/>
+      <c r="I231" s="5" t="s">
+        <v>272</v>
+      </c>
       <c r="J231" s="5"/>
     </row>
     <row r="232" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A232" s="4">
+        <v>1501</v>
+      </c>
+      <c r="B232" s="18" t="s">
+        <v>347</v>
+      </c>
+      <c r="C232" s="4">
         <v>15</v>
       </c>
-      <c r="B232" s="18" t="s">
-        <v>348</v>
-      </c>
-      <c r="C232" s="4">
-        <v>1</v>
-      </c>
       <c r="D232" s="4">
-        <v>15</v>
+        <v>1501</v>
       </c>
       <c r="E232" s="4"/>
       <c r="F232" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G232" s="5"/>
+        <v>55</v>
+      </c>
+      <c r="G232" s="18" t="s">
+        <v>351</v>
+      </c>
       <c r="H232" s="5"/>
-      <c r="I232" s="5" t="s">
-        <v>274</v>
+      <c r="I232" s="18" t="s">
+        <v>347</v>
       </c>
       <c r="J232" s="5"/>
     </row>
     <row r="233" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A233" s="4">
-        <v>1501</v>
+        <v>1502</v>
       </c>
       <c r="B233" s="18" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C233" s="4">
         <v>15</v>
       </c>
       <c r="D233" s="4">
-        <v>1501</v>
+        <v>1502</v>
       </c>
       <c r="E233" s="4"/>
       <c r="F233" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G233" s="18" t="s">
-        <v>353</v>
+        <v>359</v>
       </c>
       <c r="H233" s="5"/>
       <c r="I233" s="18" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="J233" s="5"/>
     </row>
     <row r="234" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A234" s="4">
-        <v>1502</v>
-      </c>
-      <c r="B234" s="18" t="s">
-        <v>350</v>
+        <v>1503</v>
+      </c>
+      <c r="B234" s="5" t="s">
+        <v>273</v>
       </c>
       <c r="C234" s="4">
         <v>15</v>
       </c>
       <c r="D234" s="4">
-        <v>1502</v>
+        <v>1503</v>
       </c>
       <c r="E234" s="4"/>
       <c r="F234" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="G234" s="18" t="s">
-        <v>361</v>
+      <c r="G234" s="5" t="s">
+        <v>274</v>
       </c>
       <c r="H234" s="5"/>
-      <c r="I234" s="18" t="s">
-        <v>350</v>
+      <c r="I234" s="5" t="s">
+        <v>273</v>
       </c>
       <c r="J234" s="5"/>
     </row>
     <row r="235" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A235" s="4">
-        <v>1503</v>
-      </c>
-      <c r="B235" s="5" t="s">
+      <c r="A235" s="6">
+        <v>1504</v>
+      </c>
+      <c r="B235" s="7" t="s">
         <v>275</v>
       </c>
-      <c r="C235" s="4">
+      <c r="C235" s="6">
         <v>15</v>
       </c>
-      <c r="D235" s="4">
-        <v>1503</v>
-      </c>
-      <c r="E235" s="4"/>
-      <c r="F235" s="4" t="s">
+      <c r="D235" s="6">
+        <v>1504</v>
+      </c>
+      <c r="E235" s="6"/>
+      <c r="F235" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="G235" s="5" t="s">
+      <c r="G235" s="19" t="s">
+        <v>358</v>
+      </c>
+      <c r="H235" s="7"/>
+      <c r="I235" s="7" t="s">
+        <v>275</v>
+      </c>
+      <c r="J235" s="5"/>
+    </row>
+    <row r="236" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A236" s="8">
+        <v>16</v>
+      </c>
+      <c r="B236" s="9" t="s">
         <v>276</v>
       </c>
-      <c r="H235" s="5"/>
-      <c r="I235" s="5" t="s">
-        <v>275</v>
-      </c>
-      <c r="J235" s="5"/>
-    </row>
-    <row r="236" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A236" s="6">
-        <v>1504</v>
-      </c>
-      <c r="B236" s="7" t="s">
-        <v>277</v>
-      </c>
-      <c r="C236" s="6">
-        <v>15</v>
-      </c>
-      <c r="D236" s="6">
-        <v>1504</v>
-      </c>
-      <c r="E236" s="6"/>
-      <c r="F236" s="6" t="s">
+      <c r="C236" s="8">
+        <v>1</v>
+      </c>
+      <c r="D236" s="8">
+        <v>16</v>
+      </c>
+      <c r="E236" s="8"/>
+      <c r="F236" s="8" t="s">
+        <v>52</v>
+      </c>
+      <c r="G236" s="9"/>
+      <c r="H236" s="9"/>
+      <c r="I236" s="9" t="s">
+        <v>276</v>
+      </c>
+      <c r="J236" s="5"/>
+    </row>
+    <row r="237" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A237" s="4">
+        <v>1601</v>
+      </c>
+      <c r="B237" s="10" t="s">
+        <v>362</v>
+      </c>
+      <c r="C237" s="4">
+        <v>16</v>
+      </c>
+      <c r="D237" s="4">
+        <v>1601</v>
+      </c>
+      <c r="E237" s="4"/>
+      <c r="F237" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="G236" s="19" t="s">
-        <v>360</v>
-      </c>
-      <c r="H236" s="7"/>
-      <c r="I236" s="7" t="s">
-        <v>277</v>
-      </c>
-      <c r="J236" s="5"/>
-    </row>
-    <row r="237" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A237" s="8">
-        <v>16</v>
-      </c>
-      <c r="B237" s="9" t="s">
-        <v>278</v>
-      </c>
-      <c r="C237" s="8">
-        <v>1</v>
-      </c>
-      <c r="D237" s="8">
-        <v>16</v>
-      </c>
-      <c r="E237" s="8"/>
-      <c r="F237" s="8" t="s">
-        <v>52</v>
-      </c>
-      <c r="G237" s="9"/>
-      <c r="H237" s="9"/>
-      <c r="I237" s="9" t="s">
-        <v>278</v>
+      <c r="G237" s="5" t="s">
+        <v>279</v>
+      </c>
+      <c r="H237" s="5"/>
+      <c r="I237" s="10" t="s">
+        <v>362</v>
       </c>
       <c r="J237" s="5"/>
     </row>
-    <row r="238" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A238" s="4">
-        <v>1601</v>
-      </c>
-      <c r="B238" s="10" t="s">
-        <v>364</v>
+        <v>1602</v>
+      </c>
+      <c r="B238" s="1" t="s">
+        <v>284</v>
       </c>
       <c r="C238" s="4">
         <v>16</v>
       </c>
       <c r="D238" s="4">
-        <v>1601</v>
+        <v>1602</v>
       </c>
       <c r="E238" s="4"/>
       <c r="F238" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G238" s="5" t="s">
-        <v>281</v>
-      </c>
-      <c r="H238" s="5"/>
-      <c r="I238" s="10" t="s">
-        <v>364</v>
+        <v>285</v>
+      </c>
+      <c r="I238" s="1" t="s">
+        <v>284</v>
       </c>
       <c r="J238" s="5"/>
     </row>
-    <row r="239" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A239" s="4">
-        <v>1602</v>
-      </c>
-      <c r="B239" s="1" t="s">
-        <v>286</v>
+        <v>1603</v>
+      </c>
+      <c r="B239" s="5" t="s">
+        <v>280</v>
       </c>
       <c r="C239" s="4">
         <v>16</v>
       </c>
       <c r="D239" s="4">
-        <v>1602</v>
+        <v>1603</v>
       </c>
       <c r="E239" s="4"/>
       <c r="F239" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G239" s="5" t="s">
-        <v>287</v>
-      </c>
-      <c r="I239" s="1" t="s">
-        <v>286</v>
+        <v>281</v>
+      </c>
+      <c r="H239" s="5"/>
+      <c r="I239" s="5" t="s">
+        <v>280</v>
       </c>
       <c r="J239" s="5"/>
     </row>
     <row r="240" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A240" s="4">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="B240" s="5" t="s">
         <v>282</v>
@@ -13983,7 +13977,7 @@
         <v>16</v>
       </c>
       <c r="D240" s="4">
-        <v>1603</v>
+        <v>1604</v>
       </c>
       <c r="E240" s="4"/>
       <c r="F240" s="4" t="s">
@@ -14000,94 +13994,92 @@
     </row>
     <row r="241" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A241" s="4">
-        <v>1604</v>
+        <v>1605</v>
       </c>
       <c r="B241" s="5" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="C241" s="4">
         <v>16</v>
       </c>
       <c r="D241" s="4">
-        <v>1604</v>
+        <v>1605</v>
       </c>
       <c r="E241" s="4"/>
       <c r="F241" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G241" s="5" t="s">
-        <v>285</v>
+        <v>278</v>
       </c>
       <c r="H241" s="5"/>
       <c r="I241" s="5" t="s">
-        <v>284</v>
+        <v>277</v>
       </c>
       <c r="J241" s="5"/>
     </row>
     <row r="242" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A242" s="4">
-        <v>1605</v>
-      </c>
-      <c r="B242" s="5" t="s">
-        <v>279</v>
-      </c>
-      <c r="C242" s="4">
+      <c r="A242" s="6">
+        <v>1606</v>
+      </c>
+      <c r="B242" s="20" t="s">
+        <v>360</v>
+      </c>
+      <c r="C242" s="6">
         <v>16</v>
       </c>
-      <c r="D242" s="4">
-        <v>1605</v>
-      </c>
-      <c r="E242" s="4"/>
-      <c r="F242" s="4" t="s">
+      <c r="D242" s="6">
+        <v>1607</v>
+      </c>
+      <c r="E242" s="6"/>
+      <c r="F242" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="G242" s="5" t="s">
-        <v>280</v>
-      </c>
-      <c r="H242" s="5"/>
-      <c r="I242" s="5" t="s">
-        <v>279</v>
+      <c r="G242" s="20" t="s">
+        <v>361</v>
+      </c>
+      <c r="H242" s="7"/>
+      <c r="I242" s="20" t="s">
+        <v>360</v>
       </c>
       <c r="J242" s="5"/>
     </row>
     <row r="243" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A243" s="6">
-        <v>1606</v>
-      </c>
-      <c r="B243" s="20" t="s">
-        <v>362</v>
-      </c>
-      <c r="C243" s="6">
-        <v>16</v>
-      </c>
-      <c r="D243" s="6">
-        <v>1607</v>
-      </c>
-      <c r="E243" s="6"/>
-      <c r="F243" s="6" t="s">
-        <v>55</v>
-      </c>
-      <c r="G243" s="20" t="s">
-        <v>363</v>
-      </c>
-      <c r="H243" s="7"/>
-      <c r="I243" s="20" t="s">
-        <v>362</v>
+      <c r="A243" s="4">
+        <v>2</v>
+      </c>
+      <c r="B243" s="5" t="s">
+        <v>286</v>
+      </c>
+      <c r="C243" s="4">
+        <v>-1</v>
+      </c>
+      <c r="D243" s="4">
+        <v>2</v>
+      </c>
+      <c r="E243" s="4"/>
+      <c r="F243" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="G243" s="5"/>
+      <c r="H243" s="5"/>
+      <c r="I243" s="5" t="s">
+        <v>286</v>
       </c>
       <c r="J243" s="5"/>
     </row>
     <row r="244" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A244" s="4">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="B244" s="5" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C244" s="4">
-        <v>-1</v>
+        <v>2</v>
       </c>
       <c r="D244" s="4">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="E244" s="4"/>
       <c r="F244" s="4" t="s">
@@ -14096,37 +14088,39 @@
       <c r="G244" s="5"/>
       <c r="H244" s="5"/>
       <c r="I244" s="5" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="J244" s="5"/>
     </row>
     <row r="245" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A245" s="4">
+        <v>2110</v>
+      </c>
+      <c r="B245" s="5" t="s">
+        <v>288</v>
+      </c>
+      <c r="C245" s="4">
         <v>21</v>
       </c>
-      <c r="B245" s="5" t="s">
-        <v>289</v>
-      </c>
-      <c r="C245" s="4">
-        <v>2</v>
-      </c>
       <c r="D245" s="4">
-        <v>21</v>
+        <v>2110</v>
       </c>
       <c r="E245" s="4"/>
       <c r="F245" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G245" s="5"/>
+        <v>55</v>
+      </c>
+      <c r="G245" s="5" t="s">
+        <v>289</v>
+      </c>
       <c r="H245" s="5"/>
       <c r="I245" s="5" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="J245" s="5"/>
     </row>
     <row r="246" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A246" s="4">
-        <v>2110</v>
+        <v>2111</v>
       </c>
       <c r="B246" s="5" t="s">
         <v>290</v>
@@ -14135,7 +14129,7 @@
         <v>21</v>
       </c>
       <c r="D246" s="4">
-        <v>2110</v>
+        <v>2111</v>
       </c>
       <c r="E246" s="4"/>
       <c r="F246" s="4" t="s">
@@ -14152,24 +14146,22 @@
     </row>
     <row r="247" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A247" s="4">
-        <v>2111</v>
+        <v>22</v>
       </c>
       <c r="B247" s="5" t="s">
         <v>292</v>
       </c>
       <c r="C247" s="4">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="D247" s="4">
-        <v>2111</v>
+        <v>22</v>
       </c>
       <c r="E247" s="4"/>
       <c r="F247" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G247" s="5" t="s">
-        <v>293</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G247" s="5"/>
       <c r="H247" s="5"/>
       <c r="I247" s="5" t="s">
         <v>292</v>
@@ -14178,31 +14170,33 @@
     </row>
     <row r="248" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A248" s="4">
+        <v>2201</v>
+      </c>
+      <c r="B248" s="5" t="s">
+        <v>293</v>
+      </c>
+      <c r="C248" s="4">
         <v>22</v>
       </c>
-      <c r="B248" s="5" t="s">
-        <v>294</v>
-      </c>
-      <c r="C248" s="4">
-        <v>2</v>
-      </c>
       <c r="D248" s="4">
-        <v>22</v>
+        <v>2201</v>
       </c>
       <c r="E248" s="4"/>
       <c r="F248" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G248" s="5"/>
+        <v>55</v>
+      </c>
+      <c r="G248" s="5" t="s">
+        <v>294</v>
+      </c>
       <c r="H248" s="5"/>
       <c r="I248" s="5" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="J248" s="5"/>
     </row>
     <row r="249" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A249" s="4">
-        <v>2201</v>
+        <v>2202</v>
       </c>
       <c r="B249" s="5" t="s">
         <v>295</v>
@@ -14211,7 +14205,7 @@
         <v>22</v>
       </c>
       <c r="D249" s="4">
-        <v>2201</v>
+        <v>2202</v>
       </c>
       <c r="E249" s="4"/>
       <c r="F249" s="4" t="s">
@@ -14228,7 +14222,7 @@
     </row>
     <row r="250" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A250" s="4">
-        <v>2202</v>
+        <v>2203</v>
       </c>
       <c r="B250" s="5" t="s">
         <v>297</v>
@@ -14237,7 +14231,7 @@
         <v>22</v>
       </c>
       <c r="D250" s="4">
-        <v>2202</v>
+        <v>2203</v>
       </c>
       <c r="E250" s="4"/>
       <c r="F250" s="4" t="s">
@@ -14254,24 +14248,22 @@
     </row>
     <row r="251" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A251" s="4">
-        <v>2203</v>
+        <v>23</v>
       </c>
       <c r="B251" s="5" t="s">
         <v>299</v>
       </c>
       <c r="C251" s="4">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="D251" s="4">
-        <v>2203</v>
+        <v>23</v>
       </c>
       <c r="E251" s="4"/>
       <c r="F251" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G251" s="5" t="s">
-        <v>300</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G251" s="5"/>
       <c r="H251" s="5"/>
       <c r="I251" s="5" t="s">
         <v>299</v>
@@ -14280,31 +14272,33 @@
     </row>
     <row r="252" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A252" s="4">
+        <v>2301</v>
+      </c>
+      <c r="B252" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="C252" s="4">
         <v>23</v>
       </c>
-      <c r="B252" s="5" t="s">
-        <v>301</v>
-      </c>
-      <c r="C252" s="4">
-        <v>2</v>
-      </c>
       <c r="D252" s="4">
-        <v>23</v>
+        <v>2301</v>
       </c>
       <c r="E252" s="4"/>
       <c r="F252" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G252" s="5"/>
+        <v>55</v>
+      </c>
+      <c r="G252" s="5" t="s">
+        <v>301</v>
+      </c>
       <c r="H252" s="5"/>
       <c r="I252" s="5" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J252" s="5"/>
     </row>
     <row r="253" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A253" s="4">
-        <v>2301</v>
+        <v>2302</v>
       </c>
       <c r="B253" s="5" t="s">
         <v>302</v>
@@ -14313,15 +14307,13 @@
         <v>23</v>
       </c>
       <c r="D253" s="4">
-        <v>2301</v>
+        <v>2302</v>
       </c>
       <c r="E253" s="4"/>
       <c r="F253" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G253" s="5" t="s">
-        <v>303</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G253" s="5"/>
       <c r="H253" s="5"/>
       <c r="I253" s="5" t="s">
         <v>302</v>
@@ -14330,107 +14322,109 @@
     </row>
     <row r="254" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A254" s="4">
+        <v>23021</v>
+      </c>
+      <c r="B254" s="5" t="s">
+        <v>303</v>
+      </c>
+      <c r="C254" s="4">
         <v>2302</v>
       </c>
-      <c r="B254" s="5" t="s">
-        <v>304</v>
-      </c>
-      <c r="C254" s="4">
-        <v>23</v>
-      </c>
       <c r="D254" s="4">
-        <v>2302</v>
+        <v>23021</v>
       </c>
       <c r="E254" s="4"/>
       <c r="F254" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G254" s="5"/>
+        <v>55</v>
+      </c>
+      <c r="G254" s="5" t="s">
+        <v>304</v>
+      </c>
       <c r="H254" s="5"/>
       <c r="I254" s="5" t="s">
-        <v>304</v>
+        <v>305</v>
       </c>
       <c r="J254" s="5"/>
     </row>
     <row r="255" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A255" s="4">
-        <v>23021</v>
+        <v>23022</v>
       </c>
       <c r="B255" s="5" t="s">
-        <v>305</v>
+        <v>306</v>
       </c>
       <c r="C255" s="4">
         <v>2302</v>
       </c>
       <c r="D255" s="4">
-        <v>23021</v>
+        <v>23022</v>
       </c>
       <c r="E255" s="4"/>
       <c r="F255" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G255" s="5" t="s">
-        <v>306</v>
+        <v>307</v>
       </c>
       <c r="H255" s="5"/>
       <c r="I255" s="5" t="s">
-        <v>307</v>
+        <v>308</v>
       </c>
       <c r="J255" s="5"/>
     </row>
     <row r="256" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A256" s="4">
-        <v>23022</v>
+        <v>2303</v>
       </c>
       <c r="B256" s="5" t="s">
-        <v>308</v>
+        <v>272</v>
       </c>
       <c r="C256" s="4">
-        <v>2302</v>
+        <v>23</v>
       </c>
       <c r="D256" s="4">
-        <v>23022</v>
+        <v>2303</v>
       </c>
       <c r="E256" s="4"/>
       <c r="F256" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G256" s="5" t="s">
-        <v>309</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G256" s="5"/>
       <c r="H256" s="5"/>
       <c r="I256" s="5" t="s">
-        <v>310</v>
+        <v>272</v>
       </c>
       <c r="J256" s="5"/>
     </row>
     <row r="257" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A257" s="4">
+        <v>23031</v>
+      </c>
+      <c r="B257" s="10" t="s">
+        <v>309</v>
+      </c>
+      <c r="C257" s="4">
         <v>2303</v>
       </c>
-      <c r="B257" s="5" t="s">
-        <v>274</v>
-      </c>
-      <c r="C257" s="4">
-        <v>23</v>
-      </c>
       <c r="D257" s="4">
-        <v>2303</v>
+        <v>23031</v>
       </c>
       <c r="E257" s="4"/>
       <c r="F257" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G257" s="5"/>
+        <v>55</v>
+      </c>
+      <c r="G257" s="10" t="s">
+        <v>310</v>
+      </c>
       <c r="H257" s="5"/>
-      <c r="I257" s="5" t="s">
-        <v>274</v>
+      <c r="I257" s="10" t="s">
+        <v>309</v>
       </c>
       <c r="J257" s="5"/>
     </row>
     <row r="258" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A258" s="4">
-        <v>23031</v>
+        <v>23032</v>
       </c>
       <c r="B258" s="10" t="s">
         <v>311</v>
@@ -14439,7 +14433,7 @@
         <v>2303</v>
       </c>
       <c r="D258" s="4">
-        <v>23031</v>
+        <v>23032</v>
       </c>
       <c r="E258" s="4"/>
       <c r="F258" s="4" t="s">
@@ -14456,7 +14450,7 @@
     </row>
     <row r="259" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A259" s="4">
-        <v>23032</v>
+        <v>23033</v>
       </c>
       <c r="B259" s="10" t="s">
         <v>313</v>
@@ -14465,7 +14459,7 @@
         <v>2303</v>
       </c>
       <c r="D259" s="4">
-        <v>23032</v>
+        <v>23033</v>
       </c>
       <c r="E259" s="4"/>
       <c r="F259" s="4" t="s">
@@ -14482,7 +14476,7 @@
     </row>
     <row r="260" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A260" s="4">
-        <v>23033</v>
+        <v>23034</v>
       </c>
       <c r="B260" s="10" t="s">
         <v>315</v>
@@ -14491,7 +14485,7 @@
         <v>2303</v>
       </c>
       <c r="D260" s="4">
-        <v>23033</v>
+        <v>23034</v>
       </c>
       <c r="E260" s="4"/>
       <c r="F260" s="4" t="s">
@@ -14508,7 +14502,7 @@
     </row>
     <row r="261" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A261" s="4">
-        <v>23034</v>
+        <v>23035</v>
       </c>
       <c r="B261" s="10" t="s">
         <v>317</v>
@@ -14517,7 +14511,7 @@
         <v>2303</v>
       </c>
       <c r="D261" s="4">
-        <v>23034</v>
+        <v>23035</v>
       </c>
       <c r="E261" s="4"/>
       <c r="F261" s="4" t="s">
@@ -14534,7 +14528,7 @@
     </row>
     <row r="262" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A262" s="4">
-        <v>23035</v>
+        <v>23036</v>
       </c>
       <c r="B262" s="10" t="s">
         <v>319</v>
@@ -14543,7 +14537,7 @@
         <v>2303</v>
       </c>
       <c r="D262" s="4">
-        <v>23035</v>
+        <v>23036</v>
       </c>
       <c r="E262" s="4"/>
       <c r="F262" s="4" t="s">
@@ -14560,24 +14554,22 @@
     </row>
     <row r="263" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A263" s="4">
-        <v>23036</v>
+        <v>2304</v>
       </c>
       <c r="B263" s="10" t="s">
         <v>321</v>
       </c>
       <c r="C263" s="4">
-        <v>2303</v>
+        <v>23</v>
       </c>
       <c r="D263" s="4">
-        <v>23036</v>
+        <v>2304</v>
       </c>
       <c r="E263" s="4"/>
       <c r="F263" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G263" s="10" t="s">
-        <v>322</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G263" s="5"/>
       <c r="H263" s="5"/>
       <c r="I263" s="10" t="s">
         <v>321</v>
@@ -14586,131 +14578,133 @@
     </row>
     <row r="264" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A264" s="4">
+        <v>23041</v>
+      </c>
+      <c r="B264" s="10" t="s">
+        <v>322</v>
+      </c>
+      <c r="C264" s="4">
         <v>2304</v>
       </c>
-      <c r="B264" s="10" t="s">
-        <v>323</v>
-      </c>
-      <c r="C264" s="4">
-        <v>23</v>
-      </c>
       <c r="D264" s="4">
-        <v>2304</v>
+        <v>23041</v>
       </c>
       <c r="E264" s="4"/>
       <c r="F264" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G264" s="5"/>
+        <v>55</v>
+      </c>
+      <c r="G264" s="10" t="s">
+        <v>323</v>
+      </c>
       <c r="H264" s="5"/>
       <c r="I264" s="10" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="J264" s="5"/>
     </row>
     <row r="265" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A265" s="4">
-        <v>23041</v>
-      </c>
-      <c r="B265" s="10" t="s">
-        <v>324</v>
+        <v>2305</v>
+      </c>
+      <c r="B265" s="18" t="s">
+        <v>355</v>
       </c>
       <c r="C265" s="4">
-        <v>2304</v>
+        <v>23</v>
       </c>
       <c r="D265" s="4">
-        <v>23041</v>
+        <v>2305</v>
       </c>
       <c r="E265" s="4"/>
       <c r="F265" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G265" s="10" t="s">
-        <v>325</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G265" s="5"/>
       <c r="H265" s="5"/>
-      <c r="I265" s="10" t="s">
-        <v>324</v>
+      <c r="I265" s="18" t="s">
+        <v>355</v>
       </c>
       <c r="J265" s="5"/>
     </row>
     <row r="266" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A266" s="4">
-        <v>2305</v>
+        <v>23051</v>
       </c>
       <c r="B266" s="18" t="s">
         <v>357</v>
       </c>
       <c r="C266" s="4">
-        <v>23</v>
+        <v>2305</v>
       </c>
       <c r="D266" s="4">
-        <v>2305</v>
+        <v>23051</v>
       </c>
       <c r="E266" s="4"/>
       <c r="F266" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G266" s="5"/>
+        <v>55</v>
+      </c>
+      <c r="G266" s="18" t="s">
+        <v>356</v>
+      </c>
       <c r="H266" s="5"/>
       <c r="I266" s="18" t="s">
         <v>357</v>
       </c>
       <c r="J266" s="5"/>
     </row>
-    <row r="267" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="267" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A267" s="4">
-        <v>23051</v>
-      </c>
-      <c r="B267" s="18" t="s">
-        <v>359</v>
+        <v>2306</v>
+      </c>
+      <c r="B267" s="5" t="s">
+        <v>324</v>
       </c>
       <c r="C267" s="4">
-        <v>2305</v>
+        <v>23</v>
       </c>
       <c r="D267" s="4">
-        <v>23051</v>
+        <v>2306</v>
       </c>
       <c r="E267" s="4"/>
       <c r="F267" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G267" s="18" t="s">
-        <v>358</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G267" s="5"/>
       <c r="H267" s="5"/>
-      <c r="I267" s="18" t="s">
-        <v>359</v>
+      <c r="I267" s="5" t="s">
+        <v>324</v>
       </c>
       <c r="J267" s="5"/>
     </row>
-    <row r="268" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="268" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A268" s="4">
+        <v>23061</v>
+      </c>
+      <c r="B268" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="C268" s="4">
         <v>2306</v>
       </c>
-      <c r="B268" s="5" t="s">
-        <v>326</v>
-      </c>
-      <c r="C268" s="4">
-        <v>23</v>
-      </c>
       <c r="D268" s="4">
-        <v>2306</v>
+        <v>23061</v>
       </c>
       <c r="E268" s="4"/>
       <c r="F268" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G268" s="5"/>
+        <v>55</v>
+      </c>
+      <c r="G268" s="5" t="s">
+        <v>326</v>
+      </c>
       <c r="H268" s="5"/>
       <c r="I268" s="5" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="J268" s="5"/>
     </row>
-    <row r="269" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="269" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A269" s="4">
-        <v>23061</v>
+        <v>23062</v>
       </c>
       <c r="B269" s="5" t="s">
         <v>327</v>
@@ -14719,7 +14713,7 @@
         <v>2306</v>
       </c>
       <c r="D269" s="4">
-        <v>23061</v>
+        <v>23062</v>
       </c>
       <c r="E269" s="4"/>
       <c r="F269" s="4" t="s">
@@ -14734,9 +14728,9 @@
       </c>
       <c r="J269" s="5"/>
     </row>
-    <row r="270" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="270" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A270" s="4">
-        <v>23062</v>
+        <v>23063</v>
       </c>
       <c r="B270" s="5" t="s">
         <v>329</v>
@@ -14745,7 +14739,7 @@
         <v>2306</v>
       </c>
       <c r="D270" s="4">
-        <v>23062</v>
+        <v>23063</v>
       </c>
       <c r="E270" s="4"/>
       <c r="F270" s="4" t="s">
@@ -14756,191 +14750,191 @@
       </c>
       <c r="H270" s="5"/>
       <c r="I270" s="5" t="s">
-        <v>329</v>
+        <v>331</v>
       </c>
       <c r="J270" s="5"/>
     </row>
-    <row r="271" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="271" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A271" s="4">
-        <v>23063</v>
+        <v>2307</v>
       </c>
       <c r="B271" s="5" t="s">
-        <v>331</v>
+        <v>332</v>
       </c>
       <c r="C271" s="4">
-        <v>2306</v>
+        <v>23</v>
       </c>
       <c r="D271" s="4">
-        <v>23063</v>
+        <v>2307</v>
       </c>
       <c r="E271" s="4"/>
       <c r="F271" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G271" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G271" s="4"/>
+      <c r="H271" s="4"/>
+      <c r="I271" s="5" t="s">
         <v>332</v>
-      </c>
-      <c r="H271" s="5"/>
-      <c r="I271" s="5" t="s">
-        <v>333</v>
       </c>
       <c r="J271" s="5"/>
     </row>
     <row r="272" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A272" s="4">
+        <v>23071</v>
+      </c>
+      <c r="B272" s="5" t="s">
+        <v>333</v>
+      </c>
+      <c r="C272" s="4">
         <v>2307</v>
       </c>
-      <c r="B272" s="5" t="s">
-        <v>334</v>
-      </c>
-      <c r="C272" s="4">
-        <v>23</v>
-      </c>
       <c r="D272" s="4">
-        <v>2307</v>
+        <v>23071</v>
       </c>
       <c r="E272" s="4"/>
       <c r="F272" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G272" s="4"/>
+        <v>55</v>
+      </c>
+      <c r="G272" s="18" t="s">
+        <v>352</v>
+      </c>
       <c r="H272" s="4"/>
       <c r="I272" s="5" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="J272" s="5"/>
     </row>
     <row r="273" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A273" s="4">
-        <v>23071</v>
+        <v>23072</v>
       </c>
       <c r="B273" s="5" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C273" s="4">
         <v>2307</v>
       </c>
       <c r="D273" s="4">
-        <v>23071</v>
+        <v>23072</v>
       </c>
       <c r="E273" s="4"/>
       <c r="F273" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="G273" s="18" t="s">
-        <v>354</v>
-      </c>
-      <c r="H273" s="4"/>
+      <c r="G273" s="5" t="s">
+        <v>335</v>
+      </c>
+      <c r="H273" s="5"/>
       <c r="I273" s="5" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J273" s="5"/>
     </row>
     <row r="274" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A274" s="4">
-        <v>23072</v>
-      </c>
-      <c r="B274" s="5" t="s">
-        <v>336</v>
+        <v>23073</v>
+      </c>
+      <c r="B274" s="18" t="s">
+        <v>353</v>
       </c>
       <c r="C274" s="4">
         <v>2307</v>
       </c>
       <c r="D274" s="4">
-        <v>23072</v>
+        <v>23073</v>
       </c>
       <c r="E274" s="4"/>
       <c r="F274" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="G274" s="5" t="s">
-        <v>337</v>
+      <c r="G274" s="18" t="s">
+        <v>354</v>
       </c>
       <c r="H274" s="5"/>
-      <c r="I274" s="5" t="s">
-        <v>336</v>
+      <c r="I274" s="18" t="s">
+        <v>353</v>
       </c>
       <c r="J274" s="5"/>
     </row>
     <row r="275" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A275" s="4">
-        <v>23073</v>
-      </c>
-      <c r="B275" s="18" t="s">
-        <v>355</v>
+        <v>24</v>
+      </c>
+      <c r="B275" s="5" t="s">
+        <v>336</v>
       </c>
       <c r="C275" s="4">
-        <v>2307</v>
+        <v>2</v>
       </c>
       <c r="D275" s="4">
-        <v>23073</v>
-      </c>
-      <c r="E275" s="4"/>
+        <v>24</v>
+      </c>
+      <c r="E275" s="5"/>
       <c r="F275" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G275" s="18" t="s">
-        <v>356</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G275" s="5"/>
       <c r="H275" s="5"/>
-      <c r="I275" s="18" t="s">
-        <v>355</v>
+      <c r="I275" s="5" t="s">
+        <v>336</v>
       </c>
       <c r="J275" s="5"/>
     </row>
     <row r="276" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A276" s="4">
+        <v>2401</v>
+      </c>
+      <c r="B276" s="5" t="s">
+        <v>337</v>
+      </c>
+      <c r="C276" s="4">
         <v>24</v>
       </c>
-      <c r="B276" s="5" t="s">
-        <v>338</v>
-      </c>
-      <c r="C276" s="4">
-        <v>2</v>
-      </c>
       <c r="D276" s="4">
-        <v>24</v>
+        <v>2401</v>
       </c>
       <c r="E276" s="5"/>
       <c r="F276" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G276" s="5"/>
+        <v>55</v>
+      </c>
+      <c r="G276" s="5" t="s">
+        <v>338</v>
+      </c>
       <c r="H276" s="5"/>
       <c r="I276" s="5" t="s">
-        <v>338</v>
+        <v>339</v>
       </c>
       <c r="J276" s="5"/>
     </row>
     <row r="277" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A277" s="4">
-        <v>2401</v>
+        <v>2402</v>
       </c>
       <c r="B277" s="5" t="s">
-        <v>339</v>
+        <v>340</v>
       </c>
       <c r="C277" s="4">
         <v>24</v>
       </c>
       <c r="D277" s="4">
-        <v>2401</v>
-      </c>
-      <c r="E277" s="5"/>
+        <v>2402</v>
+      </c>
+      <c r="E277" s="4"/>
       <c r="F277" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G277" s="5" t="s">
+        <v>341</v>
+      </c>
+      <c r="H277" s="4"/>
+      <c r="I277" s="5" t="s">
         <v>340</v>
       </c>
-      <c r="H277" s="5"/>
-      <c r="I277" s="5" t="s">
-        <v>341</v>
-      </c>
       <c r="J277" s="5"/>
     </row>
-    <row r="278" spans="1:26" x14ac:dyDescent="0.2">
+    <row r="278" spans="1:26" s="1" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A278" s="4">
-        <v>2402</v>
+        <v>2403</v>
       </c>
       <c r="B278" s="5" t="s">
         <v>342</v>
@@ -14949,111 +14943,85 @@
         <v>24</v>
       </c>
       <c r="D278" s="4">
-        <v>2402</v>
+        <v>2403</v>
       </c>
       <c r="E278" s="4"/>
       <c r="F278" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="G278" s="5" t="s">
+      <c r="G278" s="5"/>
+      <c r="I278" s="1" t="s">
+        <v>342</v>
+      </c>
+      <c r="J278" s="1" t="b">
+        <v>1</v>
+      </c>
+      <c r="K278"/>
+      <c r="L278"/>
+      <c r="M278"/>
+      <c r="N278"/>
+      <c r="O278"/>
+      <c r="P278"/>
+      <c r="Q278"/>
+      <c r="R278"/>
+      <c r="S278"/>
+      <c r="T278"/>
+      <c r="U278"/>
+      <c r="V278"/>
+      <c r="W278"/>
+      <c r="X278"/>
+      <c r="Y278"/>
+      <c r="Z278" s="11"/>
+    </row>
+    <row r="279" spans="1:26" x14ac:dyDescent="0.2">
+      <c r="A279" s="4">
+        <v>25</v>
+      </c>
+      <c r="B279" s="5" t="s">
         <v>343</v>
       </c>
-      <c r="H278" s="4"/>
-      <c r="I278" s="5" t="s">
-        <v>342</v>
-      </c>
-      <c r="J278" s="5"/>
-    </row>
-    <row r="279" spans="1:26" s="1" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A279" s="4">
-        <v>2403</v>
-      </c>
-      <c r="B279" s="5" t="s">
-        <v>344</v>
-      </c>
       <c r="C279" s="4">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="D279" s="4">
-        <v>2403</v>
+        <v>25</v>
       </c>
       <c r="E279" s="4"/>
       <c r="F279" s="4" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="G279" s="5"/>
-      <c r="I279" s="1" t="s">
-        <v>344</v>
-      </c>
-      <c r="J279" s="1" t="b">
-        <v>1</v>
-      </c>
-      <c r="K279"/>
-      <c r="L279"/>
-      <c r="M279"/>
-      <c r="N279"/>
-      <c r="O279"/>
-      <c r="P279"/>
-      <c r="Q279"/>
-      <c r="R279"/>
-      <c r="S279"/>
-      <c r="T279"/>
-      <c r="U279"/>
-      <c r="V279"/>
-      <c r="W279"/>
-      <c r="X279"/>
-      <c r="Y279"/>
-      <c r="Z279" s="11"/>
+      <c r="H279" s="5"/>
+      <c r="I279" s="5" t="s">
+        <v>343</v>
+      </c>
+      <c r="J279" s="5"/>
     </row>
     <row r="280" spans="1:26" x14ac:dyDescent="0.2">
       <c r="A280" s="4">
+        <v>2501</v>
+      </c>
+      <c r="B280" s="5" t="s">
+        <v>344</v>
+      </c>
+      <c r="C280" s="4">
         <v>25</v>
       </c>
-      <c r="B280" s="5" t="s">
+      <c r="D280" s="4">
+        <v>2501</v>
+      </c>
+      <c r="E280" s="5"/>
+      <c r="F280" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="G280" s="5" t="s">
         <v>345</v>
       </c>
-      <c r="C280" s="4">
-        <v>2</v>
-      </c>
-      <c r="D280" s="4">
-        <v>25</v>
-      </c>
-      <c r="E280" s="4"/>
-      <c r="F280" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G280" s="5"/>
       <c r="H280" s="5"/>
       <c r="I280" s="5" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="J280" s="5"/>
-    </row>
-    <row r="281" spans="1:26" x14ac:dyDescent="0.2">
-      <c r="A281" s="4">
-        <v>2501</v>
-      </c>
-      <c r="B281" s="5" t="s">
-        <v>346</v>
-      </c>
-      <c r="C281" s="4">
-        <v>25</v>
-      </c>
-      <c r="D281" s="4">
-        <v>2501</v>
-      </c>
-      <c r="E281" s="5"/>
-      <c r="F281" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G281" s="5" t="s">
-        <v>347</v>
-      </c>
-      <c r="H281" s="5"/>
-      <c r="I281" s="5" t="s">
-        <v>346</v>
-      </c>
-      <c r="J281" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>

</xml_diff>

<commit_message>
#91 prescan chirp 多电极校准工具统一 70# bug fix #86 MMD1.2优化
</commit_message>
<xml_diff>
--- a/Sources/Cuga-Calibration-Solution/Assets/Data/InitData.xlsx
+++ b/Sources/Cuga-Calibration-Solution/Assets/Data/InitData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\RiderProjects\semix\kaizhi.xuan\netcore_semix_cuga_calibration\Sources\Cuga-Calibration-Solution\Assets\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{25AF3DE6-A663-4B34-8B43-4415E0D90019}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB4AEC33-562E-4003-8312-C1D8C5B02295}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" firstSheet="1" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" firstSheet="1" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SysUser" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1402" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1394" uniqueCount="362">
   <si>
     <t>Id</t>
   </si>
@@ -1062,18 +1062,6 @@
   </si>
   <si>
     <t>CugaCalibration.ViewModels.Common.Windows.Tools.AODWaveform.ChirpGenerateAODWaveformWindowViewModel</t>
-  </si>
-  <si>
-    <t>Prescan AOD Waveform Uniformity</t>
-  </si>
-  <si>
-    <t>CugaCalibration.ViewModels.Common.Windows.Tools.AODWaveform.PrescanAODWaveformUniformityWindowViewModel</t>
-  </si>
-  <si>
-    <t>Chirp AOD Waveform Uniformity</t>
-  </si>
-  <si>
-    <t>CugaCalibration.ViewModels.Common.Windows.Tools.AODWaveform.ChirpAODWaveformUniformityWindowViewModel</t>
   </si>
   <si>
     <t>Prescan AOD Waveform Electrode Offset</t>
@@ -1341,7 +1329,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1380,9 +1368,6 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -7283,7 +7268,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:J283"/>
+  <dimension ref="A1:J281"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.625" style="2" customWidth="1"/>
@@ -13834,7 +13819,7 @@
       </c>
       <c r="J236" s="5"/>
     </row>
-    <row r="237" spans="1:10" s="13" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A237" s="4">
         <v>1602</v>
       </c>
@@ -13969,7 +13954,7 @@
         <v>17</v>
       </c>
       <c r="B242" s="12" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
       <c r="C242" s="4">
         <v>1</v>
@@ -13984,7 +13969,7 @@
       <c r="G242" s="5"/>
       <c r="H242" s="5"/>
       <c r="I242" s="12" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
       <c r="J242" s="5"/>
     </row>
@@ -13993,7 +13978,7 @@
         <v>1701</v>
       </c>
       <c r="B243" s="12" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="C243" s="4">
         <v>17</v>
@@ -14006,11 +13991,11 @@
         <v>55</v>
       </c>
       <c r="G243" s="12" t="s">
-        <v>365</v>
+        <v>361</v>
       </c>
       <c r="H243" s="5"/>
       <c r="I243" s="12" t="s">
-        <v>364</v>
+        <v>360</v>
       </c>
       <c r="J243" s="5"/>
     </row>
@@ -14448,8 +14433,8 @@
       <c r="A261" s="4">
         <v>23034</v>
       </c>
-      <c r="B261" s="5" t="s">
-        <v>323</v>
+      <c r="B261" s="12" t="s">
+        <v>355</v>
       </c>
       <c r="C261" s="4">
         <v>2303</v>
@@ -14461,12 +14446,12 @@
       <c r="F261" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="G261" s="5" t="s">
-        <v>324</v>
+      <c r="G261" s="12" t="s">
+        <v>358</v>
       </c>
       <c r="H261" s="5"/>
-      <c r="I261" s="5" t="s">
-        <v>323</v>
+      <c r="I261" s="12" t="s">
+        <v>355</v>
       </c>
       <c r="J261" s="5"/>
     </row>
@@ -14475,7 +14460,7 @@
         <v>23035</v>
       </c>
       <c r="B262" s="5" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="C262" s="4">
         <v>2303</v>
@@ -14488,11 +14473,11 @@
         <v>55</v>
       </c>
       <c r="G262" s="5" t="s">
-        <v>326</v>
+        <v>324</v>
       </c>
       <c r="H262" s="5"/>
       <c r="I262" s="5" t="s">
-        <v>325</v>
+        <v>323</v>
       </c>
       <c r="J262" s="5"/>
     </row>
@@ -14500,8 +14485,8 @@
       <c r="A263" s="4">
         <v>23036</v>
       </c>
-      <c r="B263" s="5" t="s">
-        <v>327</v>
+      <c r="B263" s="12" t="s">
+        <v>356</v>
       </c>
       <c r="C263" s="4">
         <v>2303</v>
@@ -14513,79 +14498,77 @@
       <c r="F263" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="G263" s="5" t="s">
-        <v>328</v>
+      <c r="G263" s="12" t="s">
+        <v>357</v>
       </c>
       <c r="H263" s="5"/>
-      <c r="I263" s="5" t="s">
-        <v>327</v>
+      <c r="I263" s="12" t="s">
+        <v>356</v>
       </c>
       <c r="J263" s="5"/>
     </row>
     <row r="264" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A264" s="4">
-        <v>23037</v>
-      </c>
-      <c r="B264" s="12" t="s">
-        <v>359</v>
+        <v>2304</v>
+      </c>
+      <c r="B264" s="5" t="s">
+        <v>325</v>
       </c>
       <c r="C264" s="4">
-        <v>2303</v>
+        <v>23</v>
       </c>
       <c r="D264" s="4">
-        <v>23037</v>
+        <v>2304</v>
       </c>
       <c r="E264" s="4"/>
       <c r="F264" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G264" s="12" t="s">
-        <v>362</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G264" s="5"/>
       <c r="H264" s="5"/>
-      <c r="I264" s="12" t="s">
-        <v>359</v>
+      <c r="I264" s="5" t="s">
+        <v>325</v>
       </c>
       <c r="J264" s="5"/>
     </row>
     <row r="265" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A265" s="4">
-        <v>23038</v>
-      </c>
-      <c r="B265" s="12" t="s">
-        <v>360</v>
+        <v>23041</v>
+      </c>
+      <c r="B265" s="5" t="s">
+        <v>326</v>
       </c>
       <c r="C265" s="4">
-        <v>2303</v>
+        <v>2304</v>
       </c>
       <c r="D265" s="4">
-        <v>23038</v>
+        <v>23041</v>
       </c>
       <c r="E265" s="4"/>
       <c r="F265" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="G265" s="12" t="s">
-        <v>361</v>
+      <c r="G265" s="5" t="s">
+        <v>327</v>
       </c>
       <c r="H265" s="5"/>
-      <c r="I265" s="12" t="s">
-        <v>360</v>
+      <c r="I265" s="5" t="s">
+        <v>326</v>
       </c>
       <c r="J265" s="5"/>
     </row>
     <row r="266" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A266" s="4">
-        <v>2304</v>
+        <v>2305</v>
       </c>
       <c r="B266" s="5" t="s">
-        <v>329</v>
+        <v>39</v>
       </c>
       <c r="C266" s="4">
         <v>23</v>
       </c>
       <c r="D266" s="4">
-        <v>2304</v>
+        <v>2305</v>
       </c>
       <c r="E266" s="4"/>
       <c r="F266" s="4" t="s">
@@ -14594,48 +14577,48 @@
       <c r="G266" s="5"/>
       <c r="H266" s="5"/>
       <c r="I266" s="5" t="s">
-        <v>329</v>
+        <v>39</v>
       </c>
       <c r="J266" s="5"/>
     </row>
     <row r="267" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A267" s="4">
-        <v>23041</v>
+        <v>23051</v>
       </c>
       <c r="B267" s="5" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
       <c r="C267" s="4">
-        <v>2304</v>
+        <v>2305</v>
       </c>
       <c r="D267" s="4">
-        <v>23041</v>
+        <v>23051</v>
       </c>
       <c r="E267" s="4"/>
       <c r="F267" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G267" s="5" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="H267" s="5"/>
       <c r="I267" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="J267" s="5"/>
+    </row>
+    <row r="268" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A268" s="4">
+        <v>2306</v>
+      </c>
+      <c r="B268" s="5" t="s">
         <v>330</v>
-      </c>
-      <c r="J267" s="5"/>
-    </row>
-    <row r="268" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A268" s="4">
-        <v>2305</v>
-      </c>
-      <c r="B268" s="5" t="s">
-        <v>39</v>
       </c>
       <c r="C268" s="4">
         <v>23</v>
       </c>
       <c r="D268" s="4">
-        <v>2305</v>
+        <v>2306</v>
       </c>
       <c r="E268" s="4"/>
       <c r="F268" s="4" t="s">
@@ -14644,63 +14627,65 @@
       <c r="G268" s="5"/>
       <c r="H268" s="5"/>
       <c r="I268" s="5" t="s">
-        <v>39</v>
+        <v>330</v>
       </c>
       <c r="J268" s="5"/>
     </row>
     <row r="269" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A269" s="4">
-        <v>23051</v>
+        <v>23061</v>
       </c>
       <c r="B269" s="5" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C269" s="4">
-        <v>2305</v>
+        <v>2306</v>
       </c>
       <c r="D269" s="4">
-        <v>23051</v>
+        <v>23061</v>
       </c>
       <c r="E269" s="4"/>
       <c r="F269" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G269" s="5" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="H269" s="5"/>
       <c r="I269" s="5" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="J269" s="5"/>
     </row>
     <row r="270" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A270" s="4">
+        <v>23062</v>
+      </c>
+      <c r="B270" s="5" t="s">
+        <v>333</v>
+      </c>
+      <c r="C270" s="4">
         <v>2306</v>
       </c>
-      <c r="B270" s="5" t="s">
-        <v>334</v>
-      </c>
-      <c r="C270" s="4">
-        <v>23</v>
-      </c>
       <c r="D270" s="4">
-        <v>2306</v>
+        <v>23062</v>
       </c>
       <c r="E270" s="4"/>
       <c r="F270" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G270" s="5"/>
+        <v>55</v>
+      </c>
+      <c r="G270" s="5" t="s">
+        <v>334</v>
+      </c>
       <c r="H270" s="5"/>
       <c r="I270" s="5" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="J270" s="5"/>
     </row>
     <row r="271" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A271" s="4">
-        <v>23061</v>
+        <v>23063</v>
       </c>
       <c r="B271" s="5" t="s">
         <v>335</v>
@@ -14709,7 +14694,7 @@
         <v>2306</v>
       </c>
       <c r="D271" s="4">
-        <v>23061</v>
+        <v>23063</v>
       </c>
       <c r="E271" s="4"/>
       <c r="F271" s="4" t="s">
@@ -14720,48 +14705,46 @@
       </c>
       <c r="H271" s="5"/>
       <c r="I271" s="5" t="s">
-        <v>335</v>
+        <v>337</v>
       </c>
       <c r="J271" s="5"/>
     </row>
     <row r="272" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A272" s="4">
-        <v>23062</v>
+        <v>2307</v>
       </c>
       <c r="B272" s="5" t="s">
-        <v>337</v>
+        <v>338</v>
       </c>
       <c r="C272" s="4">
-        <v>2306</v>
+        <v>23</v>
       </c>
       <c r="D272" s="4">
-        <v>23062</v>
+        <v>2307</v>
       </c>
       <c r="E272" s="4"/>
       <c r="F272" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G272" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="G272" s="4"/>
+      <c r="H272" s="4"/>
+      <c r="I272" s="5" t="s">
         <v>338</v>
       </c>
-      <c r="H272" s="5"/>
-      <c r="I272" s="5" t="s">
-        <v>337</v>
-      </c>
       <c r="J272" s="5"/>
     </row>
-    <row r="273" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="273" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A273" s="4">
-        <v>23063</v>
+        <v>23071</v>
       </c>
       <c r="B273" s="5" t="s">
         <v>339</v>
       </c>
       <c r="C273" s="4">
-        <v>2306</v>
+        <v>2307</v>
       </c>
       <c r="D273" s="4">
-        <v>23063</v>
+        <v>23071</v>
       </c>
       <c r="E273" s="4"/>
       <c r="F273" s="4" t="s">
@@ -14770,39 +14753,41 @@
       <c r="G273" s="5" t="s">
         <v>340</v>
       </c>
-      <c r="H273" s="5"/>
+      <c r="H273" s="4"/>
       <c r="I273" s="5" t="s">
-        <v>341</v>
+        <v>339</v>
       </c>
       <c r="J273" s="5"/>
     </row>
     <row r="274" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A274" s="4">
+        <v>23072</v>
+      </c>
+      <c r="B274" s="5" t="s">
+        <v>341</v>
+      </c>
+      <c r="C274" s="4">
         <v>2307</v>
       </c>
-      <c r="B274" s="5" t="s">
-        <v>342</v>
-      </c>
-      <c r="C274" s="4">
-        <v>23</v>
-      </c>
       <c r="D274" s="4">
-        <v>2307</v>
+        <v>23072</v>
       </c>
       <c r="E274" s="4"/>
       <c r="F274" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G274" s="4"/>
-      <c r="H274" s="4"/>
+        <v>55</v>
+      </c>
+      <c r="G274" s="5" t="s">
+        <v>342</v>
+      </c>
+      <c r="H274" s="5"/>
       <c r="I274" s="5" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="J274" s="5"/>
     </row>
     <row r="275" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A275" s="4">
-        <v>23071</v>
+        <v>23073</v>
       </c>
       <c r="B275" s="5" t="s">
         <v>343</v>
@@ -14811,7 +14796,7 @@
         <v>2307</v>
       </c>
       <c r="D275" s="4">
-        <v>23071</v>
+        <v>23073</v>
       </c>
       <c r="E275" s="4"/>
       <c r="F275" s="4" t="s">
@@ -14820,7 +14805,7 @@
       <c r="G275" s="5" t="s">
         <v>344</v>
       </c>
-      <c r="H275" s="4"/>
+      <c r="H275" s="5"/>
       <c r="I275" s="5" t="s">
         <v>343</v>
       </c>
@@ -14828,24 +14813,22 @@
     </row>
     <row r="276" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A276" s="4">
-        <v>23072</v>
+        <v>24</v>
       </c>
       <c r="B276" s="5" t="s">
         <v>345</v>
       </c>
       <c r="C276" s="4">
-        <v>2307</v>
+        <v>2</v>
       </c>
       <c r="D276" s="4">
-        <v>23072</v>
-      </c>
-      <c r="E276" s="4"/>
+        <v>24</v>
+      </c>
+      <c r="E276" s="5"/>
       <c r="F276" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G276" s="5" t="s">
-        <v>346</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G276" s="5"/>
       <c r="H276" s="5"/>
       <c r="I276" s="5" t="s">
         <v>345</v>
@@ -14854,49 +14837,51 @@
     </row>
     <row r="277" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A277" s="4">
-        <v>23073</v>
+        <v>2401</v>
       </c>
       <c r="B277" s="5" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="C277" s="4">
-        <v>2307</v>
+        <v>24</v>
       </c>
       <c r="D277" s="4">
-        <v>23073</v>
-      </c>
-      <c r="E277" s="4"/>
+        <v>2401</v>
+      </c>
+      <c r="E277" s="5"/>
       <c r="F277" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G277" s="5" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="H277" s="5"/>
       <c r="I277" s="5" t="s">
-        <v>347</v>
+        <v>348</v>
       </c>
       <c r="J277" s="5"/>
     </row>
     <row r="278" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A278" s="4">
-        <v>24</v>
+        <v>2402</v>
       </c>
       <c r="B278" s="5" t="s">
         <v>349</v>
       </c>
       <c r="C278" s="4">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="D278" s="4">
-        <v>24</v>
-      </c>
-      <c r="E278" s="5"/>
+        <v>2402</v>
+      </c>
+      <c r="E278" s="4"/>
       <c r="F278" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G278" s="5"/>
-      <c r="H278" s="5"/>
+        <v>55</v>
+      </c>
+      <c r="G278" s="5" t="s">
+        <v>350</v>
+      </c>
+      <c r="H278" s="4"/>
       <c r="I278" s="5" t="s">
         <v>349</v>
       </c>
@@ -14904,131 +14889,79 @@
     </row>
     <row r="279" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A279" s="4">
-        <v>2401</v>
+        <v>2403</v>
       </c>
       <c r="B279" s="5" t="s">
-        <v>350</v>
+        <v>351</v>
       </c>
       <c r="C279" s="4">
         <v>24</v>
       </c>
       <c r="D279" s="4">
-        <v>2401</v>
-      </c>
-      <c r="E279" s="5"/>
+        <v>2403</v>
+      </c>
+      <c r="E279" s="4"/>
       <c r="F279" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="G279" s="5" t="s">
+      <c r="G279" s="5"/>
+      <c r="H279" s="1"/>
+      <c r="I279" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="H279" s="5"/>
-      <c r="I279" s="5" t="s">
-        <v>352</v>
-      </c>
-      <c r="J279" s="5"/>
+      <c r="J279" s="1" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="280" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A280" s="4">
-        <v>2402</v>
+        <v>25</v>
       </c>
       <c r="B280" s="5" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C280" s="4">
-        <v>24</v>
+        <v>2</v>
       </c>
       <c r="D280" s="4">
-        <v>2402</v>
+        <v>25</v>
       </c>
       <c r="E280" s="4"/>
       <c r="F280" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G280" s="5" t="s">
-        <v>354</v>
-      </c>
-      <c r="H280" s="4"/>
+        <v>52</v>
+      </c>
+      <c r="G280" s="5"/>
+      <c r="H280" s="5"/>
       <c r="I280" s="5" t="s">
+        <v>352</v>
+      </c>
+      <c r="J280" s="5"/>
+    </row>
+    <row r="281" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A281" s="4">
+        <v>2501</v>
+      </c>
+      <c r="B281" s="5" t="s">
         <v>353</v>
       </c>
-      <c r="J280" s="5"/>
-    </row>
-    <row r="281" spans="1:10" s="13" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="A281" s="4">
-        <v>2403</v>
-      </c>
-      <c r="B281" s="5" t="s">
-        <v>355</v>
-      </c>
       <c r="C281" s="4">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D281" s="4">
-        <v>2403</v>
-      </c>
-      <c r="E281" s="4"/>
+        <v>2501</v>
+      </c>
+      <c r="E281" s="5"/>
       <c r="F281" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="G281" s="5"/>
-      <c r="H281" s="1"/>
-      <c r="I281" s="1" t="s">
-        <v>355</v>
-      </c>
-      <c r="J281" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="282" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A282" s="4">
-        <v>25</v>
-      </c>
-      <c r="B282" s="5" t="s">
-        <v>356</v>
-      </c>
-      <c r="C282" s="4">
-        <v>2</v>
-      </c>
-      <c r="D282" s="4">
-        <v>25</v>
-      </c>
-      <c r="E282" s="4"/>
-      <c r="F282" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G282" s="5"/>
-      <c r="H282" s="5"/>
-      <c r="I282" s="5" t="s">
-        <v>356</v>
-      </c>
-      <c r="J282" s="5"/>
-    </row>
-    <row r="283" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A283" s="4">
-        <v>2501</v>
-      </c>
-      <c r="B283" s="5" t="s">
-        <v>357</v>
-      </c>
-      <c r="C283" s="4">
-        <v>25</v>
-      </c>
-      <c r="D283" s="4">
-        <v>2501</v>
-      </c>
-      <c r="E283" s="5"/>
-      <c r="F283" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G283" s="5" t="s">
-        <v>358</v>
-      </c>
-      <c r="H283" s="5"/>
-      <c r="I283" s="5" t="s">
-        <v>357</v>
-      </c>
-      <c r="J283" s="5"/>
+      <c r="G281" s="5" t="s">
+        <v>354</v>
+      </c>
+      <c r="H281" s="5"/>
+      <c r="I281" s="5" t="s">
+        <v>353</v>
+      </c>
+      <c r="J281" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>

</xml_diff>

<commit_message>
#100 laser x pixel size to cib laser x pixel size
</commit_message>
<xml_diff>
--- a/Sources/Cuga-Calibration-Solution/Assets/Data/InitData.xlsx
+++ b/Sources/Cuga-Calibration-Solution/Assets/Data/InitData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\RiderProjects\semix\kaizhi.xuan\netcore_semix_cuga_calibration\Sources\Cuga-Calibration-Solution\Assets\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{801E4157-842C-4743-A8A1-487EB3E47910}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47DC0A97-8CEA-4A7F-8D2C-5ECB1ABA2BE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" firstSheet="1" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" firstSheet="1" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SysUser" sheetId="1" r:id="rId1"/>
@@ -898,9 +898,6 @@
     <t>X Pixel Size</t>
   </si>
   <si>
-    <t>CugaCalibration.ViewModels.Laser.LaserXPixelSizeCalibrationViewModel</t>
-  </si>
-  <si>
     <t>Line Centricity</t>
   </si>
   <si>
@@ -1206,6 +1203,10 @@
   </si>
   <si>
     <t>CugaCalibration.ViewModels.Chuck.ChuckAlignmentDegreeOffsetCalibrationViewModel</t>
+  </si>
+  <si>
+    <t>CugaCalibration.ViewModels.CIB.CIBXPixelSizeCalibrationViewModel</t>
+    <phoneticPr fontId="7" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -12894,7 +12895,7 @@
         <v>1309</v>
       </c>
       <c r="B202" s="1" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="C202" s="4">
         <v>13</v>
@@ -12907,11 +12908,11 @@
         <v>55</v>
       </c>
       <c r="G202" s="1" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="H202" s="1"/>
       <c r="I202" s="1" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="J202" s="5"/>
     </row>
@@ -13876,8 +13877,8 @@
       <c r="F238" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="G238" s="5" t="s">
-        <v>285</v>
+      <c r="G238" s="12" t="s">
+        <v>365</v>
       </c>
       <c r="H238" s="1"/>
       <c r="I238" s="1" t="s">
@@ -13890,7 +13891,7 @@
         <v>1603</v>
       </c>
       <c r="B239" s="5" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="C239" s="4">
         <v>16</v>
@@ -13903,11 +13904,11 @@
         <v>55</v>
       </c>
       <c r="G239" s="5" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="H239" s="5"/>
       <c r="I239" s="5" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="J239" s="5"/>
     </row>
@@ -13916,7 +13917,7 @@
         <v>1604</v>
       </c>
       <c r="B240" s="5" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C240" s="4">
         <v>16</v>
@@ -13929,11 +13930,11 @@
         <v>55</v>
       </c>
       <c r="G240" s="5" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="H240" s="5"/>
       <c r="I240" s="5" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="J240" s="5"/>
     </row>
@@ -13942,7 +13943,7 @@
         <v>1605</v>
       </c>
       <c r="B241" s="5" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="C241" s="4">
         <v>16</v>
@@ -13955,11 +13956,11 @@
         <v>55</v>
       </c>
       <c r="G241" s="5" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="H241" s="5"/>
       <c r="I241" s="5" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="J241" s="5"/>
     </row>
@@ -13968,7 +13969,7 @@
         <v>1606</v>
       </c>
       <c r="B242" s="5" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="C242" s="4">
         <v>16</v>
@@ -13981,11 +13982,11 @@
         <v>55</v>
       </c>
       <c r="G242" s="5" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="H242" s="5"/>
       <c r="I242" s="5" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="J242" s="5"/>
     </row>
@@ -13994,7 +13995,7 @@
         <v>1607</v>
       </c>
       <c r="B243" s="12" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="C243" s="4">
         <v>16</v>
@@ -14007,11 +14008,11 @@
         <v>55</v>
       </c>
       <c r="G243" s="12" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="H243" s="5"/>
       <c r="I243" s="12" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="J243" s="5"/>
     </row>
@@ -14020,7 +14021,7 @@
         <v>17</v>
       </c>
       <c r="B244" s="12" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C244" s="4">
         <v>1</v>
@@ -14035,7 +14036,7 @@
       <c r="G244" s="5"/>
       <c r="H244" s="5"/>
       <c r="I244" s="12" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="J244" s="5"/>
     </row>
@@ -14044,7 +14045,7 @@
         <v>1701</v>
       </c>
       <c r="B245" s="12" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="C245" s="4">
         <v>17</v>
@@ -14057,11 +14058,11 @@
         <v>55</v>
       </c>
       <c r="G245" s="12" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="H245" s="5"/>
       <c r="I245" s="12" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="J245" s="5"/>
     </row>
@@ -14070,7 +14071,7 @@
         <v>2</v>
       </c>
       <c r="B246" s="5" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C246" s="4">
         <v>-1</v>
@@ -14085,7 +14086,7 @@
       <c r="G246" s="5"/>
       <c r="H246" s="5"/>
       <c r="I246" s="5" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="J246" s="5"/>
     </row>
@@ -14094,7 +14095,7 @@
         <v>21</v>
       </c>
       <c r="B247" s="5" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="C247" s="4">
         <v>2</v>
@@ -14109,7 +14110,7 @@
       <c r="G247" s="5"/>
       <c r="H247" s="5"/>
       <c r="I247" s="5" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="J247" s="5"/>
     </row>
@@ -14118,7 +14119,7 @@
         <v>2110</v>
       </c>
       <c r="B248" s="5" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C248" s="4">
         <v>21</v>
@@ -14131,11 +14132,11 @@
         <v>55</v>
       </c>
       <c r="G248" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H248" s="5"/>
       <c r="I248" s="5" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="J248" s="5"/>
     </row>
@@ -14144,7 +14145,7 @@
         <v>2111</v>
       </c>
       <c r="B249" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C249" s="4">
         <v>21</v>
@@ -14157,11 +14158,11 @@
         <v>55</v>
       </c>
       <c r="G249" s="5" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H249" s="5"/>
       <c r="I249" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J249" s="5"/>
     </row>
@@ -14170,7 +14171,7 @@
         <v>22</v>
       </c>
       <c r="B250" s="5" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C250" s="4">
         <v>2</v>
@@ -14185,7 +14186,7 @@
       <c r="G250" s="5"/>
       <c r="H250" s="5"/>
       <c r="I250" s="5" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="J250" s="5"/>
     </row>
@@ -14194,7 +14195,7 @@
         <v>2201</v>
       </c>
       <c r="B251" s="5" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="C251" s="4">
         <v>22</v>
@@ -14207,11 +14208,11 @@
         <v>55</v>
       </c>
       <c r="G251" s="5" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="H251" s="5"/>
       <c r="I251" s="5" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="J251" s="5"/>
     </row>
@@ -14220,7 +14221,7 @@
         <v>2202</v>
       </c>
       <c r="B252" s="5" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C252" s="4">
         <v>22</v>
@@ -14233,11 +14234,11 @@
         <v>55</v>
       </c>
       <c r="G252" s="5" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="H252" s="5"/>
       <c r="I252" s="5" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="J252" s="5"/>
     </row>
@@ -14246,7 +14247,7 @@
         <v>2203</v>
       </c>
       <c r="B253" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C253" s="4">
         <v>22</v>
@@ -14259,11 +14260,11 @@
         <v>55</v>
       </c>
       <c r="G253" s="5" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H253" s="5"/>
       <c r="I253" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="J253" s="5"/>
     </row>
@@ -14272,7 +14273,7 @@
         <v>23</v>
       </c>
       <c r="B254" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C254" s="4">
         <v>2</v>
@@ -14287,7 +14288,7 @@
       <c r="G254" s="5"/>
       <c r="H254" s="5"/>
       <c r="I254" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J254" s="5"/>
     </row>
@@ -14296,7 +14297,7 @@
         <v>2301</v>
       </c>
       <c r="B255" s="5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C255" s="4">
         <v>23</v>
@@ -14309,11 +14310,11 @@
         <v>55</v>
       </c>
       <c r="G255" s="5" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="H255" s="5"/>
       <c r="I255" s="5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="J255" s="5"/>
     </row>
@@ -14322,7 +14323,7 @@
         <v>2302</v>
       </c>
       <c r="B256" s="5" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C256" s="4">
         <v>23</v>
@@ -14337,7 +14338,7 @@
       <c r="G256" s="5"/>
       <c r="H256" s="5"/>
       <c r="I256" s="5" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="J256" s="5"/>
     </row>
@@ -14346,7 +14347,7 @@
         <v>23021</v>
       </c>
       <c r="B257" s="5" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="C257" s="4">
         <v>2302</v>
@@ -14359,11 +14360,11 @@
         <v>55</v>
       </c>
       <c r="G257" s="5" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="H257" s="5"/>
       <c r="I257" s="5" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="J257" s="5"/>
     </row>
@@ -14372,7 +14373,7 @@
         <v>23022</v>
       </c>
       <c r="B258" s="5" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="C258" s="4">
         <v>2302</v>
@@ -14385,11 +14386,11 @@
         <v>55</v>
       </c>
       <c r="G258" s="5" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="H258" s="5"/>
       <c r="I258" s="5" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="J258" s="5"/>
     </row>
@@ -14422,7 +14423,7 @@
         <v>23031</v>
       </c>
       <c r="B260" s="5" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="C260" s="4">
         <v>2303</v>
@@ -14435,11 +14436,11 @@
         <v>55</v>
       </c>
       <c r="G260" s="5" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="H260" s="5"/>
       <c r="I260" s="5" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="J260" s="5"/>
     </row>
@@ -14448,7 +14449,7 @@
         <v>23032</v>
       </c>
       <c r="B261" s="5" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C261" s="4">
         <v>2303</v>
@@ -14461,11 +14462,11 @@
         <v>55</v>
       </c>
       <c r="G261" s="5" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="H261" s="5"/>
       <c r="I261" s="5" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="J261" s="5"/>
     </row>
@@ -14474,7 +14475,7 @@
         <v>23033</v>
       </c>
       <c r="B262" s="5" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="C262" s="4">
         <v>2303</v>
@@ -14487,11 +14488,11 @@
         <v>55</v>
       </c>
       <c r="G262" s="5" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="H262" s="5"/>
       <c r="I262" s="5" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="J262" s="5"/>
     </row>
@@ -14500,7 +14501,7 @@
         <v>23034</v>
       </c>
       <c r="B263" s="12" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="C263" s="4">
         <v>2303</v>
@@ -14513,11 +14514,11 @@
         <v>55</v>
       </c>
       <c r="G263" s="12" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="H263" s="5"/>
       <c r="I263" s="12" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="J263" s="5"/>
     </row>
@@ -14526,7 +14527,7 @@
         <v>23035</v>
       </c>
       <c r="B264" s="5" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C264" s="4">
         <v>2303</v>
@@ -14539,11 +14540,11 @@
         <v>55</v>
       </c>
       <c r="G264" s="5" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="H264" s="5"/>
       <c r="I264" s="5" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="J264" s="5"/>
     </row>
@@ -14552,7 +14553,7 @@
         <v>23036</v>
       </c>
       <c r="B265" s="12" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="C265" s="4">
         <v>2303</v>
@@ -14565,11 +14566,11 @@
         <v>55</v>
       </c>
       <c r="G265" s="12" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="H265" s="5"/>
       <c r="I265" s="12" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="J265" s="5"/>
     </row>
@@ -14578,7 +14579,7 @@
         <v>2304</v>
       </c>
       <c r="B266" s="5" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="C266" s="4">
         <v>23</v>
@@ -14593,7 +14594,7 @@
       <c r="G266" s="5"/>
       <c r="H266" s="5"/>
       <c r="I266" s="5" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="J266" s="5"/>
     </row>
@@ -14602,7 +14603,7 @@
         <v>23041</v>
       </c>
       <c r="B267" s="5" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C267" s="4">
         <v>2304</v>
@@ -14615,11 +14616,11 @@
         <v>55</v>
       </c>
       <c r="G267" s="5" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="H267" s="5"/>
       <c r="I267" s="5" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="J267" s="5"/>
     </row>
@@ -14652,7 +14653,7 @@
         <v>23051</v>
       </c>
       <c r="B269" s="5" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C269" s="4">
         <v>2305</v>
@@ -14665,11 +14666,11 @@
         <v>55</v>
       </c>
       <c r="G269" s="5" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="H269" s="5"/>
       <c r="I269" s="5" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="J269" s="5"/>
     </row>
@@ -14678,7 +14679,7 @@
         <v>2306</v>
       </c>
       <c r="B270" s="5" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C270" s="4">
         <v>23</v>
@@ -14693,7 +14694,7 @@
       <c r="G270" s="5"/>
       <c r="H270" s="5"/>
       <c r="I270" s="5" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J270" s="5"/>
     </row>
@@ -14702,7 +14703,7 @@
         <v>23061</v>
       </c>
       <c r="B271" s="5" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C271" s="4">
         <v>2306</v>
@@ -14715,11 +14716,11 @@
         <v>55</v>
       </c>
       <c r="G271" s="5" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="H271" s="5"/>
       <c r="I271" s="5" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="J271" s="5"/>
     </row>
@@ -14728,7 +14729,7 @@
         <v>23062</v>
       </c>
       <c r="B272" s="5" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C272" s="4">
         <v>2306</v>
@@ -14741,11 +14742,11 @@
         <v>55</v>
       </c>
       <c r="G272" s="5" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="H272" s="5"/>
       <c r="I272" s="5" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="J272" s="5"/>
     </row>
@@ -14754,7 +14755,7 @@
         <v>23063</v>
       </c>
       <c r="B273" s="5" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C273" s="4">
         <v>2306</v>
@@ -14767,11 +14768,11 @@
         <v>55</v>
       </c>
       <c r="G273" s="5" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="H273" s="5"/>
       <c r="I273" s="5" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="J273" s="5"/>
     </row>
@@ -14780,7 +14781,7 @@
         <v>2307</v>
       </c>
       <c r="B274" s="5" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="C274" s="4">
         <v>23</v>
@@ -14795,7 +14796,7 @@
       <c r="G274" s="4"/>
       <c r="H274" s="4"/>
       <c r="I274" s="5" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="J274" s="5"/>
     </row>
@@ -14804,7 +14805,7 @@
         <v>23071</v>
       </c>
       <c r="B275" s="5" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="C275" s="4">
         <v>2307</v>
@@ -14817,11 +14818,11 @@
         <v>55</v>
       </c>
       <c r="G275" s="5" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="H275" s="4"/>
       <c r="I275" s="5" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="J275" s="5"/>
     </row>
@@ -14830,7 +14831,7 @@
         <v>23072</v>
       </c>
       <c r="B276" s="5" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C276" s="4">
         <v>2307</v>
@@ -14843,11 +14844,11 @@
         <v>55</v>
       </c>
       <c r="G276" s="5" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="H276" s="5"/>
       <c r="I276" s="5" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="J276" s="5"/>
     </row>
@@ -14856,7 +14857,7 @@
         <v>23073</v>
       </c>
       <c r="B277" s="5" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C277" s="4">
         <v>2307</v>
@@ -14869,11 +14870,11 @@
         <v>55</v>
       </c>
       <c r="G277" s="5" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="H277" s="5"/>
       <c r="I277" s="5" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="J277" s="5"/>
     </row>
@@ -14882,7 +14883,7 @@
         <v>24</v>
       </c>
       <c r="B278" s="5" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="C278" s="4">
         <v>2</v>
@@ -14897,7 +14898,7 @@
       <c r="G278" s="5"/>
       <c r="H278" s="5"/>
       <c r="I278" s="5" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="J278" s="5"/>
     </row>
@@ -14906,7 +14907,7 @@
         <v>2401</v>
       </c>
       <c r="B279" s="5" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C279" s="4">
         <v>24</v>
@@ -14919,11 +14920,11 @@
         <v>55</v>
       </c>
       <c r="G279" s="5" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="H279" s="5"/>
       <c r="I279" s="5" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="J279" s="5"/>
     </row>
@@ -14932,7 +14933,7 @@
         <v>2402</v>
       </c>
       <c r="B280" s="5" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C280" s="4">
         <v>24</v>
@@ -14945,11 +14946,11 @@
         <v>55</v>
       </c>
       <c r="G280" s="5" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="H280" s="4"/>
       <c r="I280" s="5" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="J280" s="5"/>
     </row>
@@ -14958,7 +14959,7 @@
         <v>2403</v>
       </c>
       <c r="B281" s="5" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="C281" s="4">
         <v>24</v>
@@ -14973,7 +14974,7 @@
       <c r="G281" s="5"/>
       <c r="H281" s="1"/>
       <c r="I281" s="1" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="J281" s="1" t="b">
         <v>1</v>
@@ -14984,7 +14985,7 @@
         <v>25</v>
       </c>
       <c r="B282" s="5" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="C282" s="4">
         <v>2</v>
@@ -14999,7 +15000,7 @@
       <c r="G282" s="5"/>
       <c r="H282" s="5"/>
       <c r="I282" s="5" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="J282" s="5"/>
     </row>
@@ -15008,7 +15009,7 @@
         <v>2501</v>
       </c>
       <c r="B283" s="5" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="C283" s="4">
         <v>25</v>
@@ -15021,11 +15022,11 @@
         <v>55</v>
       </c>
       <c r="G283" s="5" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="H283" s="5"/>
       <c r="I283" s="5" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="J283" s="5"/>
     </row>

</xml_diff>

<commit_message>
#100 x pixel 重命名ok
</commit_message>
<xml_diff>
--- a/Sources/Cuga-Calibration-Solution/Assets/Data/InitData.xlsx
+++ b/Sources/Cuga-Calibration-Solution/Assets/Data/InitData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\RiderProjects\semix\kaizhi.xuan\netcore_semix_cuga_calibration\Sources\Cuga-Calibration-Solution\Assets\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47DC0A97-8CEA-4A7F-8D2C-5ECB1ABA2BE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C474E423-4B65-4F83-B055-FB5CC312D952}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" firstSheet="1" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1205,7 +1205,7 @@
     <t>CugaCalibration.ViewModels.Chuck.ChuckAlignmentDegreeOffsetCalibrationViewModel</t>
   </si>
   <si>
-    <t>CugaCalibration.ViewModels.CIB.CIBXPixelSizeCalibrationViewModel</t>
+    <t>CugaCalibration.ViewModels.CIB.CIBXPixelSizeViewModel</t>
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
 </sst>

</xml_diff>

<commit_message>
#100 OI NI AOD Alignment Delay Laser Optics Power Meter Laser Attenutar #104 CIB Illumination Profile #105 Optics INC
</commit_message>
<xml_diff>
--- a/Sources/Cuga-Calibration-Solution/Assets/Data/InitData.xlsx
+++ b/Sources/Cuga-Calibration-Solution/Assets/Data/InitData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\RiderProjects\semix\kaizhi.xuan\netcore_semix_cuga_calibration\Sources\Cuga-Calibration-Solution\Assets\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{801E4157-842C-4743-A8A1-487EB3E47910}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5917CABC-84A8-4B3C-B248-59857E0BBBB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" firstSheet="1" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" firstSheet="1" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SysUser" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1402" uniqueCount="366">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1305" uniqueCount="351">
   <si>
     <t>Id</t>
   </si>
@@ -778,69 +778,12 @@
     <t>CugaCalibration.ViewModels.Laser.LaserAutoFocusCalibrationViewModel</t>
   </si>
   <si>
-    <t>Auto Focus-Step0</t>
-  </si>
-  <si>
-    <t>CugaCalibration.Views.Laser.AutoFocus.Children.Step0View</t>
-  </si>
-  <si>
-    <t>Auto Focus-StepCommonNext</t>
-  </si>
-  <si>
-    <t>CugaCalibration.Views.Laser.AutoFocus.Children.StepCommonNextView</t>
-  </si>
-  <si>
-    <t>FminNumeric</t>
-  </si>
-  <si>
-    <t>FmaxNumeric</t>
-  </si>
-  <si>
-    <t>NminNumeric</t>
-  </si>
-  <si>
-    <t>NmaxNumeric</t>
-  </si>
-  <si>
-    <t>CurrentMinNumeric</t>
-  </si>
-  <si>
-    <t>CurrentMaxNumeric</t>
-  </si>
-  <si>
-    <t>CurrentIntervalNumeric</t>
-  </si>
-  <si>
-    <t>Auto Focus-Review</t>
-  </si>
-  <si>
-    <t>CugaCalibration.Views.Laser.AutoFocus.Children.Review</t>
-  </si>
-  <si>
     <t>Beam Stabilizer</t>
   </si>
   <si>
     <t>CugaCalibration.ViewModels.Laser.LaserBeamStabilizerCalibrationViewModel</t>
   </si>
   <si>
-    <t>Beam Stabilizer-Step0</t>
-  </si>
-  <si>
-    <t>CugaCalibration.Views.Laser.BeamStabilizer.Children.Step0View</t>
-  </si>
-  <si>
-    <t>Beam Stabilizer-Step1</t>
-  </si>
-  <si>
-    <t>CugaCalibration.Views.Laser.BeamStabilizer.Children.Step1View</t>
-  </si>
-  <si>
-    <t>Beam Stabilizer-Review</t>
-  </si>
-  <si>
-    <t>CugaCalibration.Views.Laser.BeamStabilizer.Children.Review</t>
-  </si>
-  <si>
     <t>Optical Power Meter</t>
   </si>
   <si>
@@ -898,9 +841,6 @@
     <t>X Pixel Size</t>
   </si>
   <si>
-    <t>CugaCalibration.ViewModels.Laser.LaserXPixelSizeCalibrationViewModel</t>
-  </si>
-  <si>
     <t>Line Centricity</t>
   </si>
   <si>
@@ -920,9 +860,6 @@
   </si>
   <si>
     <t>MMD</t>
-  </si>
-  <si>
-    <t>CugaCalibration.ViewModels.CIB.CIBMMDViewModel</t>
   </si>
   <si>
     <t>Title</t>
@@ -1206,6 +1143,30 @@
   </si>
   <si>
     <t>CugaCalibration.ViewModels.Chuck.ChuckAlignmentDegreeOffsetCalibrationViewModel</t>
+  </si>
+  <si>
+    <t>CugaCalibration.ViewModels.CIB.CIBXPixelSizeViewModel</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>INC</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>CugaCalibration.ViewModels.Optics.OpticsINCViewModel</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Illumination Profile</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>CugaCalibration.ViewModels.CIB.CIBMMDViewModel</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>CugaCalibration.ViewModels.CIB.CIBIlluminationProfileViewModel</t>
+    <phoneticPr fontId="7" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -7282,7 +7243,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:J283"/>
+  <dimension ref="A1:J264"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.625" style="2" customWidth="1"/>
@@ -7295,7 +7256,7 @@
     <col min="10" max="10" width="17.875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" ht="23.25" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -7327,7 +7288,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -7351,7 +7312,7 @@
       </c>
       <c r="J2" s="5"/>
     </row>
-    <row r="3" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="4">
         <v>11</v>
       </c>
@@ -7375,7 +7336,7 @@
       </c>
       <c r="J3" s="5"/>
     </row>
-    <row r="4" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="4">
         <v>1101</v>
       </c>
@@ -7401,7 +7362,7 @@
       </c>
       <c r="J4" s="5"/>
     </row>
-    <row r="5" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="4">
         <v>110101</v>
       </c>
@@ -7429,7 +7390,7 @@
       </c>
       <c r="J5" s="5"/>
     </row>
-    <row r="6" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="4">
         <v>110102</v>
       </c>
@@ -7457,7 +7418,7 @@
       </c>
       <c r="J6" s="5"/>
     </row>
-    <row r="7" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="4">
         <v>110103</v>
       </c>
@@ -7485,7 +7446,7 @@
       </c>
       <c r="J7" s="5"/>
     </row>
-    <row r="8" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="4">
         <v>110104</v>
       </c>
@@ -7513,7 +7474,7 @@
       </c>
       <c r="J8" s="5"/>
     </row>
-    <row r="9" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="4">
         <v>110105</v>
       </c>
@@ -7541,7 +7502,7 @@
       </c>
       <c r="J9" s="5"/>
     </row>
-    <row r="10" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="4">
         <v>110106</v>
       </c>
@@ -7569,7 +7530,7 @@
       </c>
       <c r="J10" s="5"/>
     </row>
-    <row r="11" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="4">
         <v>110107</v>
       </c>
@@ -7597,7 +7558,7 @@
       </c>
       <c r="J11" s="5"/>
     </row>
-    <row r="12" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="4">
         <v>1102</v>
       </c>
@@ -7623,7 +7584,7 @@
       </c>
       <c r="J12" s="5"/>
     </row>
-    <row r="13" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="4">
         <v>110201</v>
       </c>
@@ -7651,7 +7612,7 @@
       </c>
       <c r="J13" s="5"/>
     </row>
-    <row r="14" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="4">
         <v>110202</v>
       </c>
@@ -7679,7 +7640,7 @@
       </c>
       <c r="J14" s="5"/>
     </row>
-    <row r="15" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="4">
         <v>110203</v>
       </c>
@@ -7707,7 +7668,7 @@
       </c>
       <c r="J15" s="5"/>
     </row>
-    <row r="16" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="4">
         <v>110204</v>
       </c>
@@ -7735,7 +7696,7 @@
       </c>
       <c r="J16" s="5"/>
     </row>
-    <row r="17" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="4">
         <v>110205</v>
       </c>
@@ -7763,7 +7724,7 @@
       </c>
       <c r="J17" s="5"/>
     </row>
-    <row r="18" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="4">
         <v>110206</v>
       </c>
@@ -7791,7 +7752,7 @@
       </c>
       <c r="J18" s="5"/>
     </row>
-    <row r="19" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="4">
         <v>110207</v>
       </c>
@@ -7819,7 +7780,7 @@
       </c>
       <c r="J19" s="5"/>
     </row>
-    <row r="20" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="4">
         <v>110208</v>
       </c>
@@ -7847,7 +7808,7 @@
       </c>
       <c r="J20" s="5"/>
     </row>
-    <row r="21" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="4">
         <v>110209</v>
       </c>
@@ -7875,7 +7836,7 @@
       </c>
       <c r="J21" s="5"/>
     </row>
-    <row r="22" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="4">
         <v>110210</v>
       </c>
@@ -7903,7 +7864,7 @@
       </c>
       <c r="J22" s="5"/>
     </row>
-    <row r="23" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="4">
         <v>110211</v>
       </c>
@@ -7931,7 +7892,7 @@
       </c>
       <c r="J23" s="5"/>
     </row>
-    <row r="24" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="4">
         <v>110212</v>
       </c>
@@ -7959,7 +7920,7 @@
       </c>
       <c r="J24" s="5"/>
     </row>
-    <row r="25" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="4">
         <v>110213</v>
       </c>
@@ -7987,7 +7948,7 @@
       </c>
       <c r="J25" s="5"/>
     </row>
-    <row r="26" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="4">
         <v>110214</v>
       </c>
@@ -8015,7 +7976,7 @@
       </c>
       <c r="J26" s="5"/>
     </row>
-    <row r="27" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="4">
         <v>110215</v>
       </c>
@@ -8043,7 +8004,7 @@
       </c>
       <c r="J27" s="5"/>
     </row>
-    <row r="28" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="4">
         <v>110216</v>
       </c>
@@ -8071,7 +8032,7 @@
       </c>
       <c r="J28" s="5"/>
     </row>
-    <row r="29" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="4">
         <v>110217</v>
       </c>
@@ -8099,7 +8060,7 @@
       </c>
       <c r="J29" s="5"/>
     </row>
-    <row r="30" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="4">
         <v>110218</v>
       </c>
@@ -8127,7 +8088,7 @@
       </c>
       <c r="J30" s="5"/>
     </row>
-    <row r="31" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="4">
         <v>110219</v>
       </c>
@@ -8155,7 +8116,7 @@
       </c>
       <c r="J31" s="5"/>
     </row>
-    <row r="32" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="4">
         <v>110220</v>
       </c>
@@ -8183,7 +8144,7 @@
       </c>
       <c r="J32" s="5"/>
     </row>
-    <row r="33" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="4">
         <v>110221</v>
       </c>
@@ -8211,7 +8172,7 @@
       </c>
       <c r="J33" s="5"/>
     </row>
-    <row r="34" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="4">
         <v>110222</v>
       </c>
@@ -8239,7 +8200,7 @@
       </c>
       <c r="J34" s="5"/>
     </row>
-    <row r="35" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="4">
         <v>1103</v>
       </c>
@@ -8265,7 +8226,7 @@
       </c>
       <c r="J35" s="5"/>
     </row>
-    <row r="36" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="4">
         <v>110301</v>
       </c>
@@ -8293,7 +8254,7 @@
       </c>
       <c r="J36" s="5"/>
     </row>
-    <row r="37" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="4">
         <v>110302</v>
       </c>
@@ -8321,7 +8282,7 @@
       </c>
       <c r="J37" s="5"/>
     </row>
-    <row r="38" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="4">
         <v>110303</v>
       </c>
@@ -8349,7 +8310,7 @@
       </c>
       <c r="J38" s="5"/>
     </row>
-    <row r="39" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="4">
         <v>110304</v>
       </c>
@@ -8377,7 +8338,7 @@
       </c>
       <c r="J39" s="5"/>
     </row>
-    <row r="40" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="4">
         <v>110305</v>
       </c>
@@ -8405,7 +8366,7 @@
       </c>
       <c r="J40" s="5"/>
     </row>
-    <row r="41" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="4">
         <v>110306</v>
       </c>
@@ -8433,7 +8394,7 @@
       </c>
       <c r="J41" s="5"/>
     </row>
-    <row r="42" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="4">
         <v>110307</v>
       </c>
@@ -8461,7 +8422,7 @@
       </c>
       <c r="J42" s="5"/>
     </row>
-    <row r="43" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="4">
         <v>110308</v>
       </c>
@@ -8489,7 +8450,7 @@
       </c>
       <c r="J43" s="5"/>
     </row>
-    <row r="44" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="4">
         <v>110309</v>
       </c>
@@ -8517,7 +8478,7 @@
       </c>
       <c r="J44" s="5"/>
     </row>
-    <row r="45" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="4">
         <v>110310</v>
       </c>
@@ -8545,7 +8506,7 @@
       </c>
       <c r="J45" s="5"/>
     </row>
-    <row r="46" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="4">
         <v>110311</v>
       </c>
@@ -8573,7 +8534,7 @@
       </c>
       <c r="J46" s="5"/>
     </row>
-    <row r="47" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="4">
         <v>110312</v>
       </c>
@@ -8601,7 +8562,7 @@
       </c>
       <c r="J47" s="5"/>
     </row>
-    <row r="48" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="4">
         <v>110313</v>
       </c>
@@ -8629,7 +8590,7 @@
       </c>
       <c r="J48" s="5"/>
     </row>
-    <row r="49" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="4">
         <v>110314</v>
       </c>
@@ -8657,7 +8618,7 @@
       </c>
       <c r="J49" s="5"/>
     </row>
-    <row r="50" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="4">
         <v>110315</v>
       </c>
@@ -8685,7 +8646,7 @@
       </c>
       <c r="J50" s="5"/>
     </row>
-    <row r="51" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="4">
         <v>110316</v>
       </c>
@@ -8713,7 +8674,7 @@
       </c>
       <c r="J51" s="5"/>
     </row>
-    <row r="52" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="4">
         <v>110317</v>
       </c>
@@ -8741,7 +8702,7 @@
       </c>
       <c r="J52" s="5"/>
     </row>
-    <row r="53" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="4">
         <v>110318</v>
       </c>
@@ -8769,7 +8730,7 @@
       </c>
       <c r="J53" s="5"/>
     </row>
-    <row r="54" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="4">
         <v>110319</v>
       </c>
@@ -8797,7 +8758,7 @@
       </c>
       <c r="J54" s="5"/>
     </row>
-    <row r="55" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="4">
         <v>110320</v>
       </c>
@@ -8825,7 +8786,7 @@
       </c>
       <c r="J55" s="5"/>
     </row>
-    <row r="56" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="4">
         <v>110321</v>
       </c>
@@ -8853,7 +8814,7 @@
       </c>
       <c r="J56" s="5"/>
     </row>
-    <row r="57" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="4">
         <v>110322</v>
       </c>
@@ -8881,7 +8842,7 @@
       </c>
       <c r="J57" s="5"/>
     </row>
-    <row r="58" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="4">
         <v>110323</v>
       </c>
@@ -8909,7 +8870,7 @@
       </c>
       <c r="J58" s="5"/>
     </row>
-    <row r="59" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="4">
         <v>110324</v>
       </c>
@@ -8937,7 +8898,7 @@
       </c>
       <c r="J59" s="5"/>
     </row>
-    <row r="60" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="4">
         <v>12</v>
       </c>
@@ -8961,7 +8922,7 @@
       </c>
       <c r="J60" s="5"/>
     </row>
-    <row r="61" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="4">
         <v>1201</v>
       </c>
@@ -8987,7 +8948,7 @@
       </c>
       <c r="J61" s="5"/>
     </row>
-    <row r="62" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="4">
         <v>120101</v>
       </c>
@@ -9015,7 +8976,7 @@
       </c>
       <c r="J62" s="5"/>
     </row>
-    <row r="63" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="4">
         <v>120102</v>
       </c>
@@ -9043,7 +9004,7 @@
       </c>
       <c r="J63" s="5"/>
     </row>
-    <row r="64" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="4">
         <v>120103</v>
       </c>
@@ -9071,7 +9032,7 @@
       </c>
       <c r="J64" s="5"/>
     </row>
-    <row r="65" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="4">
         <v>120104</v>
       </c>
@@ -9099,7 +9060,7 @@
       </c>
       <c r="J65" s="5"/>
     </row>
-    <row r="66" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="4">
         <v>120105</v>
       </c>
@@ -9127,7 +9088,7 @@
       </c>
       <c r="J66" s="5"/>
     </row>
-    <row r="67" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="4">
         <v>120106</v>
       </c>
@@ -9155,7 +9116,7 @@
       </c>
       <c r="J67" s="5"/>
     </row>
-    <row r="68" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="4">
         <v>120107</v>
       </c>
@@ -9183,7 +9144,7 @@
       </c>
       <c r="J68" s="5"/>
     </row>
-    <row r="69" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="4">
         <v>120108</v>
       </c>
@@ -9211,7 +9172,7 @@
       </c>
       <c r="J69" s="5"/>
     </row>
-    <row r="70" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="4">
         <v>120109</v>
       </c>
@@ -9239,7 +9200,7 @@
       </c>
       <c r="J70" s="5"/>
     </row>
-    <row r="71" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="4">
         <v>120110</v>
       </c>
@@ -9267,7 +9228,7 @@
       </c>
       <c r="J71" s="5"/>
     </row>
-    <row r="72" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="4">
         <v>120111</v>
       </c>
@@ -9295,7 +9256,7 @@
       </c>
       <c r="J72" s="5"/>
     </row>
-    <row r="73" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="4">
         <v>120112</v>
       </c>
@@ -9323,7 +9284,7 @@
       </c>
       <c r="J73" s="5"/>
     </row>
-    <row r="74" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="4">
         <v>120113</v>
       </c>
@@ -9351,7 +9312,7 @@
       </c>
       <c r="J74" s="5"/>
     </row>
-    <row r="75" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="4">
         <v>120114</v>
       </c>
@@ -9379,7 +9340,7 @@
       </c>
       <c r="J75" s="5"/>
     </row>
-    <row r="76" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="4">
         <v>120115</v>
       </c>
@@ -9407,7 +9368,7 @@
       </c>
       <c r="J76" s="5"/>
     </row>
-    <row r="77" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="4">
         <v>1202</v>
       </c>
@@ -9433,7 +9394,7 @@
       </c>
       <c r="J77" s="5"/>
     </row>
-    <row r="78" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="4">
         <v>120201</v>
       </c>
@@ -9461,7 +9422,7 @@
       </c>
       <c r="J78" s="5"/>
     </row>
-    <row r="79" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="4">
         <v>120202</v>
       </c>
@@ -9489,7 +9450,7 @@
       </c>
       <c r="J79" s="5"/>
     </row>
-    <row r="80" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="4">
         <v>120203</v>
       </c>
@@ -9517,7 +9478,7 @@
       </c>
       <c r="J80" s="5"/>
     </row>
-    <row r="81" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="4">
         <v>120204</v>
       </c>
@@ -9545,7 +9506,7 @@
       </c>
       <c r="J81" s="5"/>
     </row>
-    <row r="82" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="4">
         <v>120205</v>
       </c>
@@ -9573,7 +9534,7 @@
       </c>
       <c r="J82" s="5"/>
     </row>
-    <row r="83" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="4">
         <v>120206</v>
       </c>
@@ -9601,7 +9562,7 @@
       </c>
       <c r="J83" s="5"/>
     </row>
-    <row r="84" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="4">
         <v>120207</v>
       </c>
@@ -9629,7 +9590,7 @@
       </c>
       <c r="J84" s="5"/>
     </row>
-    <row r="85" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="4">
         <v>120208</v>
       </c>
@@ -9657,7 +9618,7 @@
       </c>
       <c r="J85" s="5"/>
     </row>
-    <row r="86" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="4">
         <v>120209</v>
       </c>
@@ -9685,7 +9646,7 @@
       </c>
       <c r="J86" s="5"/>
     </row>
-    <row r="87" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="4">
         <v>120210</v>
       </c>
@@ -9713,7 +9674,7 @@
       </c>
       <c r="J87" s="5"/>
     </row>
-    <row r="88" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="4">
         <v>120211</v>
       </c>
@@ -9741,7 +9702,7 @@
       </c>
       <c r="J88" s="5"/>
     </row>
-    <row r="89" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="4">
         <v>120212</v>
       </c>
@@ -9769,7 +9730,7 @@
       </c>
       <c r="J89" s="5"/>
     </row>
-    <row r="90" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="4">
         <v>120213</v>
       </c>
@@ -9797,7 +9758,7 @@
       </c>
       <c r="J90" s="5"/>
     </row>
-    <row r="91" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="4">
         <v>120214</v>
       </c>
@@ -9825,7 +9786,7 @@
       </c>
       <c r="J91" s="5"/>
     </row>
-    <row r="92" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A92" s="4">
         <v>120215</v>
       </c>
@@ -9853,7 +9814,7 @@
       </c>
       <c r="J92" s="5"/>
     </row>
-    <row r="93" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A93" s="4">
         <v>120216</v>
       </c>
@@ -9881,7 +9842,7 @@
       </c>
       <c r="J93" s="5"/>
     </row>
-    <row r="94" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A94" s="4">
         <v>120217</v>
       </c>
@@ -9909,7 +9870,7 @@
       </c>
       <c r="J94" s="5"/>
     </row>
-    <row r="95" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A95" s="4">
         <v>120218</v>
       </c>
@@ -9937,7 +9898,7 @@
       </c>
       <c r="J95" s="5"/>
     </row>
-    <row r="96" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A96" s="4">
         <v>120219</v>
       </c>
@@ -9965,7 +9926,7 @@
       </c>
       <c r="J96" s="5"/>
     </row>
-    <row r="97" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A97" s="4">
         <v>120220</v>
       </c>
@@ -9993,7 +9954,7 @@
       </c>
       <c r="J97" s="5"/>
     </row>
-    <row r="98" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A98" s="4">
         <v>120221</v>
       </c>
@@ -10021,7 +9982,7 @@
       </c>
       <c r="J98" s="5"/>
     </row>
-    <row r="99" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A99" s="4">
         <v>120222</v>
       </c>
@@ -10049,7 +10010,7 @@
       </c>
       <c r="J99" s="5"/>
     </row>
-    <row r="100" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A100" s="4">
         <v>120223</v>
       </c>
@@ -10077,7 +10038,7 @@
       </c>
       <c r="J100" s="5"/>
     </row>
-    <row r="101" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A101" s="4">
         <v>120224</v>
       </c>
@@ -10105,7 +10066,7 @@
       </c>
       <c r="J101" s="5"/>
     </row>
-    <row r="102" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A102" s="4">
         <v>120225</v>
       </c>
@@ -10133,7 +10094,7 @@
       </c>
       <c r="J102" s="5"/>
     </row>
-    <row r="103" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A103" s="4">
         <v>120226</v>
       </c>
@@ -10161,7 +10122,7 @@
       </c>
       <c r="J103" s="5"/>
     </row>
-    <row r="104" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A104" s="4">
         <v>1203</v>
       </c>
@@ -10187,7 +10148,7 @@
       </c>
       <c r="J104" s="5"/>
     </row>
-    <row r="105" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A105" s="4">
         <v>120301</v>
       </c>
@@ -10215,7 +10176,7 @@
       </c>
       <c r="J105" s="5"/>
     </row>
-    <row r="106" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A106" s="4">
         <v>120302</v>
       </c>
@@ -10243,7 +10204,7 @@
       </c>
       <c r="J106" s="5"/>
     </row>
-    <row r="107" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A107" s="4">
         <v>120303</v>
       </c>
@@ -10271,7 +10232,7 @@
       </c>
       <c r="J107" s="5"/>
     </row>
-    <row r="108" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A108" s="4">
         <v>120304</v>
       </c>
@@ -10299,7 +10260,7 @@
       </c>
       <c r="J108" s="5"/>
     </row>
-    <row r="109" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A109" s="4">
         <v>120305</v>
       </c>
@@ -10327,7 +10288,7 @@
       </c>
       <c r="J109" s="5"/>
     </row>
-    <row r="110" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A110" s="4">
         <v>120306</v>
       </c>
@@ -10355,7 +10316,7 @@
       </c>
       <c r="J110" s="5"/>
     </row>
-    <row r="111" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A111" s="4">
         <v>1204</v>
       </c>
@@ -10381,7 +10342,7 @@
       </c>
       <c r="J111" s="5"/>
     </row>
-    <row r="112" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A112" s="4">
         <v>120401</v>
       </c>
@@ -10409,7 +10370,7 @@
       </c>
       <c r="J112" s="5"/>
     </row>
-    <row r="113" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A113" s="4">
         <v>120402</v>
       </c>
@@ -10437,7 +10398,7 @@
       </c>
       <c r="J113" s="5"/>
     </row>
-    <row r="114" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A114" s="4">
         <v>120403</v>
       </c>
@@ -10465,7 +10426,7 @@
       </c>
       <c r="J114" s="5"/>
     </row>
-    <row r="115" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A115" s="4">
         <v>120404</v>
       </c>
@@ -10493,7 +10454,7 @@
       </c>
       <c r="J115" s="5"/>
     </row>
-    <row r="116" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A116" s="4">
         <v>120405</v>
       </c>
@@ -10521,7 +10482,7 @@
       </c>
       <c r="J116" s="5"/>
     </row>
-    <row r="117" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A117" s="4">
         <v>120406</v>
       </c>
@@ -10549,7 +10510,7 @@
       </c>
       <c r="J117" s="5"/>
     </row>
-    <row r="118" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A118" s="4">
         <v>120407</v>
       </c>
@@ -10577,7 +10538,7 @@
       </c>
       <c r="J118" s="5"/>
     </row>
-    <row r="119" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A119" s="4">
         <v>120408</v>
       </c>
@@ -10605,7 +10566,7 @@
       </c>
       <c r="J119" s="5"/>
     </row>
-    <row r="120" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A120" s="4">
         <v>120409</v>
       </c>
@@ -10633,7 +10594,7 @@
       </c>
       <c r="J120" s="5"/>
     </row>
-    <row r="121" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A121" s="4">
         <v>120410</v>
       </c>
@@ -10661,7 +10622,7 @@
       </c>
       <c r="J121" s="5"/>
     </row>
-    <row r="122" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A122" s="4">
         <v>13</v>
       </c>
@@ -10685,7 +10646,7 @@
       </c>
       <c r="J122" s="5"/>
     </row>
-    <row r="123" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A123" s="4">
         <v>1301</v>
       </c>
@@ -10711,7 +10672,7 @@
       </c>
       <c r="J123" s="5"/>
     </row>
-    <row r="124" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A124" s="4">
         <v>130101</v>
       </c>
@@ -10739,7 +10700,7 @@
       </c>
       <c r="J124" s="5"/>
     </row>
-    <row r="125" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A125" s="4">
         <v>130102</v>
       </c>
@@ -10767,7 +10728,7 @@
       </c>
       <c r="J125" s="5"/>
     </row>
-    <row r="126" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A126" s="4">
         <v>130103</v>
       </c>
@@ -10795,7 +10756,7 @@
       </c>
       <c r="J126" s="5"/>
     </row>
-    <row r="127" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A127" s="4">
         <v>130104</v>
       </c>
@@ -10823,7 +10784,7 @@
       </c>
       <c r="J127" s="5"/>
     </row>
-    <row r="128" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A128" s="4">
         <v>130105</v>
       </c>
@@ -10851,7 +10812,7 @@
       </c>
       <c r="J128" s="5"/>
     </row>
-    <row r="129" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A129" s="4">
         <v>130106</v>
       </c>
@@ -10879,7 +10840,7 @@
       </c>
       <c r="J129" s="5"/>
     </row>
-    <row r="130" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A130" s="4">
         <v>130107</v>
       </c>
@@ -10907,7 +10868,7 @@
       </c>
       <c r="J130" s="5"/>
     </row>
-    <row r="131" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A131" s="4">
         <v>130108</v>
       </c>
@@ -10935,7 +10896,7 @@
       </c>
       <c r="J131" s="5"/>
     </row>
-    <row r="132" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A132" s="4">
         <v>130109</v>
       </c>
@@ -10963,7 +10924,7 @@
       </c>
       <c r="J132" s="5"/>
     </row>
-    <row r="133" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A133" s="4">
         <v>130110</v>
       </c>
@@ -10991,7 +10952,7 @@
       </c>
       <c r="J133" s="5"/>
     </row>
-    <row r="134" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A134" s="4">
         <v>130111</v>
       </c>
@@ -11019,7 +10980,7 @@
       </c>
       <c r="J134" s="5"/>
     </row>
-    <row r="135" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A135" s="4">
         <v>130112</v>
       </c>
@@ -11047,7 +11008,7 @@
       </c>
       <c r="J135" s="5"/>
     </row>
-    <row r="136" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A136" s="4">
         <v>130113</v>
       </c>
@@ -11075,7 +11036,7 @@
       </c>
       <c r="J136" s="5"/>
     </row>
-    <row r="137" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A137" s="4">
         <v>130114</v>
       </c>
@@ -11103,7 +11064,7 @@
       </c>
       <c r="J137" s="5"/>
     </row>
-    <row r="138" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A138" s="4">
         <v>130115</v>
       </c>
@@ -11131,7 +11092,7 @@
       </c>
       <c r="J138" s="5"/>
     </row>
-    <row r="139" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A139" s="4">
         <v>130116</v>
       </c>
@@ -11159,7 +11120,7 @@
       </c>
       <c r="J139" s="5"/>
     </row>
-    <row r="140" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A140" s="4">
         <v>130117</v>
       </c>
@@ -11187,7 +11148,7 @@
       </c>
       <c r="J140" s="5"/>
     </row>
-    <row r="141" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A141" s="4">
         <v>130118</v>
       </c>
@@ -11215,7 +11176,7 @@
       </c>
       <c r="J141" s="5"/>
     </row>
-    <row r="142" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A142" s="4">
         <v>130119</v>
       </c>
@@ -11243,7 +11204,7 @@
       </c>
       <c r="J142" s="5"/>
     </row>
-    <row r="143" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A143" s="4">
         <v>130120</v>
       </c>
@@ -11271,7 +11232,7 @@
       </c>
       <c r="J143" s="5"/>
     </row>
-    <row r="144" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A144" s="4">
         <v>130121</v>
       </c>
@@ -11299,7 +11260,7 @@
       </c>
       <c r="J144" s="5"/>
     </row>
-    <row r="145" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A145" s="4">
         <v>130122</v>
       </c>
@@ -11327,7 +11288,7 @@
       </c>
       <c r="J145" s="5"/>
     </row>
-    <row r="146" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A146" s="4">
         <v>1302</v>
       </c>
@@ -11353,7 +11314,7 @@
       </c>
       <c r="J146" s="5"/>
     </row>
-    <row r="147" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A147" s="4">
         <v>1303</v>
       </c>
@@ -11379,7 +11340,7 @@
       </c>
       <c r="J147" s="5"/>
     </row>
-    <row r="148" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A148" s="4">
         <v>130301</v>
       </c>
@@ -11407,7 +11368,7 @@
       </c>
       <c r="J148" s="5"/>
     </row>
-    <row r="149" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A149" s="4">
         <v>130302</v>
       </c>
@@ -11435,7 +11396,7 @@
       </c>
       <c r="J149" s="5"/>
     </row>
-    <row r="150" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A150" s="4">
         <v>130303</v>
       </c>
@@ -11463,7 +11424,7 @@
       </c>
       <c r="J150" s="5"/>
     </row>
-    <row r="151" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A151" s="4">
         <v>130304</v>
       </c>
@@ -11491,7 +11452,7 @@
       </c>
       <c r="J151" s="5"/>
     </row>
-    <row r="152" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A152" s="4">
         <v>130305</v>
       </c>
@@ -11519,7 +11480,7 @@
       </c>
       <c r="J152" s="5"/>
     </row>
-    <row r="153" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A153" s="4">
         <v>130306</v>
       </c>
@@ -11547,7 +11508,7 @@
       </c>
       <c r="J153" s="5"/>
     </row>
-    <row r="154" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A154" s="4">
         <v>130307</v>
       </c>
@@ -11575,7 +11536,7 @@
       </c>
       <c r="J154" s="5"/>
     </row>
-    <row r="155" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A155" s="4">
         <v>130308</v>
       </c>
@@ -11603,7 +11564,7 @@
       </c>
       <c r="J155" s="5"/>
     </row>
-    <row r="156" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A156" s="4">
         <v>130309</v>
       </c>
@@ -11631,7 +11592,7 @@
       </c>
       <c r="J156" s="5"/>
     </row>
-    <row r="157" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A157" s="4">
         <v>130310</v>
       </c>
@@ -11659,7 +11620,7 @@
       </c>
       <c r="J157" s="5"/>
     </row>
-    <row r="158" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A158" s="4">
         <v>130311</v>
       </c>
@@ -11687,7 +11648,7 @@
       </c>
       <c r="J158" s="5"/>
     </row>
-    <row r="159" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A159" s="4">
         <v>130312</v>
       </c>
@@ -11715,7 +11676,7 @@
       </c>
       <c r="J159" s="5"/>
     </row>
-    <row r="160" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A160" s="4">
         <v>130313</v>
       </c>
@@ -11743,7 +11704,7 @@
       </c>
       <c r="J160" s="5"/>
     </row>
-    <row r="161" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A161" s="4">
         <v>130314</v>
       </c>
@@ -11771,7 +11732,7 @@
       </c>
       <c r="J161" s="5"/>
     </row>
-    <row r="162" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A162" s="4">
         <v>130315</v>
       </c>
@@ -11799,7 +11760,7 @@
       </c>
       <c r="J162" s="5"/>
     </row>
-    <row r="163" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A163" s="4">
         <v>130316</v>
       </c>
@@ -11827,7 +11788,7 @@
       </c>
       <c r="J163" s="5"/>
     </row>
-    <row r="164" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A164" s="4">
         <v>130317</v>
       </c>
@@ -11855,7 +11816,7 @@
       </c>
       <c r="J164" s="5"/>
     </row>
-    <row r="165" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A165" s="4">
         <v>130318</v>
       </c>
@@ -11883,7 +11844,7 @@
       </c>
       <c r="J165" s="5"/>
     </row>
-    <row r="166" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A166" s="4">
         <v>130319</v>
       </c>
@@ -11911,7 +11872,7 @@
       </c>
       <c r="J166" s="5"/>
     </row>
-    <row r="167" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A167" s="4">
         <v>130320</v>
       </c>
@@ -11939,7 +11900,7 @@
       </c>
       <c r="J167" s="5"/>
     </row>
-    <row r="168" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A168" s="4">
         <v>130321</v>
       </c>
@@ -11967,7 +11928,7 @@
       </c>
       <c r="J168" s="5"/>
     </row>
-    <row r="169" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A169" s="4">
         <v>130322</v>
       </c>
@@ -11995,7 +11956,7 @@
       </c>
       <c r="J169" s="5"/>
     </row>
-    <row r="170" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A170" s="4">
         <v>130323</v>
       </c>
@@ -12023,7 +11984,7 @@
       </c>
       <c r="J170" s="5"/>
     </row>
-    <row r="171" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A171" s="4">
         <v>130324</v>
       </c>
@@ -12051,7 +12012,7 @@
       </c>
       <c r="J171" s="5"/>
     </row>
-    <row r="172" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A172" s="4">
         <v>130325</v>
       </c>
@@ -12079,7 +12040,7 @@
       </c>
       <c r="J172" s="5"/>
     </row>
-    <row r="173" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A173" s="4">
         <v>130326</v>
       </c>
@@ -12107,7 +12068,7 @@
       </c>
       <c r="J173" s="5"/>
     </row>
-    <row r="174" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A174" s="4">
         <v>1304</v>
       </c>
@@ -12133,7 +12094,7 @@
       </c>
       <c r="J174" s="5"/>
     </row>
-    <row r="175" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A175" s="4">
         <v>130401</v>
       </c>
@@ -12161,7 +12122,7 @@
       </c>
       <c r="J175" s="5"/>
     </row>
-    <row r="176" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A176" s="4">
         <v>130402</v>
       </c>
@@ -12189,7 +12150,7 @@
       </c>
       <c r="J176" s="5"/>
     </row>
-    <row r="177" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A177" s="4">
         <v>130403</v>
       </c>
@@ -12217,7 +12178,7 @@
       </c>
       <c r="J177" s="5"/>
     </row>
-    <row r="178" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A178" s="4">
         <v>130404</v>
       </c>
@@ -12245,7 +12206,7 @@
       </c>
       <c r="J178" s="5"/>
     </row>
-    <row r="179" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A179" s="4">
         <v>130405</v>
       </c>
@@ -12273,7 +12234,7 @@
       </c>
       <c r="J179" s="5"/>
     </row>
-    <row r="180" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A180" s="4">
         <v>130406</v>
       </c>
@@ -12301,7 +12262,7 @@
       </c>
       <c r="J180" s="5"/>
     </row>
-    <row r="181" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A181" s="4">
         <v>130407</v>
       </c>
@@ -12329,7 +12290,7 @@
       </c>
       <c r="J181" s="5"/>
     </row>
-    <row r="182" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A182" s="4">
         <v>130408</v>
       </c>
@@ -12357,7 +12318,7 @@
       </c>
       <c r="J182" s="5"/>
     </row>
-    <row r="183" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A183" s="4">
         <v>130409</v>
       </c>
@@ -12385,7 +12346,7 @@
       </c>
       <c r="J183" s="5"/>
     </row>
-    <row r="184" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A184" s="4">
         <v>130410</v>
       </c>
@@ -12413,7 +12374,7 @@
       </c>
       <c r="J184" s="5"/>
     </row>
-    <row r="185" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A185" s="4">
         <v>130411</v>
       </c>
@@ -12441,7 +12402,7 @@
       </c>
       <c r="J185" s="5"/>
     </row>
-    <row r="186" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A186" s="4">
         <v>130412</v>
       </c>
@@ -12469,7 +12430,7 @@
       </c>
       <c r="J186" s="5"/>
     </row>
-    <row r="187" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A187" s="4">
         <v>130413</v>
       </c>
@@ -12497,7 +12458,7 @@
       </c>
       <c r="J187" s="5"/>
     </row>
-    <row r="188" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A188" s="4">
         <v>130414</v>
       </c>
@@ -12525,7 +12486,7 @@
       </c>
       <c r="J188" s="5"/>
     </row>
-    <row r="189" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A189" s="4">
         <v>130415</v>
       </c>
@@ -12553,7 +12514,7 @@
       </c>
       <c r="J189" s="5"/>
     </row>
-    <row r="190" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A190" s="4">
         <v>130416</v>
       </c>
@@ -12581,7 +12542,7 @@
       </c>
       <c r="J190" s="5"/>
     </row>
-    <row r="191" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A191" s="4">
         <v>130417</v>
       </c>
@@ -12609,7 +12570,7 @@
       </c>
       <c r="J191" s="5"/>
     </row>
-    <row r="192" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A192" s="4">
         <v>130418</v>
       </c>
@@ -12637,7 +12598,7 @@
       </c>
       <c r="J192" s="5"/>
     </row>
-    <row r="193" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A193" s="4">
         <v>130419</v>
       </c>
@@ -12665,7 +12626,7 @@
       </c>
       <c r="J193" s="5"/>
     </row>
-    <row r="194" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A194" s="4">
         <v>130420</v>
       </c>
@@ -12693,7 +12654,7 @@
       </c>
       <c r="J194" s="5"/>
     </row>
-    <row r="195" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A195" s="4">
         <v>130421</v>
       </c>
@@ -12721,7 +12682,7 @@
       </c>
       <c r="J195" s="5"/>
     </row>
-    <row r="196" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A196" s="4">
         <v>130422</v>
       </c>
@@ -12749,7 +12710,7 @@
       </c>
       <c r="J196" s="5"/>
     </row>
-    <row r="197" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A197" s="4">
         <v>130423</v>
       </c>
@@ -12777,7 +12738,7 @@
       </c>
       <c r="J197" s="5"/>
     </row>
-    <row r="198" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A198" s="4">
         <v>130424</v>
       </c>
@@ -12805,7 +12766,7 @@
       </c>
       <c r="J198" s="5"/>
     </row>
-    <row r="199" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A199" s="4">
         <v>130425</v>
       </c>
@@ -12833,7 +12794,7 @@
       </c>
       <c r="J199" s="5"/>
     </row>
-    <row r="200" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A200" s="4">
         <v>130426</v>
       </c>
@@ -12861,7 +12822,7 @@
       </c>
       <c r="J200" s="5"/>
     </row>
-    <row r="201" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A201" s="4">
         <v>130427</v>
       </c>
@@ -12889,12 +12850,12 @@
       </c>
       <c r="J201" s="5"/>
     </row>
-    <row r="202" spans="1:10" ht="21" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A202" s="4">
         <v>1309</v>
       </c>
       <c r="B202" s="1" t="s">
-        <v>364</v>
+        <v>343</v>
       </c>
       <c r="C202" s="4">
         <v>13</v>
@@ -12907,15 +12868,15 @@
         <v>55</v>
       </c>
       <c r="G202" s="1" t="s">
-        <v>365</v>
+        <v>344</v>
       </c>
       <c r="H202" s="1"/>
       <c r="I202" s="1" t="s">
-        <v>364</v>
+        <v>343</v>
       </c>
       <c r="J202" s="5"/>
     </row>
-    <row r="203" spans="1:10" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A203" s="4">
         <v>1310</v>
       </c>
@@ -12941,7 +12902,7 @@
       </c>
       <c r="J203" s="5"/>
     </row>
-    <row r="204" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A204" s="4">
         <v>14</v>
       </c>
@@ -12965,7 +12926,7 @@
       </c>
       <c r="J204" s="5"/>
     </row>
-    <row r="205" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A205" s="4">
         <v>1401</v>
       </c>
@@ -12991,708 +12952,656 @@
       </c>
       <c r="J205" s="5"/>
     </row>
-    <row r="206" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A206" s="4">
-        <v>140101</v>
+        <v>1402</v>
       </c>
       <c r="B206" s="5" t="s">
         <v>245</v>
       </c>
       <c r="C206" s="4">
-        <v>1401</v>
+        <v>14</v>
       </c>
       <c r="D206" s="4">
-        <v>140101</v>
+        <v>1402</v>
       </c>
       <c r="E206" s="4"/>
       <c r="F206" s="4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G206" s="5" t="s">
         <v>246</v>
       </c>
-      <c r="H206" s="5" t="s">
-        <v>60</v>
-      </c>
+      <c r="H206" s="5"/>
       <c r="I206" s="5" t="s">
-        <v>60</v>
+        <v>245</v>
       </c>
       <c r="J206" s="5"/>
     </row>
-    <row r="207" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A207" s="4">
-        <v>140102</v>
+        <v>1403</v>
       </c>
       <c r="B207" s="5" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="C207" s="4">
-        <v>1401</v>
+        <v>14</v>
       </c>
       <c r="D207" s="4">
-        <v>140102</v>
+        <v>1403</v>
       </c>
       <c r="E207" s="4"/>
       <c r="F207" s="4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G207" s="5" t="s">
-        <v>246</v>
-      </c>
-      <c r="H207" s="5" t="s">
-        <v>61</v>
-      </c>
+        <v>248</v>
+      </c>
+      <c r="H207" s="5"/>
       <c r="I207" s="5" t="s">
-        <v>61</v>
+        <v>247</v>
       </c>
       <c r="J207" s="5"/>
     </row>
-    <row r="208" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A208" s="4">
-        <v>140103</v>
+        <v>1404</v>
       </c>
       <c r="B208" s="5" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="C208" s="4">
-        <v>1401</v>
+        <v>14</v>
       </c>
       <c r="D208" s="4">
-        <v>140103</v>
+        <v>1404</v>
       </c>
       <c r="E208" s="4"/>
       <c r="F208" s="4" t="s">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="G208" s="5" t="s">
-        <v>248</v>
-      </c>
-      <c r="H208" s="5" t="s">
-        <v>249</v>
-      </c>
+        <v>250</v>
+      </c>
+      <c r="H208" s="5"/>
       <c r="I208" s="5" t="s">
         <v>249</v>
       </c>
       <c r="J208" s="5"/>
     </row>
-    <row r="209" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A209" s="4">
-        <v>140104</v>
-      </c>
-      <c r="B209" s="5" t="s">
-        <v>247</v>
+        <v>1405</v>
+      </c>
+      <c r="B209" s="1" t="s">
+        <v>251</v>
       </c>
       <c r="C209" s="4">
-        <v>1401</v>
+        <v>14</v>
       </c>
       <c r="D209" s="4">
-        <v>140104</v>
+        <v>1405</v>
       </c>
       <c r="E209" s="4"/>
       <c r="F209" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="G209" s="5" t="s">
-        <v>248</v>
-      </c>
-      <c r="H209" s="5" t="s">
-        <v>250</v>
-      </c>
-      <c r="I209" s="5" t="s">
-        <v>250</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="G209" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="H209" s="1"/>
+      <c r="I209" s="1"/>
       <c r="J209" s="5"/>
     </row>
-    <row r="210" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A210" s="4">
-        <v>140105</v>
+        <v>15</v>
       </c>
       <c r="B210" s="5" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="C210" s="4">
-        <v>1401</v>
+        <v>1</v>
       </c>
       <c r="D210" s="4">
-        <v>140105</v>
+        <v>15</v>
       </c>
       <c r="E210" s="4"/>
       <c r="F210" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="G210" s="5" t="s">
-        <v>248</v>
-      </c>
-      <c r="H210" s="5" t="s">
-        <v>251</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G210" s="5"/>
+      <c r="H210" s="5"/>
       <c r="I210" s="5" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="J210" s="5"/>
     </row>
-    <row r="211" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A211" s="4">
-        <v>140106</v>
+        <v>1501</v>
       </c>
       <c r="B211" s="5" t="s">
-        <v>247</v>
+        <v>256</v>
       </c>
       <c r="C211" s="4">
-        <v>1401</v>
+        <v>15</v>
       </c>
       <c r="D211" s="4">
-        <v>140106</v>
+        <v>1501</v>
       </c>
       <c r="E211" s="4"/>
       <c r="F211" s="4" t="s">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="G211" s="5" t="s">
-        <v>248</v>
-      </c>
-      <c r="H211" s="5" t="s">
-        <v>252</v>
-      </c>
+        <v>257</v>
+      </c>
+      <c r="H211" s="5"/>
       <c r="I211" s="5" t="s">
-        <v>252</v>
+        <v>256</v>
       </c>
       <c r="J211" s="5"/>
     </row>
-    <row r="212" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A212" s="4">
-        <v>140107</v>
+        <v>1502</v>
       </c>
       <c r="B212" s="5" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="C212" s="4">
-        <v>1401</v>
+        <v>15</v>
       </c>
       <c r="D212" s="4">
-        <v>140107</v>
+        <v>1502</v>
       </c>
       <c r="E212" s="4"/>
       <c r="F212" s="4" t="s">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="G212" s="5" t="s">
-        <v>248</v>
-      </c>
-      <c r="H212" s="5" t="s">
-        <v>253</v>
-      </c>
+        <v>255</v>
+      </c>
+      <c r="H212" s="5"/>
       <c r="I212" s="5" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="J212" s="5"/>
     </row>
-    <row r="213" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A213" s="4">
-        <v>140108</v>
+        <v>1503</v>
       </c>
       <c r="B213" s="5" t="s">
-        <v>247</v>
+        <v>258</v>
       </c>
       <c r="C213" s="4">
-        <v>1401</v>
+        <v>15</v>
       </c>
       <c r="D213" s="4">
-        <v>140108</v>
+        <v>1503</v>
       </c>
       <c r="E213" s="4"/>
       <c r="F213" s="4" t="s">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="G213" s="5" t="s">
-        <v>248</v>
-      </c>
-      <c r="H213" s="5" t="s">
-        <v>254</v>
-      </c>
+        <v>259</v>
+      </c>
+      <c r="H213" s="5"/>
       <c r="I213" s="5" t="s">
-        <v>254</v>
+        <v>258</v>
       </c>
       <c r="J213" s="5"/>
     </row>
-    <row r="214" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A214" s="4">
-        <v>140109</v>
+        <v>1504</v>
       </c>
       <c r="B214" s="5" t="s">
-        <v>247</v>
+        <v>260</v>
       </c>
       <c r="C214" s="4">
-        <v>1401</v>
+        <v>15</v>
       </c>
       <c r="D214" s="4">
-        <v>140109</v>
+        <v>1504</v>
       </c>
       <c r="E214" s="4"/>
       <c r="F214" s="4" t="s">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="G214" s="5" t="s">
-        <v>248</v>
-      </c>
-      <c r="H214" s="5" t="s">
-        <v>255</v>
-      </c>
+        <v>261</v>
+      </c>
+      <c r="H214" s="5"/>
       <c r="I214" s="5" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="J214" s="5"/>
     </row>
-    <row r="215" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="215" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A215" s="4">
-        <v>140110</v>
+        <v>16</v>
       </c>
       <c r="B215" s="5" t="s">
-        <v>247</v>
+        <v>262</v>
       </c>
       <c r="C215" s="4">
-        <v>1401</v>
+        <v>1</v>
       </c>
       <c r="D215" s="4">
-        <v>140110</v>
+        <v>16</v>
       </c>
       <c r="E215" s="4"/>
       <c r="F215" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="G215" s="5" t="s">
-        <v>248</v>
-      </c>
-      <c r="H215" s="5" t="s">
-        <v>64</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G215" s="5"/>
+      <c r="H215" s="5"/>
       <c r="I215" s="5" t="s">
-        <v>64</v>
+        <v>262</v>
       </c>
       <c r="J215" s="5"/>
     </row>
-    <row r="216" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="216" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A216" s="4">
-        <v>140111</v>
+        <v>1601</v>
       </c>
       <c r="B216" s="5" t="s">
-        <v>247</v>
+        <v>263</v>
       </c>
       <c r="C216" s="4">
-        <v>1401</v>
+        <v>16</v>
       </c>
       <c r="D216" s="4">
-        <v>140111</v>
+        <v>1601</v>
       </c>
       <c r="E216" s="4"/>
       <c r="F216" s="4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G216" s="5" t="s">
-        <v>248</v>
-      </c>
-      <c r="H216" s="5" t="s">
-        <v>65</v>
-      </c>
+        <v>264</v>
+      </c>
+      <c r="H216" s="5"/>
       <c r="I216" s="5" t="s">
-        <v>65</v>
+        <v>263</v>
       </c>
       <c r="J216" s="5"/>
     </row>
-    <row r="217" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="217" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A217" s="4">
-        <v>140112</v>
-      </c>
-      <c r="B217" s="5" t="s">
-        <v>256</v>
+        <v>1602</v>
+      </c>
+      <c r="B217" s="1" t="s">
+        <v>265</v>
       </c>
       <c r="C217" s="4">
-        <v>1401</v>
+        <v>16</v>
       </c>
       <c r="D217" s="4">
-        <v>140112</v>
+        <v>1602</v>
       </c>
       <c r="E217" s="4"/>
       <c r="F217" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="G217" s="5" t="s">
-        <v>257</v>
-      </c>
-      <c r="H217" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="I217" s="5" t="s">
-        <v>64</v>
+        <v>55</v>
+      </c>
+      <c r="G217" s="12" t="s">
+        <v>345</v>
+      </c>
+      <c r="H217" s="1"/>
+      <c r="I217" s="1" t="s">
+        <v>265</v>
       </c>
       <c r="J217" s="5"/>
     </row>
-    <row r="218" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="218" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A218" s="4">
-        <v>140113</v>
+        <v>1603</v>
       </c>
       <c r="B218" s="5" t="s">
-        <v>256</v>
+        <v>266</v>
       </c>
       <c r="C218" s="4">
-        <v>1401</v>
+        <v>16</v>
       </c>
       <c r="D218" s="4">
-        <v>140113</v>
+        <v>1603</v>
       </c>
       <c r="E218" s="4"/>
       <c r="F218" s="4" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G218" s="5" t="s">
-        <v>257</v>
-      </c>
-      <c r="H218" s="5" t="s">
-        <v>65</v>
-      </c>
+        <v>267</v>
+      </c>
+      <c r="H218" s="5"/>
       <c r="I218" s="5" t="s">
-        <v>65</v>
+        <v>266</v>
       </c>
       <c r="J218" s="5"/>
     </row>
-    <row r="219" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="219" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A219" s="4">
-        <v>1402</v>
+        <v>1604</v>
       </c>
       <c r="B219" s="5" t="s">
-        <v>258</v>
+        <v>268</v>
       </c>
       <c r="C219" s="4">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="D219" s="4">
-        <v>1402</v>
+        <v>1604</v>
       </c>
       <c r="E219" s="4"/>
       <c r="F219" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G219" s="5" t="s">
-        <v>259</v>
+        <v>269</v>
       </c>
       <c r="H219" s="5"/>
       <c r="I219" s="5" t="s">
-        <v>258</v>
+        <v>268</v>
       </c>
       <c r="J219" s="5"/>
     </row>
-    <row r="220" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="220" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A220" s="4">
-        <v>140201</v>
-      </c>
-      <c r="B220" s="5" t="s">
-        <v>260</v>
+        <v>1605</v>
+      </c>
+      <c r="B220" s="12" t="s">
+        <v>348</v>
       </c>
       <c r="C220" s="4">
-        <v>1402</v>
+        <v>16</v>
       </c>
       <c r="D220" s="4">
-        <v>140201</v>
+        <v>1605</v>
       </c>
       <c r="E220" s="4"/>
       <c r="F220" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="G220" s="5" t="s">
-        <v>261</v>
-      </c>
-      <c r="H220" s="5" t="s">
-        <v>90</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="G220" s="12" t="s">
+        <v>350</v>
+      </c>
+      <c r="H220" s="5"/>
       <c r="I220" s="5" t="s">
-        <v>90</v>
+        <v>260</v>
       </c>
       <c r="J220" s="5"/>
     </row>
-    <row r="221" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="221" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A221" s="4">
-        <v>140202</v>
+        <v>1606</v>
       </c>
       <c r="B221" s="5" t="s">
-        <v>262</v>
+        <v>270</v>
       </c>
       <c r="C221" s="4">
-        <v>1402</v>
+        <v>16</v>
       </c>
       <c r="D221" s="4">
-        <v>140202</v>
+        <v>1606</v>
       </c>
       <c r="E221" s="4"/>
       <c r="F221" s="4" t="s">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="G221" s="5" t="s">
-        <v>263</v>
-      </c>
-      <c r="H221" s="5" t="s">
-        <v>69</v>
-      </c>
+        <v>271</v>
+      </c>
+      <c r="H221" s="5"/>
       <c r="I221" s="5" t="s">
-        <v>69</v>
+        <v>270</v>
       </c>
       <c r="J221" s="5"/>
     </row>
-    <row r="222" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="222" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A222" s="4">
-        <v>140203</v>
+        <v>1607</v>
       </c>
       <c r="B222" s="5" t="s">
-        <v>262</v>
+        <v>272</v>
       </c>
       <c r="C222" s="4">
-        <v>1402</v>
+        <v>16</v>
       </c>
       <c r="D222" s="4">
-        <v>140203</v>
+        <v>1607</v>
       </c>
       <c r="E222" s="4"/>
       <c r="F222" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="G222" s="5" t="s">
-        <v>263</v>
-      </c>
-      <c r="H222" s="5" t="s">
-        <v>64</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="G222" s="12" t="s">
+        <v>349</v>
+      </c>
+      <c r="H222" s="5"/>
       <c r="I222" s="5" t="s">
-        <v>64</v>
+        <v>272</v>
       </c>
       <c r="J222" s="5"/>
     </row>
-    <row r="223" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="223" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A223" s="4">
-        <v>140204</v>
-      </c>
-      <c r="B223" s="5" t="s">
-        <v>262</v>
+        <v>1608</v>
+      </c>
+      <c r="B223" s="12" t="s">
+        <v>342</v>
       </c>
       <c r="C223" s="4">
-        <v>1402</v>
+        <v>16</v>
       </c>
       <c r="D223" s="4">
-        <v>140204</v>
+        <v>1608</v>
       </c>
       <c r="E223" s="4"/>
       <c r="F223" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="G223" s="5" t="s">
-        <v>263</v>
-      </c>
-      <c r="H223" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="I223" s="5" t="s">
-        <v>65</v>
+        <v>55</v>
+      </c>
+      <c r="G223" s="12" t="s">
+        <v>341</v>
+      </c>
+      <c r="H223" s="5"/>
+      <c r="I223" s="12" t="s">
+        <v>342</v>
       </c>
       <c r="J223" s="5"/>
     </row>
-    <row r="224" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="224" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A224" s="4">
-        <v>140205</v>
-      </c>
-      <c r="B224" s="5" t="s">
-        <v>264</v>
+        <v>17</v>
+      </c>
+      <c r="B224" s="12" t="s">
+        <v>338</v>
       </c>
       <c r="C224" s="4">
-        <v>1402</v>
+        <v>1</v>
       </c>
       <c r="D224" s="4">
-        <v>140205</v>
+        <v>17</v>
       </c>
       <c r="E224" s="4"/>
       <c r="F224" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="G224" s="5" t="s">
-        <v>265</v>
-      </c>
-      <c r="H224" s="5" t="s">
-        <v>69</v>
-      </c>
-      <c r="I224" s="5" t="s">
-        <v>69</v>
+        <v>52</v>
+      </c>
+      <c r="G224" s="5"/>
+      <c r="H224" s="5"/>
+      <c r="I224" s="12" t="s">
+        <v>338</v>
       </c>
       <c r="J224" s="5"/>
     </row>
-    <row r="225" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="225" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A225" s="4">
-        <v>140206</v>
-      </c>
-      <c r="B225" s="5" t="s">
-        <v>264</v>
+        <v>1701</v>
+      </c>
+      <c r="B225" s="12" t="s">
+        <v>339</v>
       </c>
       <c r="C225" s="4">
-        <v>1402</v>
+        <v>17</v>
       </c>
       <c r="D225" s="4">
-        <v>140206</v>
+        <v>1701</v>
       </c>
       <c r="E225" s="4"/>
       <c r="F225" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="G225" s="5" t="s">
-        <v>265</v>
-      </c>
-      <c r="H225" s="5" t="s">
-        <v>90</v>
-      </c>
-      <c r="I225" s="5" t="s">
-        <v>90</v>
+        <v>55</v>
+      </c>
+      <c r="G225" s="12" t="s">
+        <v>340</v>
+      </c>
+      <c r="H225" s="5"/>
+      <c r="I225" s="12" t="s">
+        <v>339</v>
       </c>
       <c r="J225" s="5"/>
     </row>
-    <row r="226" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="226" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A226" s="4">
-        <v>140207</v>
-      </c>
-      <c r="B226" s="5" t="s">
-        <v>264</v>
+        <v>1702</v>
+      </c>
+      <c r="B226" s="12" t="s">
+        <v>346</v>
       </c>
       <c r="C226" s="4">
-        <v>1402</v>
+        <v>17</v>
       </c>
       <c r="D226" s="4">
-        <v>140207</v>
+        <v>1702</v>
       </c>
       <c r="E226" s="4"/>
       <c r="F226" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="G226" s="5" t="s">
-        <v>265</v>
-      </c>
-      <c r="H226" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="I226" s="5" t="s">
-        <v>64</v>
+        <v>55</v>
+      </c>
+      <c r="G226" s="12" t="s">
+        <v>347</v>
+      </c>
+      <c r="H226" s="5"/>
+      <c r="I226" s="12" t="s">
+        <v>346</v>
       </c>
       <c r="J226" s="5"/>
     </row>
-    <row r="227" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="227" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A227" s="4">
-        <v>140208</v>
+        <v>2</v>
       </c>
       <c r="B227" s="5" t="s">
-        <v>264</v>
+        <v>273</v>
       </c>
       <c r="C227" s="4">
-        <v>1402</v>
+        <v>-1</v>
       </c>
       <c r="D227" s="4">
-        <v>140208</v>
+        <v>2</v>
       </c>
       <c r="E227" s="4"/>
       <c r="F227" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="G227" s="5" t="s">
-        <v>265</v>
-      </c>
-      <c r="H227" s="5" t="s">
-        <v>65</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G227" s="5"/>
+      <c r="H227" s="5"/>
       <c r="I227" s="5" t="s">
-        <v>65</v>
+        <v>273</v>
       </c>
       <c r="J227" s="5"/>
     </row>
-    <row r="228" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="228" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A228" s="4">
-        <v>1403</v>
+        <v>21</v>
       </c>
       <c r="B228" s="5" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
       <c r="C228" s="4">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="D228" s="4">
-        <v>1403</v>
+        <v>21</v>
       </c>
       <c r="E228" s="4"/>
       <c r="F228" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G228" s="5" t="s">
-        <v>267</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G228" s="5"/>
       <c r="H228" s="5"/>
       <c r="I228" s="5" t="s">
-        <v>266</v>
+        <v>274</v>
       </c>
       <c r="J228" s="5"/>
     </row>
-    <row r="229" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="229" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A229" s="4">
-        <v>1404</v>
+        <v>2110</v>
       </c>
       <c r="B229" s="5" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="C229" s="4">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="D229" s="4">
-        <v>1404</v>
+        <v>2110</v>
       </c>
       <c r="E229" s="4"/>
       <c r="F229" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G229" s="5" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="H229" s="5"/>
       <c r="I229" s="5" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="J229" s="5"/>
     </row>
-    <row r="230" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="230" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A230" s="4">
-        <v>1405</v>
-      </c>
-      <c r="B230" s="1" t="s">
-        <v>270</v>
+        <v>2111</v>
+      </c>
+      <c r="B230" s="5" t="s">
+        <v>277</v>
       </c>
       <c r="C230" s="4">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="D230" s="4">
-        <v>1405</v>
+        <v>2111</v>
       </c>
       <c r="E230" s="4"/>
       <c r="F230" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="G230" s="1" t="s">
-        <v>271</v>
-      </c>
-      <c r="H230" s="1"/>
-      <c r="I230" s="1"/>
+      <c r="G230" s="5" t="s">
+        <v>278</v>
+      </c>
+      <c r="H230" s="5"/>
+      <c r="I230" s="5" t="s">
+        <v>277</v>
+      </c>
       <c r="J230" s="5"/>
     </row>
-    <row r="231" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="231" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A231" s="4">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="B231" s="5" t="s">
-        <v>272</v>
+        <v>279</v>
       </c>
       <c r="C231" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D231" s="4">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="E231" s="4"/>
       <c r="F231" s="4" t="s">
@@ -13701,406 +13610,406 @@
       <c r="G231" s="5"/>
       <c r="H231" s="5"/>
       <c r="I231" s="5" t="s">
-        <v>272</v>
+        <v>279</v>
       </c>
       <c r="J231" s="5"/>
     </row>
-    <row r="232" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="232" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A232" s="4">
-        <v>1501</v>
+        <v>2201</v>
       </c>
       <c r="B232" s="5" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="C232" s="4">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="D232" s="4">
-        <v>1501</v>
+        <v>2201</v>
       </c>
       <c r="E232" s="4"/>
       <c r="F232" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G232" s="5" t="s">
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="H232" s="5"/>
       <c r="I232" s="5" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="J232" s="5"/>
     </row>
-    <row r="233" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="233" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A233" s="4">
-        <v>1502</v>
+        <v>2202</v>
       </c>
       <c r="B233" s="5" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="C233" s="4">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="D233" s="4">
-        <v>1502</v>
+        <v>2202</v>
       </c>
       <c r="E233" s="4"/>
       <c r="F233" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G233" s="5" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="H233" s="5"/>
       <c r="I233" s="5" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="J233" s="5"/>
     </row>
-    <row r="234" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="234" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A234" s="4">
-        <v>1503</v>
+        <v>2203</v>
       </c>
       <c r="B234" s="5" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="C234" s="4">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="D234" s="4">
-        <v>1503</v>
+        <v>2203</v>
       </c>
       <c r="E234" s="4"/>
       <c r="F234" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G234" s="5" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="H234" s="5"/>
       <c r="I234" s="5" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
       <c r="J234" s="5"/>
     </row>
-    <row r="235" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="235" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A235" s="4">
-        <v>1504</v>
+        <v>23</v>
       </c>
       <c r="B235" s="5" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="C235" s="4">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="D235" s="4">
-        <v>1504</v>
+        <v>23</v>
       </c>
       <c r="E235" s="4"/>
       <c r="F235" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G235" s="5" t="s">
-        <v>280</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G235" s="5"/>
       <c r="H235" s="5"/>
       <c r="I235" s="5" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="J235" s="5"/>
     </row>
-    <row r="236" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="236" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A236" s="4">
-        <v>16</v>
+        <v>2301</v>
       </c>
       <c r="B236" s="5" t="s">
-        <v>281</v>
+        <v>287</v>
       </c>
       <c r="C236" s="4">
-        <v>1</v>
+        <v>23</v>
       </c>
       <c r="D236" s="4">
-        <v>16</v>
+        <v>2301</v>
       </c>
       <c r="E236" s="4"/>
       <c r="F236" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G236" s="5"/>
+        <v>55</v>
+      </c>
+      <c r="G236" s="5" t="s">
+        <v>288</v>
+      </c>
       <c r="H236" s="5"/>
       <c r="I236" s="5" t="s">
-        <v>281</v>
+        <v>287</v>
       </c>
       <c r="J236" s="5"/>
     </row>
-    <row r="237" spans="1:10" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="237" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A237" s="4">
-        <v>1601</v>
+        <v>2302</v>
       </c>
       <c r="B237" s="5" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="C237" s="4">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="D237" s="4">
-        <v>1601</v>
+        <v>2302</v>
       </c>
       <c r="E237" s="4"/>
       <c r="F237" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G237" s="5" t="s">
-        <v>283</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G237" s="5"/>
       <c r="H237" s="5"/>
       <c r="I237" s="5" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="J237" s="5"/>
     </row>
-    <row r="238" spans="1:10" x14ac:dyDescent="0.2">
+    <row r="238" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A238" s="4">
-        <v>1602</v>
-      </c>
-      <c r="B238" s="1" t="s">
-        <v>284</v>
+        <v>23021</v>
+      </c>
+      <c r="B238" s="5" t="s">
+        <v>290</v>
       </c>
       <c r="C238" s="4">
-        <v>16</v>
+        <v>2302</v>
       </c>
       <c r="D238" s="4">
-        <v>1602</v>
+        <v>23021</v>
       </c>
       <c r="E238" s="4"/>
       <c r="F238" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G238" s="5" t="s">
-        <v>285</v>
-      </c>
-      <c r="H238" s="1"/>
-      <c r="I238" s="1" t="s">
-        <v>284</v>
+        <v>291</v>
+      </c>
+      <c r="H238" s="5"/>
+      <c r="I238" s="5" t="s">
+        <v>292</v>
       </c>
       <c r="J238" s="5"/>
     </row>
-    <row r="239" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="239" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A239" s="4">
-        <v>1603</v>
+        <v>23022</v>
       </c>
       <c r="B239" s="5" t="s">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="C239" s="4">
-        <v>16</v>
+        <v>2302</v>
       </c>
       <c r="D239" s="4">
-        <v>1603</v>
+        <v>23022</v>
       </c>
       <c r="E239" s="4"/>
       <c r="F239" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G239" s="5" t="s">
-        <v>287</v>
+        <v>294</v>
       </c>
       <c r="H239" s="5"/>
       <c r="I239" s="5" t="s">
-        <v>286</v>
+        <v>295</v>
       </c>
       <c r="J239" s="5"/>
     </row>
-    <row r="240" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="240" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A240" s="4">
-        <v>1604</v>
+        <v>2303</v>
       </c>
       <c r="B240" s="5" t="s">
-        <v>288</v>
+        <v>253</v>
       </c>
       <c r="C240" s="4">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="D240" s="4">
-        <v>1604</v>
+        <v>2303</v>
       </c>
       <c r="E240" s="4"/>
       <c r="F240" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G240" s="5" t="s">
-        <v>289</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G240" s="5"/>
       <c r="H240" s="5"/>
       <c r="I240" s="5" t="s">
-        <v>288</v>
+        <v>253</v>
       </c>
       <c r="J240" s="5"/>
     </row>
-    <row r="241" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="241" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A241" s="4">
-        <v>1605</v>
+        <v>23031</v>
       </c>
       <c r="B241" s="5" t="s">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="C241" s="4">
-        <v>16</v>
+        <v>2303</v>
       </c>
       <c r="D241" s="4">
-        <v>1605</v>
+        <v>23031</v>
       </c>
       <c r="E241" s="4"/>
       <c r="F241" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G241" s="5" t="s">
-        <v>291</v>
+        <v>297</v>
       </c>
       <c r="H241" s="5"/>
       <c r="I241" s="5" t="s">
-        <v>290</v>
+        <v>296</v>
       </c>
       <c r="J241" s="5"/>
     </row>
-    <row r="242" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="242" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A242" s="4">
-        <v>1606</v>
+        <v>23032</v>
       </c>
       <c r="B242" s="5" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="C242" s="4">
-        <v>16</v>
+        <v>2303</v>
       </c>
       <c r="D242" s="4">
-        <v>1606</v>
+        <v>23032</v>
       </c>
       <c r="E242" s="4"/>
       <c r="F242" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G242" s="5" t="s">
-        <v>293</v>
+        <v>299</v>
       </c>
       <c r="H242" s="5"/>
       <c r="I242" s="5" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
       <c r="J242" s="5"/>
     </row>
-    <row r="243" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="243" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A243" s="4">
-        <v>1607</v>
-      </c>
-      <c r="B243" s="12" t="s">
-        <v>363</v>
+        <v>23033</v>
+      </c>
+      <c r="B243" s="5" t="s">
+        <v>300</v>
       </c>
       <c r="C243" s="4">
-        <v>16</v>
+        <v>2303</v>
       </c>
       <c r="D243" s="4">
-        <v>1607</v>
+        <v>23033</v>
       </c>
       <c r="E243" s="4"/>
       <c r="F243" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="G243" s="12" t="s">
-        <v>362</v>
+      <c r="G243" s="5" t="s">
+        <v>301</v>
       </c>
       <c r="H243" s="5"/>
-      <c r="I243" s="12" t="s">
-        <v>363</v>
+      <c r="I243" s="5" t="s">
+        <v>300</v>
       </c>
       <c r="J243" s="5"/>
     </row>
-    <row r="244" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="244" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A244" s="4">
-        <v>17</v>
+        <v>23034</v>
       </c>
       <c r="B244" s="12" t="s">
-        <v>359</v>
+        <v>334</v>
       </c>
       <c r="C244" s="4">
-        <v>1</v>
+        <v>2303</v>
       </c>
       <c r="D244" s="4">
-        <v>17</v>
+        <v>23034</v>
       </c>
       <c r="E244" s="4"/>
       <c r="F244" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G244" s="5"/>
+        <v>55</v>
+      </c>
+      <c r="G244" s="12" t="s">
+        <v>337</v>
+      </c>
       <c r="H244" s="5"/>
       <c r="I244" s="12" t="s">
-        <v>359</v>
+        <v>334</v>
       </c>
       <c r="J244" s="5"/>
     </row>
-    <row r="245" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="245" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A245" s="4">
-        <v>1701</v>
-      </c>
-      <c r="B245" s="12" t="s">
-        <v>360</v>
+        <v>23035</v>
+      </c>
+      <c r="B245" s="5" t="s">
+        <v>302</v>
       </c>
       <c r="C245" s="4">
-        <v>17</v>
+        <v>2303</v>
       </c>
       <c r="D245" s="4">
-        <v>1701</v>
+        <v>23035</v>
       </c>
       <c r="E245" s="4"/>
       <c r="F245" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="G245" s="12" t="s">
-        <v>361</v>
+      <c r="G245" s="5" t="s">
+        <v>303</v>
       </c>
       <c r="H245" s="5"/>
-      <c r="I245" s="12" t="s">
-        <v>360</v>
+      <c r="I245" s="5" t="s">
+        <v>302</v>
       </c>
       <c r="J245" s="5"/>
     </row>
-    <row r="246" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="246" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A246" s="4">
-        <v>2</v>
-      </c>
-      <c r="B246" s="5" t="s">
-        <v>294</v>
+        <v>23036</v>
+      </c>
+      <c r="B246" s="12" t="s">
+        <v>335</v>
       </c>
       <c r="C246" s="4">
-        <v>-1</v>
+        <v>2303</v>
       </c>
       <c r="D246" s="4">
-        <v>2</v>
+        <v>23036</v>
       </c>
       <c r="E246" s="4"/>
       <c r="F246" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G246" s="5"/>
+        <v>55</v>
+      </c>
+      <c r="G246" s="12" t="s">
+        <v>336</v>
+      </c>
       <c r="H246" s="5"/>
-      <c r="I246" s="5" t="s">
-        <v>294</v>
+      <c r="I246" s="12" t="s">
+        <v>335</v>
       </c>
       <c r="J246" s="5"/>
     </row>
-    <row r="247" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="247" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A247" s="4">
-        <v>21</v>
+        <v>2304</v>
       </c>
       <c r="B247" s="5" t="s">
-        <v>295</v>
+        <v>304</v>
       </c>
       <c r="C247" s="4">
-        <v>2</v>
+        <v>23</v>
       </c>
       <c r="D247" s="4">
-        <v>21</v>
+        <v>2304</v>
       </c>
       <c r="E247" s="4"/>
       <c r="F247" s="4" t="s">
@@ -14109,925 +14018,441 @@
       <c r="G247" s="5"/>
       <c r="H247" s="5"/>
       <c r="I247" s="5" t="s">
-        <v>295</v>
+        <v>304</v>
       </c>
       <c r="J247" s="5"/>
     </row>
-    <row r="248" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="248" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A248" s="4">
-        <v>2110</v>
+        <v>23041</v>
       </c>
       <c r="B248" s="5" t="s">
-        <v>296</v>
+        <v>305</v>
       </c>
       <c r="C248" s="4">
-        <v>21</v>
+        <v>2304</v>
       </c>
       <c r="D248" s="4">
-        <v>2110</v>
+        <v>23041</v>
       </c>
       <c r="E248" s="4"/>
       <c r="F248" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G248" s="5" t="s">
-        <v>297</v>
+        <v>306</v>
       </c>
       <c r="H248" s="5"/>
       <c r="I248" s="5" t="s">
-        <v>296</v>
+        <v>305</v>
       </c>
       <c r="J248" s="5"/>
     </row>
-    <row r="249" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="249" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A249" s="4">
-        <v>2111</v>
+        <v>2305</v>
       </c>
       <c r="B249" s="5" t="s">
-        <v>298</v>
+        <v>39</v>
       </c>
       <c r="C249" s="4">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D249" s="4">
-        <v>2111</v>
+        <v>2305</v>
       </c>
       <c r="E249" s="4"/>
       <c r="F249" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G249" s="5" t="s">
-        <v>299</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G249" s="5"/>
       <c r="H249" s="5"/>
       <c r="I249" s="5" t="s">
-        <v>298</v>
+        <v>39</v>
       </c>
       <c r="J249" s="5"/>
     </row>
-    <row r="250" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="250" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A250" s="4">
-        <v>22</v>
+        <v>23051</v>
       </c>
       <c r="B250" s="5" t="s">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="C250" s="4">
-        <v>2</v>
+        <v>2305</v>
       </c>
       <c r="D250" s="4">
-        <v>22</v>
+        <v>23051</v>
       </c>
       <c r="E250" s="4"/>
       <c r="F250" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G250" s="5"/>
+        <v>55</v>
+      </c>
+      <c r="G250" s="5" t="s">
+        <v>308</v>
+      </c>
       <c r="H250" s="5"/>
       <c r="I250" s="5" t="s">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="J250" s="5"/>
     </row>
-    <row r="251" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="251" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A251" s="4">
-        <v>2201</v>
+        <v>2306</v>
       </c>
       <c r="B251" s="5" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
       <c r="C251" s="4">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D251" s="4">
-        <v>2201</v>
+        <v>2306</v>
       </c>
       <c r="E251" s="4"/>
       <c r="F251" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G251" s="5" t="s">
-        <v>302</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G251" s="5"/>
       <c r="H251" s="5"/>
       <c r="I251" s="5" t="s">
-        <v>301</v>
+        <v>309</v>
       </c>
       <c r="J251" s="5"/>
     </row>
-    <row r="252" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="252" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A252" s="4">
-        <v>2202</v>
+        <v>23061</v>
       </c>
       <c r="B252" s="5" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="C252" s="4">
-        <v>22</v>
+        <v>2306</v>
       </c>
       <c r="D252" s="4">
-        <v>2202</v>
+        <v>23061</v>
       </c>
       <c r="E252" s="4"/>
       <c r="F252" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G252" s="5" t="s">
-        <v>304</v>
+        <v>311</v>
       </c>
       <c r="H252" s="5"/>
       <c r="I252" s="5" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="J252" s="5"/>
     </row>
-    <row r="253" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="253" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A253" s="4">
-        <v>2203</v>
+        <v>23062</v>
       </c>
       <c r="B253" s="5" t="s">
-        <v>305</v>
+        <v>312</v>
       </c>
       <c r="C253" s="4">
-        <v>22</v>
+        <v>2306</v>
       </c>
       <c r="D253" s="4">
-        <v>2203</v>
+        <v>23062</v>
       </c>
       <c r="E253" s="4"/>
       <c r="F253" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G253" s="5" t="s">
-        <v>306</v>
+        <v>313</v>
       </c>
       <c r="H253" s="5"/>
       <c r="I253" s="5" t="s">
-        <v>305</v>
+        <v>312</v>
       </c>
       <c r="J253" s="5"/>
     </row>
-    <row r="254" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="254" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A254" s="4">
-        <v>23</v>
+        <v>23063</v>
       </c>
       <c r="B254" s="5" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
       <c r="C254" s="4">
-        <v>2</v>
+        <v>2306</v>
       </c>
       <c r="D254" s="4">
-        <v>23</v>
+        <v>23063</v>
       </c>
       <c r="E254" s="4"/>
       <c r="F254" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G254" s="5"/>
+        <v>55</v>
+      </c>
+      <c r="G254" s="5" t="s">
+        <v>315</v>
+      </c>
       <c r="H254" s="5"/>
       <c r="I254" s="5" t="s">
-        <v>307</v>
+        <v>316</v>
       </c>
       <c r="J254" s="5"/>
     </row>
-    <row r="255" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="255" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A255" s="4">
-        <v>2301</v>
+        <v>2307</v>
       </c>
       <c r="B255" s="5" t="s">
-        <v>308</v>
+        <v>317</v>
       </c>
       <c r="C255" s="4">
         <v>23</v>
       </c>
       <c r="D255" s="4">
-        <v>2301</v>
+        <v>2307</v>
       </c>
       <c r="E255" s="4"/>
       <c r="F255" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G255" s="5" t="s">
-        <v>309</v>
-      </c>
-      <c r="H255" s="5"/>
+        <v>52</v>
+      </c>
+      <c r="G255" s="4"/>
+      <c r="H255" s="4"/>
       <c r="I255" s="5" t="s">
-        <v>308</v>
+        <v>317</v>
       </c>
       <c r="J255" s="5"/>
     </row>
-    <row r="256" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="256" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A256" s="4">
-        <v>2302</v>
+        <v>23071</v>
       </c>
       <c r="B256" s="5" t="s">
-        <v>310</v>
+        <v>318</v>
       </c>
       <c r="C256" s="4">
-        <v>23</v>
+        <v>2307</v>
       </c>
       <c r="D256" s="4">
-        <v>2302</v>
+        <v>23071</v>
       </c>
       <c r="E256" s="4"/>
       <c r="F256" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G256" s="5"/>
-      <c r="H256" s="5"/>
+        <v>55</v>
+      </c>
+      <c r="G256" s="5" t="s">
+        <v>319</v>
+      </c>
+      <c r="H256" s="4"/>
       <c r="I256" s="5" t="s">
-        <v>310</v>
+        <v>318</v>
       </c>
       <c r="J256" s="5"/>
     </row>
-    <row r="257" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="257" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A257" s="4">
-        <v>23021</v>
+        <v>23072</v>
       </c>
       <c r="B257" s="5" t="s">
-        <v>311</v>
+        <v>320</v>
       </c>
       <c r="C257" s="4">
-        <v>2302</v>
+        <v>2307</v>
       </c>
       <c r="D257" s="4">
-        <v>23021</v>
+        <v>23072</v>
       </c>
       <c r="E257" s="4"/>
       <c r="F257" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G257" s="5" t="s">
-        <v>312</v>
+        <v>321</v>
       </c>
       <c r="H257" s="5"/>
       <c r="I257" s="5" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="J257" s="5"/>
     </row>
-    <row r="258" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="258" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A258" s="4">
-        <v>23022</v>
+        <v>23073</v>
       </c>
       <c r="B258" s="5" t="s">
-        <v>314</v>
+        <v>322</v>
       </c>
       <c r="C258" s="4">
-        <v>2302</v>
+        <v>2307</v>
       </c>
       <c r="D258" s="4">
-        <v>23022</v>
+        <v>23073</v>
       </c>
       <c r="E258" s="4"/>
       <c r="F258" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G258" s="5" t="s">
-        <v>315</v>
+        <v>323</v>
       </c>
       <c r="H258" s="5"/>
       <c r="I258" s="5" t="s">
-        <v>316</v>
+        <v>322</v>
       </c>
       <c r="J258" s="5"/>
     </row>
-    <row r="259" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="259" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A259" s="4">
-        <v>2303</v>
+        <v>24</v>
       </c>
       <c r="B259" s="5" t="s">
-        <v>272</v>
+        <v>324</v>
       </c>
       <c r="C259" s="4">
-        <v>23</v>
+        <v>2</v>
       </c>
       <c r="D259" s="4">
-        <v>2303</v>
-      </c>
-      <c r="E259" s="4"/>
+        <v>24</v>
+      </c>
+      <c r="E259" s="5"/>
       <c r="F259" s="4" t="s">
         <v>52</v>
       </c>
       <c r="G259" s="5"/>
       <c r="H259" s="5"/>
       <c r="I259" s="5" t="s">
-        <v>272</v>
+        <v>324</v>
       </c>
       <c r="J259" s="5"/>
     </row>
-    <row r="260" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="260" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A260" s="4">
-        <v>23031</v>
+        <v>2401</v>
       </c>
       <c r="B260" s="5" t="s">
-        <v>317</v>
+        <v>325</v>
       </c>
       <c r="C260" s="4">
-        <v>2303</v>
+        <v>24</v>
       </c>
       <c r="D260" s="4">
-        <v>23031</v>
-      </c>
-      <c r="E260" s="4"/>
+        <v>2401</v>
+      </c>
+      <c r="E260" s="5"/>
       <c r="F260" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G260" s="5" t="s">
-        <v>318</v>
+        <v>326</v>
       </c>
       <c r="H260" s="5"/>
       <c r="I260" s="5" t="s">
-        <v>317</v>
+        <v>327</v>
       </c>
       <c r="J260" s="5"/>
     </row>
-    <row r="261" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="261" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A261" s="4">
-        <v>23032</v>
+        <v>2402</v>
       </c>
       <c r="B261" s="5" t="s">
-        <v>319</v>
+        <v>328</v>
       </c>
       <c r="C261" s="4">
-        <v>2303</v>
+        <v>24</v>
       </c>
       <c r="D261" s="4">
-        <v>23032</v>
+        <v>2402</v>
       </c>
       <c r="E261" s="4"/>
       <c r="F261" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G261" s="5" t="s">
-        <v>320</v>
-      </c>
-      <c r="H261" s="5"/>
+        <v>329</v>
+      </c>
+      <c r="H261" s="4"/>
       <c r="I261" s="5" t="s">
-        <v>319</v>
+        <v>328</v>
       </c>
       <c r="J261" s="5"/>
     </row>
-    <row r="262" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="262" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A262" s="4">
-        <v>23033</v>
+        <v>2403</v>
       </c>
       <c r="B262" s="5" t="s">
-        <v>321</v>
+        <v>330</v>
       </c>
       <c r="C262" s="4">
-        <v>2303</v>
+        <v>24</v>
       </c>
       <c r="D262" s="4">
-        <v>23033</v>
+        <v>2403</v>
       </c>
       <c r="E262" s="4"/>
       <c r="F262" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="G262" s="5" t="s">
-        <v>322</v>
-      </c>
-      <c r="H262" s="5"/>
-      <c r="I262" s="5" t="s">
-        <v>321</v>
-      </c>
-      <c r="J262" s="5"/>
-    </row>
-    <row r="263" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="G262" s="5"/>
+      <c r="H262" s="1"/>
+      <c r="I262" s="1" t="s">
+        <v>330</v>
+      </c>
+      <c r="J262" s="1" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="263" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A263" s="4">
-        <v>23034</v>
-      </c>
-      <c r="B263" s="12" t="s">
-        <v>355</v>
+        <v>25</v>
+      </c>
+      <c r="B263" s="5" t="s">
+        <v>331</v>
       </c>
       <c r="C263" s="4">
-        <v>2303</v>
+        <v>2</v>
       </c>
       <c r="D263" s="4">
-        <v>23034</v>
+        <v>25</v>
       </c>
       <c r="E263" s="4"/>
       <c r="F263" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G263" s="12" t="s">
-        <v>358</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G263" s="5"/>
       <c r="H263" s="5"/>
-      <c r="I263" s="12" t="s">
-        <v>355</v>
+      <c r="I263" s="5" t="s">
+        <v>331</v>
       </c>
       <c r="J263" s="5"/>
     </row>
-    <row r="264" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="264" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A264" s="4">
-        <v>23035</v>
+        <v>2501</v>
       </c>
       <c r="B264" s="5" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
       <c r="C264" s="4">
-        <v>2303</v>
+        <v>25</v>
       </c>
       <c r="D264" s="4">
-        <v>23035</v>
-      </c>
-      <c r="E264" s="4"/>
+        <v>2501</v>
+      </c>
+      <c r="E264" s="5"/>
       <c r="F264" s="4" t="s">
         <v>55</v>
       </c>
       <c r="G264" s="5" t="s">
-        <v>324</v>
+        <v>333</v>
       </c>
       <c r="H264" s="5"/>
       <c r="I264" s="5" t="s">
-        <v>323</v>
+        <v>332</v>
       </c>
       <c r="J264" s="5"/>
-    </row>
-    <row r="265" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A265" s="4">
-        <v>23036</v>
-      </c>
-      <c r="B265" s="12" t="s">
-        <v>356</v>
-      </c>
-      <c r="C265" s="4">
-        <v>2303</v>
-      </c>
-      <c r="D265" s="4">
-        <v>23036</v>
-      </c>
-      <c r="E265" s="4"/>
-      <c r="F265" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G265" s="12" t="s">
-        <v>357</v>
-      </c>
-      <c r="H265" s="5"/>
-      <c r="I265" s="12" t="s">
-        <v>356</v>
-      </c>
-      <c r="J265" s="5"/>
-    </row>
-    <row r="266" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A266" s="4">
-        <v>2304</v>
-      </c>
-      <c r="B266" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="C266" s="4">
-        <v>23</v>
-      </c>
-      <c r="D266" s="4">
-        <v>2304</v>
-      </c>
-      <c r="E266" s="4"/>
-      <c r="F266" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G266" s="5"/>
-      <c r="H266" s="5"/>
-      <c r="I266" s="5" t="s">
-        <v>325</v>
-      </c>
-      <c r="J266" s="5"/>
-    </row>
-    <row r="267" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A267" s="4">
-        <v>23041</v>
-      </c>
-      <c r="B267" s="5" t="s">
-        <v>326</v>
-      </c>
-      <c r="C267" s="4">
-        <v>2304</v>
-      </c>
-      <c r="D267" s="4">
-        <v>23041</v>
-      </c>
-      <c r="E267" s="4"/>
-      <c r="F267" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G267" s="5" t="s">
-        <v>327</v>
-      </c>
-      <c r="H267" s="5"/>
-      <c r="I267" s="5" t="s">
-        <v>326</v>
-      </c>
-      <c r="J267" s="5"/>
-    </row>
-    <row r="268" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A268" s="4">
-        <v>2305</v>
-      </c>
-      <c r="B268" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="C268" s="4">
-        <v>23</v>
-      </c>
-      <c r="D268" s="4">
-        <v>2305</v>
-      </c>
-      <c r="E268" s="4"/>
-      <c r="F268" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G268" s="5"/>
-      <c r="H268" s="5"/>
-      <c r="I268" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="J268" s="5"/>
-    </row>
-    <row r="269" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A269" s="4">
-        <v>23051</v>
-      </c>
-      <c r="B269" s="5" t="s">
-        <v>328</v>
-      </c>
-      <c r="C269" s="4">
-        <v>2305</v>
-      </c>
-      <c r="D269" s="4">
-        <v>23051</v>
-      </c>
-      <c r="E269" s="4"/>
-      <c r="F269" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G269" s="5" t="s">
-        <v>329</v>
-      </c>
-      <c r="H269" s="5"/>
-      <c r="I269" s="5" t="s">
-        <v>328</v>
-      </c>
-      <c r="J269" s="5"/>
-    </row>
-    <row r="270" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A270" s="4">
-        <v>2306</v>
-      </c>
-      <c r="B270" s="5" t="s">
-        <v>330</v>
-      </c>
-      <c r="C270" s="4">
-        <v>23</v>
-      </c>
-      <c r="D270" s="4">
-        <v>2306</v>
-      </c>
-      <c r="E270" s="4"/>
-      <c r="F270" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G270" s="5"/>
-      <c r="H270" s="5"/>
-      <c r="I270" s="5" t="s">
-        <v>330</v>
-      </c>
-      <c r="J270" s="5"/>
-    </row>
-    <row r="271" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A271" s="4">
-        <v>23061</v>
-      </c>
-      <c r="B271" s="5" t="s">
-        <v>331</v>
-      </c>
-      <c r="C271" s="4">
-        <v>2306</v>
-      </c>
-      <c r="D271" s="4">
-        <v>23061</v>
-      </c>
-      <c r="E271" s="4"/>
-      <c r="F271" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G271" s="5" t="s">
-        <v>332</v>
-      </c>
-      <c r="H271" s="5"/>
-      <c r="I271" s="5" t="s">
-        <v>331</v>
-      </c>
-      <c r="J271" s="5"/>
-    </row>
-    <row r="272" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A272" s="4">
-        <v>23062</v>
-      </c>
-      <c r="B272" s="5" t="s">
-        <v>333</v>
-      </c>
-      <c r="C272" s="4">
-        <v>2306</v>
-      </c>
-      <c r="D272" s="4">
-        <v>23062</v>
-      </c>
-      <c r="E272" s="4"/>
-      <c r="F272" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G272" s="5" t="s">
-        <v>334</v>
-      </c>
-      <c r="H272" s="5"/>
-      <c r="I272" s="5" t="s">
-        <v>333</v>
-      </c>
-      <c r="J272" s="5"/>
-    </row>
-    <row r="273" spans="1:10" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A273" s="4">
-        <v>23063</v>
-      </c>
-      <c r="B273" s="5" t="s">
-        <v>335</v>
-      </c>
-      <c r="C273" s="4">
-        <v>2306</v>
-      </c>
-      <c r="D273" s="4">
-        <v>23063</v>
-      </c>
-      <c r="E273" s="4"/>
-      <c r="F273" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G273" s="5" t="s">
-        <v>336</v>
-      </c>
-      <c r="H273" s="5"/>
-      <c r="I273" s="5" t="s">
-        <v>337</v>
-      </c>
-      <c r="J273" s="5"/>
-    </row>
-    <row r="274" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A274" s="4">
-        <v>2307</v>
-      </c>
-      <c r="B274" s="5" t="s">
-        <v>338</v>
-      </c>
-      <c r="C274" s="4">
-        <v>23</v>
-      </c>
-      <c r="D274" s="4">
-        <v>2307</v>
-      </c>
-      <c r="E274" s="4"/>
-      <c r="F274" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G274" s="4"/>
-      <c r="H274" s="4"/>
-      <c r="I274" s="5" t="s">
-        <v>338</v>
-      </c>
-      <c r="J274" s="5"/>
-    </row>
-    <row r="275" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A275" s="4">
-        <v>23071</v>
-      </c>
-      <c r="B275" s="5" t="s">
-        <v>339</v>
-      </c>
-      <c r="C275" s="4">
-        <v>2307</v>
-      </c>
-      <c r="D275" s="4">
-        <v>23071</v>
-      </c>
-      <c r="E275" s="4"/>
-      <c r="F275" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G275" s="5" t="s">
-        <v>340</v>
-      </c>
-      <c r="H275" s="4"/>
-      <c r="I275" s="5" t="s">
-        <v>339</v>
-      </c>
-      <c r="J275" s="5"/>
-    </row>
-    <row r="276" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A276" s="4">
-        <v>23072</v>
-      </c>
-      <c r="B276" s="5" t="s">
-        <v>341</v>
-      </c>
-      <c r="C276" s="4">
-        <v>2307</v>
-      </c>
-      <c r="D276" s="4">
-        <v>23072</v>
-      </c>
-      <c r="E276" s="4"/>
-      <c r="F276" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G276" s="5" t="s">
-        <v>342</v>
-      </c>
-      <c r="H276" s="5"/>
-      <c r="I276" s="5" t="s">
-        <v>341</v>
-      </c>
-      <c r="J276" s="5"/>
-    </row>
-    <row r="277" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A277" s="4">
-        <v>23073</v>
-      </c>
-      <c r="B277" s="5" t="s">
-        <v>343</v>
-      </c>
-      <c r="C277" s="4">
-        <v>2307</v>
-      </c>
-      <c r="D277" s="4">
-        <v>23073</v>
-      </c>
-      <c r="E277" s="4"/>
-      <c r="F277" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G277" s="5" t="s">
-        <v>344</v>
-      </c>
-      <c r="H277" s="5"/>
-      <c r="I277" s="5" t="s">
-        <v>343</v>
-      </c>
-      <c r="J277" s="5"/>
-    </row>
-    <row r="278" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A278" s="4">
-        <v>24</v>
-      </c>
-      <c r="B278" s="5" t="s">
-        <v>345</v>
-      </c>
-      <c r="C278" s="4">
-        <v>2</v>
-      </c>
-      <c r="D278" s="4">
-        <v>24</v>
-      </c>
-      <c r="E278" s="5"/>
-      <c r="F278" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G278" s="5"/>
-      <c r="H278" s="5"/>
-      <c r="I278" s="5" t="s">
-        <v>345</v>
-      </c>
-      <c r="J278" s="5"/>
-    </row>
-    <row r="279" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A279" s="4">
-        <v>2401</v>
-      </c>
-      <c r="B279" s="5" t="s">
-        <v>346</v>
-      </c>
-      <c r="C279" s="4">
-        <v>24</v>
-      </c>
-      <c r="D279" s="4">
-        <v>2401</v>
-      </c>
-      <c r="E279" s="5"/>
-      <c r="F279" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G279" s="5" t="s">
-        <v>347</v>
-      </c>
-      <c r="H279" s="5"/>
-      <c r="I279" s="5" t="s">
-        <v>348</v>
-      </c>
-      <c r="J279" s="5"/>
-    </row>
-    <row r="280" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A280" s="4">
-        <v>2402</v>
-      </c>
-      <c r="B280" s="5" t="s">
-        <v>349</v>
-      </c>
-      <c r="C280" s="4">
-        <v>24</v>
-      </c>
-      <c r="D280" s="4">
-        <v>2402</v>
-      </c>
-      <c r="E280" s="4"/>
-      <c r="F280" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G280" s="5" t="s">
-        <v>350</v>
-      </c>
-      <c r="H280" s="4"/>
-      <c r="I280" s="5" t="s">
-        <v>349</v>
-      </c>
-      <c r="J280" s="5"/>
-    </row>
-    <row r="281" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A281" s="4">
-        <v>2403</v>
-      </c>
-      <c r="B281" s="5" t="s">
-        <v>351</v>
-      </c>
-      <c r="C281" s="4">
-        <v>24</v>
-      </c>
-      <c r="D281" s="4">
-        <v>2403</v>
-      </c>
-      <c r="E281" s="4"/>
-      <c r="F281" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G281" s="5"/>
-      <c r="H281" s="1"/>
-      <c r="I281" s="1" t="s">
-        <v>351</v>
-      </c>
-      <c r="J281" s="1" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="282" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A282" s="4">
-        <v>25</v>
-      </c>
-      <c r="B282" s="5" t="s">
-        <v>352</v>
-      </c>
-      <c r="C282" s="4">
-        <v>2</v>
-      </c>
-      <c r="D282" s="4">
-        <v>25</v>
-      </c>
-      <c r="E282" s="4"/>
-      <c r="F282" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="G282" s="5"/>
-      <c r="H282" s="5"/>
-      <c r="I282" s="5" t="s">
-        <v>352</v>
-      </c>
-      <c r="J282" s="5"/>
-    </row>
-    <row r="283" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="A283" s="4">
-        <v>2501</v>
-      </c>
-      <c r="B283" s="5" t="s">
-        <v>353</v>
-      </c>
-      <c r="C283" s="4">
-        <v>25</v>
-      </c>
-      <c r="D283" s="4">
-        <v>2501</v>
-      </c>
-      <c r="E283" s="5"/>
-      <c r="F283" s="4" t="s">
-        <v>55</v>
-      </c>
-      <c r="G283" s="5" t="s">
-        <v>354</v>
-      </c>
-      <c r="H283" s="5"/>
-      <c r="I283" s="5" t="s">
-        <v>353</v>
-      </c>
-      <c r="J283" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="7" type="noConversion"/>

</xml_diff>

<commit_message>
#108 remove old ip
</commit_message>
<xml_diff>
--- a/Sources/Cuga-Calibration-Solution/Assets/Data/InitData.xlsx
+++ b/Sources/Cuga-Calibration-Solution/Assets/Data/InitData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\RiderProjects\semix\kaizhi.xuan\netcore_semix_cuga_calibration\Sources\Cuga-Calibration-Solution\Assets\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E635020B-A551-47D5-8166-B5BB867DCD27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F10CC0C6-780B-4B60-AC7F-51B8902B91E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" firstSheet="1" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" firstSheet="1" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SysUser" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1305" uniqueCount="351">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1305" uniqueCount="352">
   <si>
     <t>Id</t>
   </si>
@@ -824,9 +824,6 @@
   </si>
   <si>
     <t>Illumination Profile</t>
-  </si>
-  <si>
-    <t>CugaCalibration.ViewModels.Laser.LaserIlluminationProfileCalibrationViewModel</t>
   </si>
   <si>
     <t>CIB</t>
@@ -1168,6 +1165,14 @@
   </si>
   <si>
     <t>CugaCalibration.ViewModels.CIB.CIBXTCViewModel</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Uniformity</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>CugaCalibration.ViewModels.AOD.AODUniformityViewModel</t>
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
 </sst>
@@ -12857,7 +12862,7 @@
         <v>1309</v>
       </c>
       <c r="B202" s="1" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="C202" s="4">
         <v>13</v>
@@ -12870,11 +12875,11 @@
         <v>55</v>
       </c>
       <c r="G202" s="1" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="H202" s="1"/>
       <c r="I202" s="1" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="J202" s="5"/>
     </row>
@@ -13162,8 +13167,8 @@
       <c r="A214" s="4">
         <v>1504</v>
       </c>
-      <c r="B214" s="5" t="s">
-        <v>260</v>
+      <c r="B214" s="12" t="s">
+        <v>350</v>
       </c>
       <c r="C214" s="4">
         <v>15</v>
@@ -13175,12 +13180,12 @@
       <c r="F214" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="G214" s="5" t="s">
-        <v>261</v>
+      <c r="G214" s="12" t="s">
+        <v>351</v>
       </c>
       <c r="H214" s="5"/>
-      <c r="I214" s="5" t="s">
-        <v>260</v>
+      <c r="I214" s="12" t="s">
+        <v>350</v>
       </c>
       <c r="J214" s="5"/>
     </row>
@@ -13189,7 +13194,7 @@
         <v>16</v>
       </c>
       <c r="B215" s="5" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="C215" s="4">
         <v>1</v>
@@ -13204,7 +13209,7 @@
       <c r="G215" s="5"/>
       <c r="H215" s="5"/>
       <c r="I215" s="5" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="J215" s="5"/>
     </row>
@@ -13213,7 +13218,7 @@
         <v>1601</v>
       </c>
       <c r="B216" s="5" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="C216" s="4">
         <v>16</v>
@@ -13226,11 +13231,11 @@
         <v>55</v>
       </c>
       <c r="G216" s="5" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="H216" s="5"/>
       <c r="I216" s="5" t="s">
-        <v>263</v>
+        <v>262</v>
       </c>
       <c r="J216" s="5"/>
     </row>
@@ -13239,7 +13244,7 @@
         <v>1602</v>
       </c>
       <c r="B217" s="1" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="C217" s="4">
         <v>16</v>
@@ -13252,11 +13257,11 @@
         <v>55</v>
       </c>
       <c r="G217" s="12" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="H217" s="1"/>
       <c r="I217" s="1" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="J217" s="5"/>
     </row>
@@ -13265,7 +13270,7 @@
         <v>1603</v>
       </c>
       <c r="B218" s="5" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="C218" s="4">
         <v>16</v>
@@ -13278,11 +13283,11 @@
         <v>55</v>
       </c>
       <c r="G218" s="5" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="H218" s="5"/>
       <c r="I218" s="5" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="J218" s="5"/>
     </row>
@@ -13291,7 +13296,7 @@
         <v>1604</v>
       </c>
       <c r="B219" s="5" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C219" s="4">
         <v>16</v>
@@ -13304,11 +13309,11 @@
         <v>55</v>
       </c>
       <c r="G219" s="5" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="H219" s="5"/>
       <c r="I219" s="5" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="J219" s="5"/>
     </row>
@@ -13317,7 +13322,7 @@
         <v>1605</v>
       </c>
       <c r="B220" s="12" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="C220" s="4">
         <v>16</v>
@@ -13330,7 +13335,7 @@
         <v>55</v>
       </c>
       <c r="G220" s="12" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="H220" s="5"/>
       <c r="I220" s="5" t="s">
@@ -13343,7 +13348,7 @@
         <v>1606</v>
       </c>
       <c r="B221" s="12" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="C221" s="4">
         <v>16</v>
@@ -13356,11 +13361,11 @@
         <v>55</v>
       </c>
       <c r="G221" s="12" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="H221" s="5"/>
       <c r="I221" s="12" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="J221" s="5"/>
     </row>
@@ -13369,7 +13374,7 @@
         <v>1607</v>
       </c>
       <c r="B222" s="5" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C222" s="4">
         <v>16</v>
@@ -13382,11 +13387,11 @@
         <v>55</v>
       </c>
       <c r="G222" s="12" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="H222" s="5"/>
       <c r="I222" s="5" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="J222" s="5"/>
     </row>
@@ -13395,7 +13400,7 @@
         <v>1608</v>
       </c>
       <c r="B223" s="12" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="C223" s="4">
         <v>16</v>
@@ -13408,11 +13413,11 @@
         <v>55</v>
       </c>
       <c r="G223" s="12" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="H223" s="5"/>
       <c r="I223" s="12" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="J223" s="5"/>
     </row>
@@ -13421,7 +13426,7 @@
         <v>17</v>
       </c>
       <c r="B224" s="12" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C224" s="4">
         <v>1</v>
@@ -13436,7 +13441,7 @@
       <c r="G224" s="5"/>
       <c r="H224" s="5"/>
       <c r="I224" s="12" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="J224" s="5"/>
     </row>
@@ -13445,7 +13450,7 @@
         <v>1701</v>
       </c>
       <c r="B225" s="12" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C225" s="4">
         <v>17</v>
@@ -13458,11 +13463,11 @@
         <v>55</v>
       </c>
       <c r="G225" s="12" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="H225" s="5"/>
       <c r="I225" s="12" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="J225" s="5"/>
     </row>
@@ -13471,7 +13476,7 @@
         <v>1702</v>
       </c>
       <c r="B226" s="12" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="C226" s="4">
         <v>17</v>
@@ -13484,11 +13489,11 @@
         <v>55</v>
       </c>
       <c r="G226" s="12" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="H226" s="5"/>
       <c r="I226" s="12" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="J226" s="5"/>
     </row>
@@ -13497,7 +13502,7 @@
         <v>2</v>
       </c>
       <c r="B227" s="5" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="C227" s="4">
         <v>-1</v>
@@ -13512,7 +13517,7 @@
       <c r="G227" s="5"/>
       <c r="H227" s="5"/>
       <c r="I227" s="5" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="J227" s="5"/>
     </row>
@@ -13521,7 +13526,7 @@
         <v>21</v>
       </c>
       <c r="B228" s="5" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="C228" s="4">
         <v>2</v>
@@ -13536,7 +13541,7 @@
       <c r="G228" s="5"/>
       <c r="H228" s="5"/>
       <c r="I228" s="5" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="J228" s="5"/>
     </row>
@@ -13545,7 +13550,7 @@
         <v>2110</v>
       </c>
       <c r="B229" s="5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="C229" s="4">
         <v>21</v>
@@ -13558,11 +13563,11 @@
         <v>55</v>
       </c>
       <c r="G229" s="5" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
       <c r="H229" s="5"/>
       <c r="I229" s="5" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="J229" s="5"/>
     </row>
@@ -13571,7 +13576,7 @@
         <v>2111</v>
       </c>
       <c r="B230" s="5" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="C230" s="4">
         <v>21</v>
@@ -13584,11 +13589,11 @@
         <v>55</v>
       </c>
       <c r="G230" s="5" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="H230" s="5"/>
       <c r="I230" s="5" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="J230" s="5"/>
     </row>
@@ -13597,7 +13602,7 @@
         <v>22</v>
       </c>
       <c r="B231" s="5" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="C231" s="4">
         <v>2</v>
@@ -13612,7 +13617,7 @@
       <c r="G231" s="5"/>
       <c r="H231" s="5"/>
       <c r="I231" s="5" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="J231" s="5"/>
     </row>
@@ -13621,7 +13626,7 @@
         <v>2201</v>
       </c>
       <c r="B232" s="5" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="C232" s="4">
         <v>22</v>
@@ -13634,11 +13639,11 @@
         <v>55</v>
       </c>
       <c r="G232" s="5" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="H232" s="5"/>
       <c r="I232" s="5" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="J232" s="5"/>
     </row>
@@ -13647,7 +13652,7 @@
         <v>2202</v>
       </c>
       <c r="B233" s="5" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="C233" s="4">
         <v>22</v>
@@ -13660,11 +13665,11 @@
         <v>55</v>
       </c>
       <c r="G233" s="5" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="H233" s="5"/>
       <c r="I233" s="5" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="J233" s="5"/>
     </row>
@@ -13673,7 +13678,7 @@
         <v>2203</v>
       </c>
       <c r="B234" s="5" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C234" s="4">
         <v>22</v>
@@ -13686,11 +13691,11 @@
         <v>55</v>
       </c>
       <c r="G234" s="5" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="H234" s="5"/>
       <c r="I234" s="5" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="J234" s="5"/>
     </row>
@@ -13699,7 +13704,7 @@
         <v>23</v>
       </c>
       <c r="B235" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="C235" s="4">
         <v>2</v>
@@ -13714,7 +13719,7 @@
       <c r="G235" s="5"/>
       <c r="H235" s="5"/>
       <c r="I235" s="5" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="J235" s="5"/>
     </row>
@@ -13723,7 +13728,7 @@
         <v>2301</v>
       </c>
       <c r="B236" s="5" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="C236" s="4">
         <v>23</v>
@@ -13736,11 +13741,11 @@
         <v>55</v>
       </c>
       <c r="G236" s="5" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="H236" s="5"/>
       <c r="I236" s="5" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="J236" s="5"/>
     </row>
@@ -13749,7 +13754,7 @@
         <v>2302</v>
       </c>
       <c r="B237" s="5" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="C237" s="4">
         <v>23</v>
@@ -13764,7 +13769,7 @@
       <c r="G237" s="5"/>
       <c r="H237" s="5"/>
       <c r="I237" s="5" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="J237" s="5"/>
     </row>
@@ -13773,7 +13778,7 @@
         <v>23021</v>
       </c>
       <c r="B238" s="5" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C238" s="4">
         <v>2302</v>
@@ -13786,11 +13791,11 @@
         <v>55</v>
       </c>
       <c r="G238" s="5" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="H238" s="5"/>
       <c r="I238" s="5" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="J238" s="5"/>
     </row>
@@ -13799,7 +13804,7 @@
         <v>23022</v>
       </c>
       <c r="B239" s="5" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C239" s="4">
         <v>2302</v>
@@ -13812,11 +13817,11 @@
         <v>55</v>
       </c>
       <c r="G239" s="5" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="H239" s="5"/>
       <c r="I239" s="5" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="J239" s="5"/>
     </row>
@@ -13849,7 +13854,7 @@
         <v>23031</v>
       </c>
       <c r="B241" s="5" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C241" s="4">
         <v>2303</v>
@@ -13862,11 +13867,11 @@
         <v>55</v>
       </c>
       <c r="G241" s="5" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="H241" s="5"/>
       <c r="I241" s="5" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="J241" s="5"/>
     </row>
@@ -13875,7 +13880,7 @@
         <v>23032</v>
       </c>
       <c r="B242" s="5" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="C242" s="4">
         <v>2303</v>
@@ -13888,11 +13893,11 @@
         <v>55</v>
       </c>
       <c r="G242" s="5" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="H242" s="5"/>
       <c r="I242" s="5" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="J242" s="5"/>
     </row>
@@ -13901,7 +13906,7 @@
         <v>23033</v>
       </c>
       <c r="B243" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="C243" s="4">
         <v>2303</v>
@@ -13914,11 +13919,11 @@
         <v>55</v>
       </c>
       <c r="G243" s="5" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="H243" s="5"/>
       <c r="I243" s="5" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="J243" s="5"/>
     </row>
@@ -13927,7 +13932,7 @@
         <v>23034</v>
       </c>
       <c r="B244" s="12" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C244" s="4">
         <v>2303</v>
@@ -13940,11 +13945,11 @@
         <v>55</v>
       </c>
       <c r="G244" s="12" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="H244" s="5"/>
       <c r="I244" s="12" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="J244" s="5"/>
     </row>
@@ -13953,7 +13958,7 @@
         <v>23035</v>
       </c>
       <c r="B245" s="5" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="C245" s="4">
         <v>2303</v>
@@ -13966,11 +13971,11 @@
         <v>55</v>
       </c>
       <c r="G245" s="5" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="H245" s="5"/>
       <c r="I245" s="5" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="J245" s="5"/>
     </row>
@@ -13979,7 +13984,7 @@
         <v>23036</v>
       </c>
       <c r="B246" s="12" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C246" s="4">
         <v>2303</v>
@@ -13992,11 +13997,11 @@
         <v>55</v>
       </c>
       <c r="G246" s="12" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="H246" s="5"/>
       <c r="I246" s="12" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="J246" s="5"/>
     </row>
@@ -14005,7 +14010,7 @@
         <v>2304</v>
       </c>
       <c r="B247" s="5" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="C247" s="4">
         <v>23</v>
@@ -14020,7 +14025,7 @@
       <c r="G247" s="5"/>
       <c r="H247" s="5"/>
       <c r="I247" s="5" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="J247" s="5"/>
     </row>
@@ -14029,7 +14034,7 @@
         <v>23041</v>
       </c>
       <c r="B248" s="5" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="C248" s="4">
         <v>2304</v>
@@ -14042,11 +14047,11 @@
         <v>55</v>
       </c>
       <c r="G248" s="5" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="H248" s="5"/>
       <c r="I248" s="5" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="J248" s="5"/>
     </row>
@@ -14079,7 +14084,7 @@
         <v>23051</v>
       </c>
       <c r="B250" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="C250" s="4">
         <v>2305</v>
@@ -14092,11 +14097,11 @@
         <v>55</v>
       </c>
       <c r="G250" s="5" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="H250" s="5"/>
       <c r="I250" s="5" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="J250" s="5"/>
     </row>
@@ -14105,7 +14110,7 @@
         <v>2306</v>
       </c>
       <c r="B251" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="C251" s="4">
         <v>23</v>
@@ -14120,7 +14125,7 @@
       <c r="G251" s="5"/>
       <c r="H251" s="5"/>
       <c r="I251" s="5" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="J251" s="5"/>
     </row>
@@ -14129,7 +14134,7 @@
         <v>23061</v>
       </c>
       <c r="B252" s="5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="C252" s="4">
         <v>2306</v>
@@ -14142,11 +14147,11 @@
         <v>55</v>
       </c>
       <c r="G252" s="5" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="H252" s="5"/>
       <c r="I252" s="5" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="J252" s="5"/>
     </row>
@@ -14155,7 +14160,7 @@
         <v>23062</v>
       </c>
       <c r="B253" s="5" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="C253" s="4">
         <v>2306</v>
@@ -14168,11 +14173,11 @@
         <v>55</v>
       </c>
       <c r="G253" s="5" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="H253" s="5"/>
       <c r="I253" s="5" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="J253" s="5"/>
     </row>
@@ -14181,7 +14186,7 @@
         <v>23063</v>
       </c>
       <c r="B254" s="5" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="C254" s="4">
         <v>2306</v>
@@ -14194,11 +14199,11 @@
         <v>55</v>
       </c>
       <c r="G254" s="5" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="H254" s="5"/>
       <c r="I254" s="5" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="J254" s="5"/>
     </row>
@@ -14207,7 +14212,7 @@
         <v>2307</v>
       </c>
       <c r="B255" s="5" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C255" s="4">
         <v>23</v>
@@ -14222,7 +14227,7 @@
       <c r="G255" s="4"/>
       <c r="H255" s="4"/>
       <c r="I255" s="5" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="J255" s="5"/>
     </row>
@@ -14231,7 +14236,7 @@
         <v>23071</v>
       </c>
       <c r="B256" s="5" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C256" s="4">
         <v>2307</v>
@@ -14244,11 +14249,11 @@
         <v>55</v>
       </c>
       <c r="G256" s="5" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="H256" s="4"/>
       <c r="I256" s="5" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="J256" s="5"/>
     </row>
@@ -14257,7 +14262,7 @@
         <v>23072</v>
       </c>
       <c r="B257" s="5" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C257" s="4">
         <v>2307</v>
@@ -14270,11 +14275,11 @@
         <v>55</v>
       </c>
       <c r="G257" s="5" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="H257" s="5"/>
       <c r="I257" s="5" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="J257" s="5"/>
     </row>
@@ -14283,7 +14288,7 @@
         <v>23073</v>
       </c>
       <c r="B258" s="5" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="C258" s="4">
         <v>2307</v>
@@ -14296,11 +14301,11 @@
         <v>55</v>
       </c>
       <c r="G258" s="5" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="H258" s="5"/>
       <c r="I258" s="5" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="J258" s="5"/>
     </row>
@@ -14309,7 +14314,7 @@
         <v>24</v>
       </c>
       <c r="B259" s="5" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="C259" s="4">
         <v>2</v>
@@ -14324,7 +14329,7 @@
       <c r="G259" s="5"/>
       <c r="H259" s="5"/>
       <c r="I259" s="5" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="J259" s="5"/>
     </row>
@@ -14333,7 +14338,7 @@
         <v>2401</v>
       </c>
       <c r="B260" s="5" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="C260" s="4">
         <v>24</v>
@@ -14346,11 +14351,11 @@
         <v>55</v>
       </c>
       <c r="G260" s="5" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="H260" s="5"/>
       <c r="I260" s="5" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="J260" s="5"/>
     </row>
@@ -14359,7 +14364,7 @@
         <v>2402</v>
       </c>
       <c r="B261" s="5" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="C261" s="4">
         <v>24</v>
@@ -14372,11 +14377,11 @@
         <v>55</v>
       </c>
       <c r="G261" s="5" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="H261" s="4"/>
       <c r="I261" s="5" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="J261" s="5"/>
     </row>
@@ -14385,7 +14390,7 @@
         <v>2403</v>
       </c>
       <c r="B262" s="5" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="C262" s="4">
         <v>24</v>
@@ -14400,7 +14405,7 @@
       <c r="G262" s="5"/>
       <c r="H262" s="1"/>
       <c r="I262" s="1" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="J262" s="1" t="b">
         <v>1</v>
@@ -14411,7 +14416,7 @@
         <v>25</v>
       </c>
       <c r="B263" s="5" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="C263" s="4">
         <v>2</v>
@@ -14426,7 +14431,7 @@
       <c r="G263" s="5"/>
       <c r="H263" s="5"/>
       <c r="I263" s="5" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="J263" s="5"/>
     </row>
@@ -14435,7 +14440,7 @@
         <v>2501</v>
       </c>
       <c r="B264" s="5" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="C264" s="4">
         <v>25</v>
@@ -14448,11 +14453,11 @@
         <v>55</v>
       </c>
       <c r="G264" s="5" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="H264" s="5"/>
       <c r="I264" s="5" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="J264" s="5"/>
     </row>

</xml_diff>

<commit_message>
#146 BestFocus2.0 NISC OISC校准、#147 多光斑BestFocus诊断工具
</commit_message>
<xml_diff>
--- a/Sources/Cuga-Calibration-Solution/Assets/Data/InitData.xlsx
+++ b/Sources/Cuga-Calibration-Solution/Assets/Data/InitData.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\RiderProjects\semix\kaizhi.xuan\netcore_semix_cuga_calibration\Sources\Cuga-Calibration-Solution\Assets\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEF32DD2-F524-406A-8EBB-1FCBA9C8DD39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{568339CC-3490-4BBF-9955-9BB93A2D88B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SysUser" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="172">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="173">
   <si>
     <t>Id</t>
   </si>
@@ -505,24 +505,6 @@
     <t>Objective Y Angle</t>
   </si>
   <si>
-    <t>CugaCalibration.ViewModels.Common.Windows.Tools.Optics.OpticsObjectiveYAngleWindowViewModel</t>
-  </si>
-  <si>
-    <t>Grab And Template</t>
-  </si>
-  <si>
-    <t>Grabbing Dark Image</t>
-  </si>
-  <si>
-    <t>CugaCalibration.ViewModels.Common.Windows.Tools.GrabbingDarkImageWindowViewModel</t>
-  </si>
-  <si>
-    <t>Create Dark Image Template</t>
-  </si>
-  <si>
-    <t>CugaCalibration.ViewModels.Common.Windows.Tools.CreateDarkImageTemplateWindowViewModel</t>
-  </si>
-  <si>
     <t>Diagnosis</t>
   </si>
   <si>
@@ -604,6 +586,34 @@
   </si>
   <si>
     <t>Delay</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>SC</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>CugaCalibration.ViewModels.Optics.OpticsSCViewModel</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Best Focus</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>CugaCalibration.ViewModels.Common.Windows.Tools.Optics.OpticsObjectiveYAngleWindowViewModel</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>CugaCalibration.ViewModels.Common.Windows.Tools.Optics.OpticsBestFocusWindowViewModel</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>CugaCalibration.ViewModels.Common.Windows.Tools.Optics.OpticsGrabbingImageWindowViewModel</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Grabbing Image</t>
     <phoneticPr fontId="5" type="noConversion"/>
   </si>
 </sst>
@@ -1206,7 +1216,7 @@
   <sheetData>
     <row r="1" spans="1:9" ht="23.25" x14ac:dyDescent="0.2">
       <c r="A1" s="9" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
@@ -1238,17 +1248,17 @@
         <v>1</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="C2" s="6">
         <v>1</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="E2" s="6"/>
       <c r="F2" s="12" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="G2" s="6">
         <v>666666</v>
@@ -1257,7 +1267,7 @@
         <v>9</v>
       </c>
       <c r="I2" s="10" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
@@ -1265,17 +1275,17 @@
         <v>2</v>
       </c>
       <c r="B3" s="11" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="C3" s="7">
         <v>1</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="E3" s="7"/>
       <c r="F3" s="12" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="G3" s="6">
         <v>666666</v>
@@ -1284,7 +1294,7 @@
         <v>9</v>
       </c>
       <c r="I3" s="11" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
@@ -1292,17 +1302,17 @@
         <v>3</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="C4" s="7">
         <v>1</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="E4" s="7"/>
       <c r="F4" s="12" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="G4" s="6">
         <v>666666</v>
@@ -1311,7 +1321,7 @@
         <v>9</v>
       </c>
       <c r="I4" s="11" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
     </row>
     <row r="5" spans="1:9" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
@@ -2415,16 +2425,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="C2" s="10" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="D2" s="6">
         <v>0</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
@@ -2432,16 +2442,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="D3" s="6">
         <v>1</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
@@ -2449,16 +2459,16 @@
         <v>3</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="D4" s="7">
         <v>2</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
@@ -2689,7 +2699,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="C2" s="6" t="s">
         <v>21</v>
@@ -2698,7 +2708,7 @@
         <v>0</v>
       </c>
       <c r="E2" s="10" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
@@ -2706,7 +2716,7 @@
         <v>2</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="C3" s="6" t="s">
         <v>21</v>
@@ -2715,7 +2725,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
     </row>
     <row r="4" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
@@ -2723,7 +2733,7 @@
         <v>3</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
       <c r="C4" s="6" t="s">
         <v>21</v>
@@ -2732,7 +2742,7 @@
         <v>2</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>166</v>
+        <v>160</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.2">
@@ -3815,7 +3825,7 @@
         <v>1501</v>
       </c>
       <c r="B24" s="13" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="C24" s="3">
         <v>15</v>
@@ -3832,7 +3842,7 @@
       </c>
       <c r="H24" s="4"/>
       <c r="I24" s="13" t="s">
-        <v>170</v>
+        <v>164</v>
       </c>
       <c r="J24" s="4"/>
     </row>
@@ -3841,7 +3851,7 @@
         <v>1502</v>
       </c>
       <c r="B25" s="13" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="C25" s="3">
         <v>15</v>
@@ -3858,7 +3868,7 @@
       </c>
       <c r="H25" s="4"/>
       <c r="I25" s="13" t="s">
-        <v>171</v>
+        <v>165</v>
       </c>
       <c r="J25" s="4"/>
     </row>
@@ -4276,8 +4286,8 @@
       <c r="A42" s="3">
         <v>1801</v>
       </c>
-      <c r="B42" s="4" t="s">
-        <v>98</v>
+      <c r="B42" s="13" t="s">
+        <v>166</v>
       </c>
       <c r="C42" s="3">
         <v>18</v>
@@ -4289,12 +4299,12 @@
       <c r="F42" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="G42" s="4" t="s">
-        <v>99</v>
+      <c r="G42" s="13" t="s">
+        <v>167</v>
       </c>
       <c r="H42" s="4"/>
-      <c r="I42" s="4" t="s">
-        <v>98</v>
+      <c r="I42" s="13" t="s">
+        <v>166</v>
       </c>
       <c r="J42" s="4"/>
     </row>
@@ -4303,7 +4313,7 @@
         <v>1802</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C43" s="3">
         <v>18</v>
@@ -4316,11 +4326,11 @@
         <v>32</v>
       </c>
       <c r="G43" s="4" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="H43" s="4"/>
       <c r="I43" s="4" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="J43" s="4"/>
     </row>
@@ -4329,7 +4339,7 @@
         <v>1803</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C44" s="3">
         <v>18</v>
@@ -4342,11 +4352,11 @@
         <v>32</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="H44" s="4"/>
       <c r="I44" s="4" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="J44" s="4"/>
     </row>
@@ -4354,8 +4364,8 @@
       <c r="A45" s="3">
         <v>1804</v>
       </c>
-      <c r="B45" s="13" t="s">
-        <v>169</v>
+      <c r="B45" s="4" t="s">
+        <v>102</v>
       </c>
       <c r="C45" s="3">
         <v>18</v>
@@ -4367,51 +4377,53 @@
       <c r="F45" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="G45" s="13" t="s">
-        <v>168</v>
+      <c r="G45" s="4" t="s">
+        <v>103</v>
       </c>
       <c r="H45" s="4"/>
-      <c r="I45" s="13" t="s">
-        <v>169</v>
+      <c r="I45" s="4" t="s">
+        <v>102</v>
       </c>
       <c r="J45" s="4"/>
     </row>
     <row r="46" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="3">
-        <v>2</v>
-      </c>
-      <c r="B46" s="4" t="s">
-        <v>104</v>
+        <v>1805</v>
+      </c>
+      <c r="B46" s="13" t="s">
+        <v>163</v>
       </c>
       <c r="C46" s="3">
-        <v>-1</v>
+        <v>18</v>
       </c>
       <c r="D46" s="3">
-        <v>2</v>
+        <v>1805</v>
       </c>
       <c r="E46" s="3"/>
       <c r="F46" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G46" s="4"/>
+        <v>32</v>
+      </c>
+      <c r="G46" s="13" t="s">
+        <v>162</v>
+      </c>
       <c r="H46" s="4"/>
-      <c r="I46" s="4" t="s">
-        <v>104</v>
+      <c r="I46" s="13" t="s">
+        <v>163</v>
       </c>
       <c r="J46" s="4"/>
     </row>
     <row r="47" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="3">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C47" s="3">
+        <v>-1</v>
+      </c>
+      <c r="D47" s="3">
         <v>2</v>
-      </c>
-      <c r="D47" s="3">
-        <v>21</v>
       </c>
       <c r="E47" s="3"/>
       <c r="F47" s="3" t="s">
@@ -4420,100 +4432,98 @@
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
       <c r="I47" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="J47" s="4"/>
     </row>
     <row r="48" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="3">
-        <v>2110</v>
+        <v>21</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C48" s="3">
+        <v>2</v>
+      </c>
+      <c r="D48" s="3">
         <v>21</v>
-      </c>
-      <c r="D48" s="3">
-        <v>2110</v>
       </c>
       <c r="E48" s="3"/>
       <c r="F48" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G48" s="4" t="s">
-        <v>107</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="G48" s="4"/>
       <c r="H48" s="4"/>
       <c r="I48" s="4" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="J48" s="4"/>
     </row>
     <row r="49" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="3">
-        <v>2111</v>
+        <v>2110</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C49" s="3">
         <v>21</v>
       </c>
       <c r="D49" s="3">
-        <v>2111</v>
+        <v>2110</v>
       </c>
       <c r="E49" s="3"/>
       <c r="F49" s="3" t="s">
         <v>32</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="H49" s="4"/>
       <c r="I49" s="4" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="J49" s="4"/>
     </row>
     <row r="50" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="3">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C50" s="3">
         <v>21</v>
       </c>
       <c r="D50" s="3">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="E50" s="3"/>
       <c r="F50" s="3" t="s">
         <v>32</v>
       </c>
       <c r="G50" s="4" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="H50" s="4"/>
       <c r="I50" s="4" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="J50" s="4"/>
     </row>
     <row r="51" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="3">
-        <v>2113</v>
+        <v>2112</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C51" s="3">
         <v>21</v>
       </c>
       <c r="D51" s="3">
-        <v>2113</v>
+        <v>2112</v>
       </c>
       <c r="E51" s="3"/>
       <c r="F51" s="3" t="s">
@@ -4524,565 +4534,567 @@
       </c>
       <c r="H51" s="4"/>
       <c r="I51" s="4" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="J51" s="4"/>
     </row>
     <row r="52" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="3">
-        <v>22</v>
+        <v>2113</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C52" s="3">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="D52" s="3">
-        <v>22</v>
+        <v>2113</v>
       </c>
       <c r="E52" s="3"/>
       <c r="F52" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G52" s="4"/>
+        <v>32</v>
+      </c>
+      <c r="G52" s="4" t="s">
+        <v>107</v>
+      </c>
       <c r="H52" s="4"/>
       <c r="I52" s="4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="J52" s="4"/>
     </row>
     <row r="53" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="3">
-        <v>2201</v>
+        <v>22</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C53" s="3">
+        <v>2</v>
+      </c>
+      <c r="D53" s="3">
         <v>22</v>
-      </c>
-      <c r="D53" s="3">
-        <v>2201</v>
       </c>
       <c r="E53" s="3"/>
       <c r="F53" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G53" s="4" t="s">
-        <v>114</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="G53" s="4"/>
       <c r="H53" s="4"/>
       <c r="I53" s="4" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="J53" s="4"/>
     </row>
     <row r="54" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="3">
-        <v>2202</v>
+        <v>2201</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C54" s="3">
         <v>22</v>
       </c>
       <c r="D54" s="3">
-        <v>2202</v>
+        <v>2201</v>
       </c>
       <c r="E54" s="3"/>
       <c r="F54" s="3" t="s">
         <v>32</v>
       </c>
       <c r="G54" s="4" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="H54" s="4"/>
       <c r="I54" s="4" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="J54" s="4"/>
     </row>
     <row r="55" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="3">
-        <v>2203</v>
+        <v>2202</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C55" s="3">
         <v>22</v>
       </c>
       <c r="D55" s="3">
-        <v>2203</v>
+        <v>2202</v>
       </c>
       <c r="E55" s="3"/>
       <c r="F55" s="3" t="s">
         <v>32</v>
       </c>
       <c r="G55" s="4" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="H55" s="4"/>
       <c r="I55" s="4" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="J55" s="4"/>
     </row>
     <row r="56" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="3">
-        <v>23</v>
+        <v>2203</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C56" s="3">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D56" s="3">
-        <v>23</v>
+        <v>2203</v>
       </c>
       <c r="E56" s="3"/>
       <c r="F56" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G56" s="4"/>
+        <v>32</v>
+      </c>
+      <c r="G56" s="4" t="s">
+        <v>118</v>
+      </c>
       <c r="H56" s="4"/>
       <c r="I56" s="4" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="J56" s="4"/>
     </row>
     <row r="57" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="3">
-        <v>2301</v>
+        <v>23</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C57" s="3">
+        <v>2</v>
+      </c>
+      <c r="D57" s="3">
         <v>23</v>
-      </c>
-      <c r="D57" s="3">
-        <v>2301</v>
       </c>
       <c r="E57" s="3"/>
       <c r="F57" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G57" s="4" t="s">
-        <v>121</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="G57" s="4"/>
       <c r="H57" s="4"/>
       <c r="I57" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="J57" s="4"/>
     </row>
     <row r="58" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="3">
-        <v>2302</v>
+        <v>2301</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C58" s="3">
         <v>23</v>
       </c>
       <c r="D58" s="3">
-        <v>2302</v>
+        <v>2301</v>
       </c>
       <c r="E58" s="3"/>
       <c r="F58" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G58" s="4"/>
+        <v>32</v>
+      </c>
+      <c r="G58" s="4" t="s">
+        <v>121</v>
+      </c>
       <c r="H58" s="4"/>
       <c r="I58" s="4" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="J58" s="4"/>
     </row>
     <row r="59" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="3">
-        <v>23021</v>
+        <v>2302</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C59" s="3">
+        <v>23</v>
+      </c>
+      <c r="D59" s="3">
         <v>2302</v>
-      </c>
-      <c r="D59" s="3">
-        <v>23021</v>
       </c>
       <c r="E59" s="3"/>
       <c r="F59" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G59" s="4" t="s">
-        <v>124</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="G59" s="4"/>
       <c r="H59" s="4"/>
       <c r="I59" s="4" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="J59" s="4"/>
     </row>
     <row r="60" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="3">
-        <v>23022</v>
+        <v>23021</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C60" s="3">
         <v>2302</v>
       </c>
       <c r="D60" s="3">
-        <v>23022</v>
+        <v>23021</v>
       </c>
       <c r="E60" s="3"/>
       <c r="F60" s="3" t="s">
         <v>32</v>
       </c>
       <c r="G60" s="4" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="H60" s="4"/>
       <c r="I60" s="4" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="J60" s="4"/>
     </row>
     <row r="61" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="3">
-        <v>2303</v>
+        <v>23022</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>67</v>
+        <v>125</v>
       </c>
       <c r="C61" s="3">
-        <v>23</v>
+        <v>2302</v>
       </c>
       <c r="D61" s="3">
-        <v>2303</v>
+        <v>23022</v>
       </c>
       <c r="E61" s="3"/>
       <c r="F61" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G61" s="4"/>
+        <v>32</v>
+      </c>
+      <c r="G61" s="4" t="s">
+        <v>126</v>
+      </c>
       <c r="H61" s="4"/>
       <c r="I61" s="4" t="s">
-        <v>67</v>
+        <v>125</v>
       </c>
       <c r="J61" s="4"/>
     </row>
     <row r="62" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="3">
-        <v>23031</v>
+        <v>2303</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>127</v>
+        <v>67</v>
       </c>
       <c r="C62" s="3">
+        <v>23</v>
+      </c>
+      <c r="D62" s="3">
         <v>2303</v>
-      </c>
-      <c r="D62" s="3">
-        <v>23031</v>
       </c>
       <c r="E62" s="3"/>
       <c r="F62" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G62" s="4" t="s">
-        <v>128</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="G62" s="4"/>
       <c r="H62" s="4"/>
       <c r="I62" s="4" t="s">
-        <v>127</v>
+        <v>67</v>
       </c>
       <c r="J62" s="4"/>
     </row>
     <row r="63" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="3">
-        <v>23032</v>
+        <v>23031</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C63" s="3">
         <v>2303</v>
       </c>
       <c r="D63" s="3">
-        <v>23032</v>
+        <v>23031</v>
       </c>
       <c r="E63" s="3"/>
       <c r="F63" s="3" t="s">
         <v>32</v>
       </c>
       <c r="G63" s="4" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="H63" s="4"/>
       <c r="I63" s="4" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="J63" s="4"/>
     </row>
     <row r="64" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="3">
-        <v>23033</v>
+        <v>23032</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C64" s="3">
         <v>2303</v>
       </c>
       <c r="D64" s="3">
-        <v>23033</v>
+        <v>23032</v>
       </c>
       <c r="E64" s="3"/>
       <c r="F64" s="3" t="s">
         <v>32</v>
       </c>
       <c r="G64" s="4" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="H64" s="4"/>
       <c r="I64" s="4" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="J64" s="4"/>
     </row>
     <row r="65" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="3">
-        <v>23034</v>
+        <v>23033</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C65" s="3">
         <v>2303</v>
       </c>
       <c r="D65" s="3">
-        <v>23034</v>
+        <v>23033</v>
       </c>
       <c r="E65" s="3"/>
       <c r="F65" s="3" t="s">
         <v>32</v>
       </c>
       <c r="G65" s="4" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="H65" s="4"/>
       <c r="I65" s="4" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="J65" s="4"/>
     </row>
     <row r="66" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="3">
-        <v>23035</v>
+        <v>23034</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C66" s="3">
         <v>2303</v>
       </c>
       <c r="D66" s="3">
-        <v>23035</v>
+        <v>23034</v>
       </c>
       <c r="E66" s="3"/>
       <c r="F66" s="3" t="s">
         <v>32</v>
       </c>
       <c r="G66" s="4" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="H66" s="4"/>
       <c r="I66" s="4" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="J66" s="4"/>
     </row>
     <row r="67" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="3">
-        <v>2304</v>
+        <v>23035</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="C67" s="3">
-        <v>23</v>
+        <v>2303</v>
       </c>
       <c r="D67" s="3">
-        <v>2304</v>
+        <v>23035</v>
       </c>
       <c r="E67" s="3"/>
       <c r="F67" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G67" s="4"/>
+        <v>32</v>
+      </c>
+      <c r="G67" s="4" t="s">
+        <v>136</v>
+      </c>
       <c r="H67" s="4"/>
       <c r="I67" s="4" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="J67" s="4"/>
     </row>
     <row r="68" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="3">
-        <v>23041</v>
+        <v>2304</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="C68" s="3">
+        <v>23</v>
+      </c>
+      <c r="D68" s="3">
         <v>2304</v>
-      </c>
-      <c r="D68" s="3">
-        <v>23041</v>
       </c>
       <c r="E68" s="3"/>
       <c r="F68" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G68" s="4" t="s">
-        <v>139</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="G68" s="4"/>
       <c r="H68" s="4"/>
       <c r="I68" s="4" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="J68" s="4"/>
     </row>
     <row r="69" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="3">
-        <v>2305</v>
+        <v>23041</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>18</v>
+        <v>138</v>
       </c>
       <c r="C69" s="3">
-        <v>23</v>
+        <v>2304</v>
       </c>
       <c r="D69" s="3">
-        <v>2305</v>
+        <v>23041</v>
       </c>
       <c r="E69" s="3"/>
       <c r="F69" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G69" s="4"/>
+        <v>32</v>
+      </c>
+      <c r="G69" s="4" t="s">
+        <v>139</v>
+      </c>
       <c r="H69" s="4"/>
       <c r="I69" s="4" t="s">
-        <v>18</v>
+        <v>138</v>
       </c>
       <c r="J69" s="4"/>
     </row>
     <row r="70" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="3">
-        <v>23051</v>
+        <v>2305</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>140</v>
+        <v>18</v>
       </c>
       <c r="C70" s="3">
+        <v>23</v>
+      </c>
+      <c r="D70" s="3">
         <v>2305</v>
-      </c>
-      <c r="D70" s="3">
-        <v>23051</v>
       </c>
       <c r="E70" s="3"/>
       <c r="F70" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G70" s="4" t="s">
-        <v>141</v>
-      </c>
+        <v>29</v>
+      </c>
+      <c r="G70" s="4"/>
       <c r="H70" s="4"/>
       <c r="I70" s="4" t="s">
-        <v>140</v>
+        <v>18</v>
       </c>
       <c r="J70" s="4"/>
     </row>
     <row r="71" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="3">
-        <v>2306</v>
+        <v>23051</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C71" s="3">
-        <v>23</v>
+        <v>2305</v>
       </c>
       <c r="D71" s="3">
-        <v>2306</v>
+        <v>23051</v>
       </c>
       <c r="E71" s="3"/>
       <c r="F71" s="3" t="s">
-        <v>29</v>
-      </c>
-      <c r="G71" s="4"/>
+        <v>32</v>
+      </c>
+      <c r="G71" s="13" t="s">
+        <v>169</v>
+      </c>
       <c r="H71" s="4"/>
       <c r="I71" s="4" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="J71" s="4"/>
     </row>
     <row r="72" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="3">
-        <v>23061</v>
-      </c>
-      <c r="B72" s="4" t="s">
-        <v>143</v>
+        <v>23052</v>
+      </c>
+      <c r="B72" s="13" t="s">
+        <v>172</v>
       </c>
       <c r="C72" s="3">
-        <v>2306</v>
+        <v>2305</v>
       </c>
       <c r="D72" s="3">
-        <v>23061</v>
+        <v>23052</v>
       </c>
       <c r="E72" s="3"/>
       <c r="F72" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="G72" s="4" t="s">
-        <v>144</v>
+      <c r="G72" s="13" t="s">
+        <v>171</v>
       </c>
       <c r="H72" s="4"/>
-      <c r="I72" s="4" t="s">
-        <v>143</v>
+      <c r="I72" s="13" t="s">
+        <v>172</v>
       </c>
       <c r="J72" s="4"/>
     </row>
     <row r="73" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="3">
-        <v>23062</v>
-      </c>
-      <c r="B73" s="4" t="s">
-        <v>145</v>
+        <v>23053</v>
+      </c>
+      <c r="B73" s="13" t="s">
+        <v>168</v>
       </c>
       <c r="C73" s="3">
-        <v>2306</v>
+        <v>2305</v>
       </c>
       <c r="D73" s="3">
-        <v>23062</v>
+        <v>23053</v>
       </c>
       <c r="E73" s="3"/>
       <c r="F73" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="G73" s="4" t="s">
-        <v>146</v>
+      <c r="G73" s="13" t="s">
+        <v>170</v>
       </c>
       <c r="H73" s="4"/>
-      <c r="I73" s="4" t="s">
-        <v>145</v>
+      <c r="I73" s="13" t="s">
+        <v>168</v>
       </c>
       <c r="J73" s="4"/>
     </row>
@@ -5091,7 +5103,7 @@
         <v>2307</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="C74" s="3">
         <v>23</v>
@@ -5106,7 +5118,7 @@
       <c r="G74" s="3"/>
       <c r="H74" s="3"/>
       <c r="I74" s="4" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="J74" s="4"/>
     </row>
@@ -5115,7 +5127,7 @@
         <v>23071</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="C75" s="3">
         <v>2307</v>
@@ -5128,11 +5140,11 @@
         <v>32</v>
       </c>
       <c r="G75" s="4" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="H75" s="3"/>
       <c r="I75" s="4" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="J75" s="4"/>
     </row>
@@ -5141,7 +5153,7 @@
         <v>23072</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="C76" s="3">
         <v>2307</v>
@@ -5154,11 +5166,11 @@
         <v>32</v>
       </c>
       <c r="G76" s="4" t="s">
-        <v>151</v>
+        <v>145</v>
       </c>
       <c r="H76" s="4"/>
       <c r="I76" s="4" t="s">
-        <v>150</v>
+        <v>144</v>
       </c>
       <c r="J76" s="4"/>
     </row>
@@ -5167,7 +5179,7 @@
         <v>23073</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="C77" s="3">
         <v>2307</v>
@@ -5180,11 +5192,11 @@
         <v>32</v>
       </c>
       <c r="G77" s="4" t="s">
-        <v>153</v>
+        <v>147</v>
       </c>
       <c r="H77" s="4"/>
       <c r="I77" s="4" t="s">
-        <v>152</v>
+        <v>146</v>
       </c>
       <c r="J77" s="4"/>
     </row>
@@ -5193,7 +5205,7 @@
         <v>24</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="C78" s="3">
         <v>2</v>
@@ -5208,7 +5220,7 @@
       <c r="G78" s="4"/>
       <c r="H78" s="4"/>
       <c r="I78" s="4" t="s">
-        <v>154</v>
+        <v>148</v>
       </c>
       <c r="J78" s="4"/>
     </row>
@@ -5217,7 +5229,7 @@
         <v>2401</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="C79" s="3">
         <v>24</v>
@@ -5230,11 +5242,11 @@
         <v>32</v>
       </c>
       <c r="G79" s="4" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="H79" s="4"/>
       <c r="I79" s="4" t="s">
-        <v>155</v>
+        <v>149</v>
       </c>
       <c r="J79" s="4"/>
     </row>
@@ -5243,7 +5255,7 @@
         <v>2402</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="C80" s="3">
         <v>24</v>
@@ -5256,11 +5268,11 @@
         <v>32</v>
       </c>
       <c r="G80" s="4" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="H80" s="3"/>
       <c r="I80" s="4" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="J80" s="4"/>
     </row>
@@ -5269,7 +5281,7 @@
         <v>2403</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="C81" s="3">
         <v>24</v>
@@ -5284,7 +5296,7 @@
       <c r="G81" s="4"/>
       <c r="H81" s="5"/>
       <c r="I81" s="4" t="s">
-        <v>159</v>
+        <v>153</v>
       </c>
       <c r="J81" s="5" t="b">
         <v>1</v>
@@ -5295,7 +5307,7 @@
         <v>25</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="C82" s="3">
         <v>2</v>
@@ -5310,7 +5322,7 @@
       <c r="G82" s="4"/>
       <c r="H82" s="4"/>
       <c r="I82" s="4" t="s">
-        <v>160</v>
+        <v>154</v>
       </c>
       <c r="J82" s="4"/>
     </row>
@@ -5319,7 +5331,7 @@
         <v>2501</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="C83" s="3">
         <v>25</v>
@@ -5332,11 +5344,11 @@
         <v>32</v>
       </c>
       <c r="G83" s="4" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="H83" s="4"/>
       <c r="I83" s="4" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="J83" s="4"/>
     </row>

</xml_diff>

<commit_message>
#144 Dark Auto Focus
</commit_message>
<xml_diff>
--- a/Sources/Cuga-Calibration-Solution/Assets/Data/InitData.xlsx
+++ b/Sources/Cuga-Calibration-Solution/Assets/Data/InitData.xlsx
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="389" uniqueCount="171">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="388" uniqueCount="170">
   <si>
     <t>Id</t>
   </si>
@@ -280,7 +280,7 @@
     <t>Dark Auto Focus</t>
   </si>
   <si>
-    <t>CugaCalibration.ViewModels.Laser.LaserAutoFocusCalibrationViewModel</t>
+    <t>CugaCalibration.ViewModels.AutoFocus.AutoFocusDarkAutoFocusViewModel</t>
   </si>
   <si>
     <t>Global Focus Offset</t>
@@ -319,7 +319,7 @@
     <t>Line Orientation Offset</t>
   </si>
   <si>
-    <t>CugaCalibration.ViewModels.CIB.CIBLineOrientationOffsetViewModel</t>
+    <t>CugaCalibration.ViewModels.Laser.LaserLineOrientationOffsetCalibrationViewModel</t>
   </si>
   <si>
     <t>Illumination Profile</t>
@@ -347,12 +347,6 @@
   </si>
   <si>
     <t>Optics</t>
-  </si>
-  <si>
-    <t>SC</t>
-  </si>
-  <si>
-    <t>CugaCalibration.ViewModels.Optics.OpticsSCViewModel</t>
   </si>
   <si>
     <t>Relay</t>
@@ -542,16 +536,19 @@
     <t>CugaCalibration.ViewModels.Common.Windows.Tools.Optics.OpticsObjectiveYAngleWindowViewModel</t>
   </si>
   <si>
-    <t>Grabbing Image</t>
-  </si>
-  <si>
-    <t>CugaCalibration.ViewModels.Common.Windows.Tools.Optics.OpticsGrabbingImageWindowViewModel</t>
-  </si>
-  <si>
-    <t>Best Focus</t>
-  </si>
-  <si>
-    <t>CugaCalibration.ViewModels.Common.Windows.Tools.Optics.OpticsBestFocusWindowViewModel</t>
+    <t>Grab And Template</t>
+  </si>
+  <si>
+    <t>Grabbing Dark Image</t>
+  </si>
+  <si>
+    <t>CugaCalibration.ViewModels.Common.Windows.Tools.GrabbingDarkImageWindowViewModel</t>
+  </si>
+  <si>
+    <t>Create Dark Image Template</t>
+  </si>
+  <si>
+    <t>CugaCalibration.ViewModels.Common.Windows.Tools.CreateDarkImageTemplateWindowViewModel</t>
   </si>
   <si>
     <t>Diagnosis</t>
@@ -4888,7 +4885,7 @@
       <c r="A42" s="3">
         <v>1801</v>
       </c>
-      <c r="B42" s="6" t="s">
+      <c r="B42" s="4" t="s">
         <v>104</v>
       </c>
       <c r="C42" s="3">
@@ -4901,11 +4898,11 @@
       <c r="F42" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G42" s="6" t="s">
+      <c r="G42" s="4" t="s">
         <v>105</v>
       </c>
       <c r="H42" s="4"/>
-      <c r="I42" s="6" t="s">
+      <c r="I42" s="4" t="s">
         <v>104</v>
       </c>
       <c r="J42" s="4"/>
@@ -4966,7 +4963,7 @@
       <c r="A45" s="3">
         <v>1804</v>
       </c>
-      <c r="B45" s="4" t="s">
+      <c r="B45" s="6" t="s">
         <v>110</v>
       </c>
       <c r="C45" s="3">
@@ -4979,53 +4976,51 @@
       <c r="F45" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G45" s="4" t="s">
+      <c r="G45" s="6" t="s">
         <v>111</v>
       </c>
       <c r="H45" s="4"/>
-      <c r="I45" s="4" t="s">
+      <c r="I45" s="6" t="s">
         <v>110</v>
       </c>
       <c r="J45" s="4"/>
     </row>
     <row r="46" ht="15" customHeight="1" spans="1:10">
       <c r="A46" s="3">
-        <v>1805</v>
-      </c>
-      <c r="B46" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="B46" s="4" t="s">
         <v>112</v>
       </c>
       <c r="C46" s="3">
-        <v>18</v>
+        <v>-1</v>
       </c>
       <c r="D46" s="3">
-        <v>1805</v>
+        <v>2</v>
       </c>
       <c r="E46" s="3"/>
       <c r="F46" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G46" s="6" t="s">
-        <v>113</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="G46" s="4"/>
       <c r="H46" s="4"/>
-      <c r="I46" s="6" t="s">
+      <c r="I46" s="4" t="s">
         <v>112</v>
       </c>
       <c r="J46" s="4"/>
     </row>
     <row r="47" ht="15" customHeight="1" spans="1:10">
       <c r="A47" s="3">
+        <v>21</v>
+      </c>
+      <c r="B47" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="C47" s="3">
         <v>2</v>
       </c>
-      <c r="B47" s="4" t="s">
-        <v>114</v>
-      </c>
-      <c r="C47" s="3">
-        <v>-1</v>
-      </c>
       <c r="D47" s="3">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="E47" s="3"/>
       <c r="F47" s="3" t="s">
@@ -5034,37 +5029,39 @@
       <c r="G47" s="4"/>
       <c r="H47" s="4"/>
       <c r="I47" s="4" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="J47" s="4"/>
     </row>
     <row r="48" ht="15" customHeight="1" spans="1:10">
       <c r="A48" s="3">
+        <v>2110</v>
+      </c>
+      <c r="B48" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="C48" s="3">
         <v>21</v>
       </c>
-      <c r="B48" s="4" t="s">
-        <v>115</v>
-      </c>
-      <c r="C48" s="3">
-        <v>2</v>
-      </c>
       <c r="D48" s="3">
-        <v>21</v>
+        <v>2110</v>
       </c>
       <c r="E48" s="3"/>
       <c r="F48" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G48" s="4"/>
+        <v>35</v>
+      </c>
+      <c r="G48" s="4" t="s">
+        <v>115</v>
+      </c>
       <c r="H48" s="4"/>
       <c r="I48" s="4" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="J48" s="4"/>
     </row>
     <row r="49" ht="15" customHeight="1" spans="1:10">
       <c r="A49" s="3">
-        <v>2110</v>
+        <v>2111</v>
       </c>
       <c r="B49" s="4" t="s">
         <v>116</v>
@@ -5073,7 +5070,7 @@
         <v>21</v>
       </c>
       <c r="D49" s="3">
-        <v>2110</v>
+        <v>2111</v>
       </c>
       <c r="E49" s="3"/>
       <c r="F49" s="3" t="s">
@@ -5090,7 +5087,7 @@
     </row>
     <row r="50" ht="15" customHeight="1" spans="1:10">
       <c r="A50" s="3">
-        <v>2111</v>
+        <v>2112</v>
       </c>
       <c r="B50" s="4" t="s">
         <v>118</v>
@@ -5099,14 +5096,14 @@
         <v>21</v>
       </c>
       <c r="D50" s="3">
-        <v>2111</v>
+        <v>2112</v>
       </c>
       <c r="E50" s="3"/>
       <c r="F50" s="3" t="s">
         <v>35</v>
       </c>
       <c r="G50" s="4" t="s">
-        <v>119</v>
+        <v>115</v>
       </c>
       <c r="H50" s="4"/>
       <c r="I50" s="4" t="s">
@@ -5116,83 +5113,83 @@
     </row>
     <row r="51" ht="15" customHeight="1" spans="1:10">
       <c r="A51" s="3">
-        <v>2112</v>
+        <v>2113</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C51" s="3">
         <v>21</v>
       </c>
       <c r="D51" s="3">
-        <v>2112</v>
+        <v>2113</v>
       </c>
       <c r="E51" s="3"/>
       <c r="F51" s="3" t="s">
         <v>35</v>
       </c>
       <c r="G51" s="4" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="H51" s="4"/>
       <c r="I51" s="4" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="J51" s="4"/>
     </row>
     <row r="52" ht="15" customHeight="1" spans="1:10">
       <c r="A52" s="3">
-        <v>2113</v>
+        <v>22</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C52" s="3">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="D52" s="3">
-        <v>2113</v>
+        <v>22</v>
       </c>
       <c r="E52" s="3"/>
       <c r="F52" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G52" s="4" t="s">
-        <v>117</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="G52" s="4"/>
       <c r="H52" s="4"/>
       <c r="I52" s="4" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="J52" s="4"/>
     </row>
     <row r="53" ht="15" customHeight="1" spans="1:10">
       <c r="A53" s="3">
+        <v>2201</v>
+      </c>
+      <c r="B53" s="4" t="s">
+        <v>121</v>
+      </c>
+      <c r="C53" s="3">
         <v>22</v>
       </c>
-      <c r="B53" s="4" t="s">
-        <v>122</v>
-      </c>
-      <c r="C53" s="3">
-        <v>2</v>
-      </c>
       <c r="D53" s="3">
-        <v>22</v>
+        <v>2201</v>
       </c>
       <c r="E53" s="3"/>
       <c r="F53" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G53" s="4"/>
+        <v>35</v>
+      </c>
+      <c r="G53" s="4" t="s">
+        <v>122</v>
+      </c>
       <c r="H53" s="4"/>
       <c r="I53" s="4" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="J53" s="4"/>
     </row>
     <row r="54" ht="15" customHeight="1" spans="1:10">
       <c r="A54" s="3">
-        <v>2201</v>
+        <v>2202</v>
       </c>
       <c r="B54" s="4" t="s">
         <v>123</v>
@@ -5201,7 +5198,7 @@
         <v>22</v>
       </c>
       <c r="D54" s="3">
-        <v>2201</v>
+        <v>2202</v>
       </c>
       <c r="E54" s="3"/>
       <c r="F54" s="3" t="s">
@@ -5218,7 +5215,7 @@
     </row>
     <row r="55" ht="15" customHeight="1" spans="1:10">
       <c r="A55" s="3">
-        <v>2202</v>
+        <v>2203</v>
       </c>
       <c r="B55" s="4" t="s">
         <v>125</v>
@@ -5227,7 +5224,7 @@
         <v>22</v>
       </c>
       <c r="D55" s="3">
-        <v>2202</v>
+        <v>2203</v>
       </c>
       <c r="E55" s="3"/>
       <c r="F55" s="3" t="s">
@@ -5244,24 +5241,22 @@
     </row>
     <row r="56" ht="15" customHeight="1" spans="1:10">
       <c r="A56" s="3">
-        <v>2203</v>
+        <v>23</v>
       </c>
       <c r="B56" s="4" t="s">
         <v>127</v>
       </c>
       <c r="C56" s="3">
-        <v>22</v>
+        <v>2</v>
       </c>
       <c r="D56" s="3">
-        <v>2203</v>
+        <v>23</v>
       </c>
       <c r="E56" s="3"/>
       <c r="F56" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G56" s="4" t="s">
-        <v>128</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="G56" s="4"/>
       <c r="H56" s="4"/>
       <c r="I56" s="4" t="s">
         <v>127</v>
@@ -5270,81 +5265,83 @@
     </row>
     <row r="57" ht="15" customHeight="1" spans="1:10">
       <c r="A57" s="3">
+        <v>2301</v>
+      </c>
+      <c r="B57" s="4" t="s">
+        <v>128</v>
+      </c>
+      <c r="C57" s="3">
         <v>23</v>
       </c>
-      <c r="B57" s="4" t="s">
-        <v>129</v>
-      </c>
-      <c r="C57" s="3">
-        <v>2</v>
-      </c>
       <c r="D57" s="3">
-        <v>23</v>
+        <v>2301</v>
       </c>
       <c r="E57" s="3"/>
       <c r="F57" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G57" s="4"/>
+        <v>35</v>
+      </c>
+      <c r="G57" s="4" t="s">
+        <v>129</v>
+      </c>
       <c r="H57" s="4"/>
       <c r="I57" s="4" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="J57" s="4"/>
     </row>
     <row r="58" ht="15" customHeight="1" spans="1:10">
       <c r="A58" s="3">
-        <v>2301</v>
+        <v>2302</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>130</v>
+        <v>71</v>
       </c>
       <c r="C58" s="3">
         <v>23</v>
       </c>
       <c r="D58" s="3">
-        <v>2301</v>
+        <v>2302</v>
       </c>
       <c r="E58" s="3"/>
       <c r="F58" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G58" s="4" t="s">
-        <v>131</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="G58" s="4"/>
       <c r="H58" s="4"/>
       <c r="I58" s="4" t="s">
-        <v>130</v>
+        <v>71</v>
       </c>
       <c r="J58" s="4"/>
     </row>
     <row r="59" ht="15" customHeight="1" spans="1:10">
       <c r="A59" s="3">
+        <v>23021</v>
+      </c>
+      <c r="B59" s="4" t="s">
+        <v>130</v>
+      </c>
+      <c r="C59" s="3">
         <v>2302</v>
       </c>
-      <c r="B59" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="C59" s="3">
-        <v>23</v>
-      </c>
       <c r="D59" s="3">
-        <v>2302</v>
+        <v>23021</v>
       </c>
       <c r="E59" s="3"/>
       <c r="F59" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G59" s="4"/>
+        <v>35</v>
+      </c>
+      <c r="G59" s="4" t="s">
+        <v>131</v>
+      </c>
       <c r="H59" s="4"/>
       <c r="I59" s="4" t="s">
-        <v>71</v>
+        <v>130</v>
       </c>
       <c r="J59" s="4"/>
     </row>
     <row r="60" ht="15" customHeight="1" spans="1:10">
       <c r="A60" s="3">
-        <v>23021</v>
+        <v>23022</v>
       </c>
       <c r="B60" s="4" t="s">
         <v>132</v>
@@ -5353,7 +5350,7 @@
         <v>2302</v>
       </c>
       <c r="D60" s="3">
-        <v>23021</v>
+        <v>23022</v>
       </c>
       <c r="E60" s="3"/>
       <c r="F60" s="3" t="s">
@@ -5370,57 +5367,57 @@
     </row>
     <row r="61" ht="15" customHeight="1" spans="1:10">
       <c r="A61" s="3">
-        <v>23022</v>
+        <v>2303</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>134</v>
+        <v>70</v>
       </c>
       <c r="C61" s="3">
-        <v>2302</v>
+        <v>23</v>
       </c>
       <c r="D61" s="3">
-        <v>23022</v>
+        <v>2303</v>
       </c>
       <c r="E61" s="3"/>
       <c r="F61" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G61" s="4" t="s">
-        <v>135</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="G61" s="4"/>
       <c r="H61" s="4"/>
       <c r="I61" s="4" t="s">
-        <v>134</v>
+        <v>70</v>
       </c>
       <c r="J61" s="4"/>
     </row>
     <row r="62" ht="15" customHeight="1" spans="1:10">
       <c r="A62" s="3">
+        <v>23031</v>
+      </c>
+      <c r="B62" s="4" t="s">
+        <v>134</v>
+      </c>
+      <c r="C62" s="3">
         <v>2303</v>
       </c>
-      <c r="B62" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="C62" s="3">
-        <v>23</v>
-      </c>
       <c r="D62" s="3">
-        <v>2303</v>
+        <v>23031</v>
       </c>
       <c r="E62" s="3"/>
       <c r="F62" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G62" s="4"/>
+        <v>35</v>
+      </c>
+      <c r="G62" s="4" t="s">
+        <v>135</v>
+      </c>
       <c r="H62" s="4"/>
       <c r="I62" s="4" t="s">
-        <v>70</v>
+        <v>134</v>
       </c>
       <c r="J62" s="4"/>
     </row>
     <row r="63" ht="15" customHeight="1" spans="1:10">
       <c r="A63" s="3">
-        <v>23031</v>
+        <v>23032</v>
       </c>
       <c r="B63" s="4" t="s">
         <v>136</v>
@@ -5429,7 +5426,7 @@
         <v>2303</v>
       </c>
       <c r="D63" s="3">
-        <v>23031</v>
+        <v>23032</v>
       </c>
       <c r="E63" s="3"/>
       <c r="F63" s="3" t="s">
@@ -5446,7 +5443,7 @@
     </row>
     <row r="64" ht="15" customHeight="1" spans="1:10">
       <c r="A64" s="3">
-        <v>23032</v>
+        <v>23033</v>
       </c>
       <c r="B64" s="4" t="s">
         <v>138</v>
@@ -5455,7 +5452,7 @@
         <v>2303</v>
       </c>
       <c r="D64" s="3">
-        <v>23032</v>
+        <v>23033</v>
       </c>
       <c r="E64" s="3"/>
       <c r="F64" s="3" t="s">
@@ -5472,7 +5469,7 @@
     </row>
     <row r="65" ht="15" customHeight="1" spans="1:10">
       <c r="A65" s="3">
-        <v>23033</v>
+        <v>23034</v>
       </c>
       <c r="B65" s="4" t="s">
         <v>140</v>
@@ -5481,7 +5478,7 @@
         <v>2303</v>
       </c>
       <c r="D65" s="3">
-        <v>23033</v>
+        <v>23034</v>
       </c>
       <c r="E65" s="3"/>
       <c r="F65" s="3" t="s">
@@ -5498,7 +5495,7 @@
     </row>
     <row r="66" ht="15" customHeight="1" spans="1:10">
       <c r="A66" s="3">
-        <v>23034</v>
+        <v>23035</v>
       </c>
       <c r="B66" s="4" t="s">
         <v>142</v>
@@ -5507,7 +5504,7 @@
         <v>2303</v>
       </c>
       <c r="D66" s="3">
-        <v>23034</v>
+        <v>23035</v>
       </c>
       <c r="E66" s="3"/>
       <c r="F66" s="3" t="s">
@@ -5524,24 +5521,22 @@
     </row>
     <row r="67" ht="15" customHeight="1" spans="1:10">
       <c r="A67" s="3">
-        <v>23035</v>
+        <v>2304</v>
       </c>
       <c r="B67" s="4" t="s">
         <v>144</v>
       </c>
       <c r="C67" s="3">
-        <v>2303</v>
+        <v>23</v>
       </c>
       <c r="D67" s="3">
-        <v>23035</v>
+        <v>2304</v>
       </c>
       <c r="E67" s="3"/>
       <c r="F67" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G67" s="4" t="s">
-        <v>145</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="G67" s="4"/>
       <c r="H67" s="4"/>
       <c r="I67" s="4" t="s">
         <v>144</v>
@@ -5550,98 +5545,98 @@
     </row>
     <row r="68" ht="15" customHeight="1" spans="1:10">
       <c r="A68" s="3">
+        <v>23041</v>
+      </c>
+      <c r="B68" s="4" t="s">
+        <v>145</v>
+      </c>
+      <c r="C68" s="3">
         <v>2304</v>
       </c>
-      <c r="B68" s="4" t="s">
-        <v>146</v>
-      </c>
-      <c r="C68" s="3">
-        <v>23</v>
-      </c>
       <c r="D68" s="3">
-        <v>2304</v>
+        <v>23041</v>
       </c>
       <c r="E68" s="3"/>
       <c r="F68" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G68" s="4"/>
+        <v>35</v>
+      </c>
+      <c r="G68" s="4" t="s">
+        <v>146</v>
+      </c>
       <c r="H68" s="4"/>
       <c r="I68" s="4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="J68" s="4"/>
     </row>
     <row r="69" ht="15" customHeight="1" spans="1:10">
       <c r="A69" s="3">
-        <v>23041</v>
+        <v>2305</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>147</v>
+        <v>103</v>
       </c>
       <c r="C69" s="3">
-        <v>2304</v>
+        <v>23</v>
       </c>
       <c r="D69" s="3">
-        <v>23041</v>
+        <v>2305</v>
       </c>
       <c r="E69" s="3"/>
       <c r="F69" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G69" s="4" t="s">
-        <v>148</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="G69" s="4"/>
       <c r="H69" s="4"/>
       <c r="I69" s="4" t="s">
-        <v>147</v>
+        <v>103</v>
       </c>
       <c r="J69" s="4"/>
     </row>
     <row r="70" ht="15" customHeight="1" spans="1:10">
       <c r="A70" s="3">
+        <v>23051</v>
+      </c>
+      <c r="B70" s="4" t="s">
+        <v>147</v>
+      </c>
+      <c r="C70" s="3">
         <v>2305</v>
       </c>
-      <c r="B70" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="C70" s="3">
-        <v>23</v>
-      </c>
       <c r="D70" s="3">
-        <v>2305</v>
+        <v>23051</v>
       </c>
       <c r="E70" s="3"/>
       <c r="F70" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G70" s="4"/>
+        <v>35</v>
+      </c>
+      <c r="G70" s="4" t="s">
+        <v>148</v>
+      </c>
       <c r="H70" s="4"/>
       <c r="I70" s="4" t="s">
-        <v>103</v>
+        <v>147</v>
       </c>
       <c r="J70" s="4"/>
     </row>
     <row r="71" ht="15" customHeight="1" spans="1:10">
       <c r="A71" s="3">
-        <v>23051</v>
+        <v>2306</v>
       </c>
       <c r="B71" s="4" t="s">
         <v>149</v>
       </c>
       <c r="C71" s="3">
-        <v>2305</v>
+        <v>23</v>
       </c>
       <c r="D71" s="3">
-        <v>23051</v>
+        <v>2306</v>
       </c>
       <c r="E71" s="3"/>
       <c r="F71" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G71" s="6" t="s">
-        <v>150</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="G71" s="4"/>
       <c r="H71" s="4"/>
       <c r="I71" s="4" t="s">
         <v>149</v>
@@ -5650,53 +5645,53 @@
     </row>
     <row r="72" ht="15" customHeight="1" spans="1:10">
       <c r="A72" s="3">
-        <v>23052</v>
-      </c>
-      <c r="B72" s="6" t="s">
-        <v>151</v>
+        <v>23061</v>
+      </c>
+      <c r="B72" s="4" t="s">
+        <v>150</v>
       </c>
       <c r="C72" s="3">
-        <v>2305</v>
+        <v>2306</v>
       </c>
       <c r="D72" s="3">
-        <v>23052</v>
+        <v>23061</v>
       </c>
       <c r="E72" s="3"/>
       <c r="F72" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G72" s="6" t="s">
-        <v>152</v>
+      <c r="G72" s="4" t="s">
+        <v>151</v>
       </c>
       <c r="H72" s="4"/>
-      <c r="I72" s="6" t="s">
-        <v>151</v>
+      <c r="I72" s="4" t="s">
+        <v>150</v>
       </c>
       <c r="J72" s="4"/>
     </row>
     <row r="73" ht="15" customHeight="1" spans="1:10">
       <c r="A73" s="3">
-        <v>23053</v>
-      </c>
-      <c r="B73" s="6" t="s">
-        <v>153</v>
+        <v>23062</v>
+      </c>
+      <c r="B73" s="4" t="s">
+        <v>152</v>
       </c>
       <c r="C73" s="3">
-        <v>2305</v>
+        <v>2306</v>
       </c>
       <c r="D73" s="3">
-        <v>23053</v>
+        <v>23062</v>
       </c>
       <c r="E73" s="3"/>
       <c r="F73" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G73" s="6" t="s">
-        <v>154</v>
+      <c r="G73" s="4" t="s">
+        <v>153</v>
       </c>
       <c r="H73" s="4"/>
-      <c r="I73" s="6" t="s">
-        <v>153</v>
+      <c r="I73" s="4" t="s">
+        <v>152</v>
       </c>
       <c r="J73" s="4"/>
     </row>
@@ -5705,7 +5700,7 @@
         <v>2307</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C74" s="3">
         <v>23</v>
@@ -5720,7 +5715,7 @@
       <c r="G74" s="3"/>
       <c r="H74" s="3"/>
       <c r="I74" s="4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="J74" s="4"/>
     </row>
@@ -5729,7 +5724,7 @@
         <v>23071</v>
       </c>
       <c r="B75" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C75" s="3">
         <v>2307</v>
@@ -5742,11 +5737,11 @@
         <v>35</v>
       </c>
       <c r="G75" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="H75" s="3"/>
       <c r="I75" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="J75" s="4"/>
     </row>
@@ -5755,7 +5750,7 @@
         <v>23072</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C76" s="3">
         <v>2307</v>
@@ -5768,11 +5763,11 @@
         <v>35</v>
       </c>
       <c r="G76" s="4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="H76" s="4"/>
       <c r="I76" s="4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="J76" s="4"/>
     </row>
@@ -5781,7 +5776,7 @@
         <v>23073</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C77" s="3">
         <v>2307</v>
@@ -5794,11 +5789,11 @@
         <v>35</v>
       </c>
       <c r="G77" s="4" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="H77" s="4"/>
       <c r="I77" s="4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="J77" s="4"/>
     </row>
@@ -5807,7 +5802,7 @@
         <v>24</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C78" s="3">
         <v>2</v>
@@ -5822,7 +5817,7 @@
       <c r="G78" s="4"/>
       <c r="H78" s="4"/>
       <c r="I78" s="4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="J78" s="4"/>
     </row>
@@ -5831,7 +5826,7 @@
         <v>2401</v>
       </c>
       <c r="B79" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C79" s="3">
         <v>24</v>
@@ -5844,11 +5839,11 @@
         <v>35</v>
       </c>
       <c r="G79" s="4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="H79" s="4"/>
       <c r="I79" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="J79" s="4"/>
     </row>
@@ -5857,7 +5852,7 @@
         <v>2402</v>
       </c>
       <c r="B80" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C80" s="3">
         <v>24</v>
@@ -5870,11 +5865,11 @@
         <v>35</v>
       </c>
       <c r="G80" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H80" s="3"/>
       <c r="I80" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="J80" s="4"/>
     </row>
@@ -5883,7 +5878,7 @@
         <v>2403</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C81" s="3">
         <v>24</v>
@@ -5898,7 +5893,7 @@
       <c r="G81" s="4"/>
       <c r="H81" s="5"/>
       <c r="I81" s="4" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="J81" s="5" t="b">
         <v>1</v>
@@ -5909,7 +5904,7 @@
         <v>25</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C82" s="3">
         <v>2</v>
@@ -5924,7 +5919,7 @@
       <c r="G82" s="4"/>
       <c r="H82" s="4"/>
       <c r="I82" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J82" s="4"/>
     </row>
@@ -5933,7 +5928,7 @@
         <v>2501</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="C83" s="3">
         <v>25</v>
@@ -5946,11 +5941,11 @@
         <v>35</v>
       </c>
       <c r="G83" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="H83" s="4"/>
       <c r="I83" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="J83" s="4"/>
     </row>

</xml_diff>

<commit_message>
#119 Coss talk diagnosis合并
</commit_message>
<xml_diff>
--- a/Sources/Cuga-Calibration-Solution/Assets/Data/InitData.xlsx
+++ b/Sources/Cuga-Calibration-Solution/Assets/Data/InitData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Calibration_Chj\netcore_semix_cuga_calibration\Sources\Cuga-Calibration-Solution\Assets\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E991C02-59D8-4A75-AB57-5D5378906142}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A26FB339-5F54-4BB8-BD1B-CF065FA13233}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="30960" windowHeight="16800" tabRatio="500" firstSheet="1" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1340" uniqueCount="363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1344" uniqueCount="366">
   <si>
     <t>Id</t>
   </si>
@@ -1186,12 +1186,24 @@
     <t>CugaCalibration.ViewModels.Common.Windows.Tools.Collection.CollectionYGhostWindowViewModel</t>
     <phoneticPr fontId="7" type="noConversion"/>
   </si>
+  <si>
+    <t>Collection</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>CugaCalibration.ViewModels.Common.Windows.Tools.Collection.CollectionCrossTalkWindowViewModel</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
+  <si>
+    <t>Collection CrossTalk</t>
+    <phoneticPr fontId="7" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -1239,6 +1251,13 @@
     </font>
     <font>
       <sz val="9"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="等线"/>
       <family val="3"/>
       <charset val="134"/>
@@ -1315,7 +1334,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1354,6 +1373,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -7254,7 +7276,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:J273"/>
+  <dimension ref="A1:J274"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.625" style="1" customWidth="1"/>
@@ -14169,8 +14191,8 @@
       <c r="A253" s="3">
         <v>2304</v>
       </c>
-      <c r="B253" s="4" t="s">
-        <v>329</v>
+      <c r="B253" s="13" t="s">
+        <v>363</v>
       </c>
       <c r="C253" s="3">
         <v>23</v>
@@ -14217,489 +14239,515 @@
     </row>
     <row r="255" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A255" s="3">
-        <v>23043</v>
-      </c>
-      <c r="B255" s="4" t="s">
-        <v>361</v>
+        <v>23042</v>
+      </c>
+      <c r="B255" s="13" t="s">
+        <v>365</v>
       </c>
       <c r="C255" s="3">
         <v>2304</v>
       </c>
       <c r="D255" s="3">
-        <v>23043</v>
+        <v>23042</v>
       </c>
       <c r="E255" s="3"/>
       <c r="F255" s="3" t="s">
         <v>55</v>
       </c>
       <c r="G255" s="4" t="s">
-        <v>362</v>
+        <v>364</v>
       </c>
       <c r="H255" s="4"/>
-      <c r="I255" s="4" t="s">
-        <v>361</v>
+      <c r="I255" s="13" t="s">
+        <v>365</v>
       </c>
       <c r="J255" s="4"/>
     </row>
     <row r="256" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A256" s="3">
-        <v>2305</v>
+        <v>23043</v>
       </c>
       <c r="B256" s="4" t="s">
-        <v>39</v>
+        <v>361</v>
       </c>
       <c r="C256" s="3">
-        <v>23</v>
+        <v>2304</v>
       </c>
       <c r="D256" s="3">
-        <v>2305</v>
+        <v>23043</v>
       </c>
       <c r="E256" s="3"/>
       <c r="F256" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="G256" s="4"/>
+        <v>55</v>
+      </c>
+      <c r="G256" s="4" t="s">
+        <v>362</v>
+      </c>
       <c r="H256" s="4"/>
       <c r="I256" s="4" t="s">
-        <v>39</v>
+        <v>361</v>
       </c>
       <c r="J256" s="4"/>
     </row>
     <row r="257" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A257" s="3">
-        <v>23051</v>
+        <v>2305</v>
       </c>
       <c r="B257" s="4" t="s">
-        <v>332</v>
+        <v>39</v>
       </c>
       <c r="C257" s="3">
+        <v>23</v>
+      </c>
+      <c r="D257" s="3">
         <v>2305</v>
-      </c>
-      <c r="D257" s="3">
-        <v>23051</v>
       </c>
       <c r="E257" s="3"/>
       <c r="F257" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="G257" s="4" t="s">
-        <v>333</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G257" s="4"/>
       <c r="H257" s="4"/>
       <c r="I257" s="4" t="s">
-        <v>332</v>
+        <v>39</v>
       </c>
       <c r="J257" s="4"/>
     </row>
     <row r="258" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A258" s="3">
-        <v>2306</v>
+        <v>23051</v>
       </c>
       <c r="B258" s="4" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="C258" s="3">
-        <v>23</v>
+        <v>2305</v>
       </c>
       <c r="D258" s="3">
-        <v>2306</v>
+        <v>23051</v>
       </c>
       <c r="E258" s="3"/>
       <c r="F258" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="G258" s="4"/>
+        <v>55</v>
+      </c>
+      <c r="G258" s="4" t="s">
+        <v>333</v>
+      </c>
       <c r="H258" s="4"/>
       <c r="I258" s="4" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="J258" s="4"/>
     </row>
     <row r="259" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A259" s="3">
-        <v>23061</v>
+        <v>2306</v>
       </c>
       <c r="B259" s="4" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C259" s="3">
+        <v>23</v>
+      </c>
+      <c r="D259" s="3">
         <v>2306</v>
-      </c>
-      <c r="D259" s="3">
-        <v>23061</v>
       </c>
       <c r="E259" s="3"/>
       <c r="F259" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="G259" s="4" t="s">
-        <v>336</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G259" s="4"/>
       <c r="H259" s="4"/>
       <c r="I259" s="4" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="J259" s="4"/>
     </row>
     <row r="260" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A260" s="3">
-        <v>23062</v>
+        <v>23061</v>
       </c>
       <c r="B260" s="4" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="C260" s="3">
         <v>2306</v>
       </c>
       <c r="D260" s="3">
-        <v>23062</v>
+        <v>23061</v>
       </c>
       <c r="E260" s="3"/>
       <c r="F260" s="3" t="s">
         <v>55</v>
       </c>
       <c r="G260" s="4" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="H260" s="4"/>
       <c r="I260" s="4" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="J260" s="4"/>
     </row>
     <row r="261" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A261" s="3">
-        <v>23063</v>
+        <v>23062</v>
       </c>
       <c r="B261" s="4" t="s">
-        <v>339</v>
+        <v>337</v>
       </c>
       <c r="C261" s="3">
         <v>2306</v>
       </c>
       <c r="D261" s="3">
-        <v>23063</v>
+        <v>23062</v>
       </c>
       <c r="E261" s="3"/>
       <c r="F261" s="3" t="s">
         <v>55</v>
       </c>
       <c r="G261" s="4" t="s">
-        <v>340</v>
+        <v>338</v>
       </c>
       <c r="H261" s="4"/>
       <c r="I261" s="4" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
       <c r="J261" s="4"/>
     </row>
     <row r="262" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A262" s="3">
-        <v>2307</v>
+        <v>23063</v>
       </c>
       <c r="B262" s="4" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="C262" s="3">
-        <v>23</v>
+        <v>2306</v>
       </c>
       <c r="D262" s="3">
-        <v>2307</v>
+        <v>23063</v>
       </c>
       <c r="E262" s="3"/>
       <c r="F262" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="G262" s="3"/>
-      <c r="H262" s="3"/>
+        <v>55</v>
+      </c>
+      <c r="G262" s="4" t="s">
+        <v>340</v>
+      </c>
+      <c r="H262" s="4"/>
       <c r="I262" s="4" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="J262" s="4"/>
     </row>
     <row r="263" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A263" s="3">
-        <v>23071</v>
+        <v>2307</v>
       </c>
       <c r="B263" s="4" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="C263" s="3">
+        <v>23</v>
+      </c>
+      <c r="D263" s="3">
         <v>2307</v>
-      </c>
-      <c r="D263" s="3">
-        <v>23071</v>
       </c>
       <c r="E263" s="3"/>
       <c r="F263" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="G263" s="4" t="s">
-        <v>344</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G263" s="3"/>
       <c r="H263" s="3"/>
       <c r="I263" s="4" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="J263" s="4"/>
     </row>
     <row r="264" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A264" s="3">
-        <v>23072</v>
+        <v>23071</v>
       </c>
       <c r="B264" s="4" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="C264" s="3">
         <v>2307</v>
       </c>
       <c r="D264" s="3">
-        <v>23072</v>
+        <v>23071</v>
       </c>
       <c r="E264" s="3"/>
       <c r="F264" s="3" t="s">
         <v>55</v>
       </c>
       <c r="G264" s="4" t="s">
-        <v>346</v>
-      </c>
-      <c r="H264" s="4"/>
+        <v>344</v>
+      </c>
+      <c r="H264" s="3"/>
       <c r="I264" s="4" t="s">
-        <v>345</v>
+        <v>343</v>
       </c>
       <c r="J264" s="4"/>
     </row>
     <row r="265" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A265" s="3">
-        <v>23073</v>
+        <v>23072</v>
       </c>
       <c r="B265" s="4" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="C265" s="3">
         <v>2307</v>
       </c>
       <c r="D265" s="3">
-        <v>23073</v>
+        <v>23072</v>
       </c>
       <c r="E265" s="3"/>
       <c r="F265" s="3" t="s">
         <v>55</v>
       </c>
       <c r="G265" s="4" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
       <c r="H265" s="4"/>
       <c r="I265" s="4" t="s">
-        <v>347</v>
+        <v>345</v>
       </c>
       <c r="J265" s="4"/>
     </row>
     <row r="266" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A266" s="3">
-        <v>24</v>
+        <v>23073</v>
       </c>
       <c r="B266" s="4" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="C266" s="3">
-        <v>2</v>
+        <v>2307</v>
       </c>
       <c r="D266" s="3">
-        <v>24</v>
-      </c>
-      <c r="E266" s="4"/>
+        <v>23073</v>
+      </c>
+      <c r="E266" s="3"/>
       <c r="F266" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="G266" s="4"/>
+        <v>55</v>
+      </c>
+      <c r="G266" s="4" t="s">
+        <v>348</v>
+      </c>
       <c r="H266" s="4"/>
       <c r="I266" s="4" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
       <c r="J266" s="4"/>
     </row>
     <row r="267" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A267" s="3">
-        <v>2401</v>
+        <v>24</v>
       </c>
       <c r="B267" s="4" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="C267" s="3">
+        <v>2</v>
+      </c>
+      <c r="D267" s="3">
         <v>24</v>
-      </c>
-      <c r="D267" s="3">
-        <v>2401</v>
       </c>
       <c r="E267" s="4"/>
       <c r="F267" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="G267" s="4" t="s">
-        <v>351</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G267" s="4"/>
       <c r="H267" s="4"/>
       <c r="I267" s="4" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="J267" s="4"/>
     </row>
     <row r="268" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A268" s="3">
-        <v>25</v>
+        <v>2401</v>
       </c>
       <c r="B268" s="4" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="C268" s="3">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="D268" s="3">
-        <v>25</v>
+        <v>2401</v>
       </c>
       <c r="E268" s="4"/>
       <c r="F268" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="G268" s="4"/>
+        <v>55</v>
+      </c>
+      <c r="G268" s="4" t="s">
+        <v>351</v>
+      </c>
       <c r="H268" s="4"/>
       <c r="I268" s="4" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="J268" s="4"/>
     </row>
     <row r="269" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A269" s="3">
-        <v>2501</v>
+        <v>25</v>
       </c>
       <c r="B269" s="4" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="C269" s="3">
+        <v>2</v>
+      </c>
+      <c r="D269" s="3">
         <v>25</v>
       </c>
-      <c r="D269" s="3">
-        <v>2501</v>
-      </c>
-      <c r="E269" s="3"/>
+      <c r="E269" s="4"/>
       <c r="F269" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="G269" s="4" t="s">
-        <v>354</v>
-      </c>
-      <c r="H269" s="3"/>
+        <v>52</v>
+      </c>
+      <c r="G269" s="4"/>
+      <c r="H269" s="4"/>
       <c r="I269" s="4" t="s">
-        <v>349</v>
+        <v>353</v>
       </c>
       <c r="J269" s="4"/>
     </row>
     <row r="270" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A270" s="3">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="B270" s="4" t="s">
-        <v>355</v>
+        <v>349</v>
       </c>
       <c r="C270" s="3">
         <v>25</v>
       </c>
       <c r="D270" s="3">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="E270" s="3"/>
       <c r="F270" s="3" t="s">
         <v>55</v>
       </c>
       <c r="G270" s="4" t="s">
-        <v>356</v>
-      </c>
-      <c r="H270" s="5"/>
-      <c r="I270" s="5" t="s">
-        <v>355</v>
-      </c>
-      <c r="J270" s="5"/>
+        <v>354</v>
+      </c>
+      <c r="H270" s="3"/>
+      <c r="I270" s="4" t="s">
+        <v>349</v>
+      </c>
+      <c r="J270" s="4"/>
     </row>
     <row r="271" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A271" s="3">
-        <v>2503</v>
+        <v>2502</v>
       </c>
       <c r="B271" s="4" t="s">
-        <v>357</v>
+        <v>355</v>
       </c>
       <c r="C271" s="3">
         <v>25</v>
       </c>
       <c r="D271" s="3">
-        <v>2503</v>
+        <v>2502</v>
       </c>
       <c r="E271" s="3"/>
       <c r="F271" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="G271" s="4"/>
+      <c r="G271" s="4" t="s">
+        <v>356</v>
+      </c>
       <c r="H271" s="5"/>
       <c r="I271" s="5" t="s">
-        <v>357</v>
-      </c>
-      <c r="J271" s="5" t="b">
-        <v>1</v>
-      </c>
+        <v>355</v>
+      </c>
+      <c r="J271" s="5"/>
     </row>
     <row r="272" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A272" s="3">
-        <v>26</v>
+        <v>2503</v>
       </c>
       <c r="B272" s="4" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="C272" s="3">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="D272" s="3">
-        <v>26</v>
+        <v>2503</v>
       </c>
       <c r="E272" s="3"/>
       <c r="F272" s="3" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="G272" s="4"/>
-      <c r="H272" s="4"/>
-      <c r="I272" s="4" t="s">
-        <v>358</v>
-      </c>
-      <c r="J272" s="4"/>
+      <c r="H272" s="5"/>
+      <c r="I272" s="5" t="s">
+        <v>357</v>
+      </c>
+      <c r="J272" s="5" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="273" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A273" s="3">
-        <v>2601</v>
+        <v>26</v>
       </c>
       <c r="B273" s="4" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="C273" s="3">
+        <v>2</v>
+      </c>
+      <c r="D273" s="3">
         <v>26</v>
       </c>
-      <c r="D273" s="3">
-        <v>2601</v>
-      </c>
-      <c r="E273" s="4"/>
+      <c r="E273" s="3"/>
       <c r="F273" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="G273" s="4" t="s">
-        <v>360</v>
-      </c>
+        <v>52</v>
+      </c>
+      <c r="G273" s="4"/>
       <c r="H273" s="4"/>
       <c r="I273" s="4" t="s">
+        <v>358</v>
+      </c>
+      <c r="J273" s="4"/>
+    </row>
+    <row r="274" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A274" s="3">
+        <v>2601</v>
+      </c>
+      <c r="B274" s="4" t="s">
         <v>359</v>
       </c>
-      <c r="J273" s="4"/>
+      <c r="C274" s="3">
+        <v>26</v>
+      </c>
+      <c r="D274" s="3">
+        <v>2601</v>
+      </c>
+      <c r="E274" s="4"/>
+      <c r="F274" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="G274" s="4" t="s">
+        <v>360</v>
+      </c>
+      <c r="H274" s="4"/>
+      <c r="I274" s="4" t="s">
+        <v>359</v>
+      </c>
+      <c r="J274" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>
   <pageMargins left="0.70069444444444495" right="0.70069444444444495" top="0.75208333333333299" bottom="0.75208333333333299" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
#156 AGC Delay 2.0
</commit_message>
<xml_diff>
--- a/Sources/Cuga-Calibration-Solution/Assets/Data/InitData.xlsx
+++ b/Sources/Cuga-Calibration-Solution/Assets/Data/InitData.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\RiderProjects\semix\kaizhi.xuan\netcore_semix_cuga_calibration\Sources\Cuga-Calibration-Solution\Assets\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{951CD411-5BC8-4A49-9B7C-6F394DEE390C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B72FF501-B905-49BF-B18D-CBD9166777FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="425" uniqueCount="190">
   <si>
     <t>Id</t>
   </si>
@@ -341,9 +341,6 @@
   </si>
   <si>
     <t>MMD</t>
-  </si>
-  <si>
-    <t>CugaCalibration.ViewModels.CIB.CIBMMDViewModel</t>
   </si>
   <si>
     <t>Light Matching</t>
@@ -655,6 +652,22 @@
   </si>
   <si>
     <t>Collector Slit</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>XTC</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>AGC Delay</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>CugaCalibration.ViewModels.CIB.CIBMMDViewModel</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>CugaCalibration.ViewModels.CIB.CIBAGCDelayViewModel</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
@@ -3241,7 +3254,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:J91"/>
+  <dimension ref="A1:J92"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.625" style="1" customWidth="1"/>
@@ -4210,8 +4223,8 @@
       <c r="A38" s="3">
         <v>1706</v>
       </c>
-      <c r="B38" s="4" t="s">
-        <v>97</v>
+      <c r="B38" s="11" t="s">
+        <v>187</v>
       </c>
       <c r="C38" s="3">
         <v>17</v>
@@ -4223,12 +4236,12 @@
       <c r="F38" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G38" s="4" t="s">
-        <v>98</v>
+      <c r="G38" s="11" t="s">
+        <v>189</v>
       </c>
       <c r="H38" s="4"/>
-      <c r="I38" s="4" t="s">
-        <v>97</v>
+      <c r="I38" s="11" t="s">
+        <v>187</v>
       </c>
       <c r="J38" s="4"/>
     </row>
@@ -4236,8 +4249,8 @@
       <c r="A39" s="3">
         <v>1707</v>
       </c>
-      <c r="B39" s="4" t="s">
-        <v>99</v>
+      <c r="B39" s="11" t="s">
+        <v>186</v>
       </c>
       <c r="C39" s="3">
         <v>17</v>
@@ -4250,11 +4263,11 @@
         <v>35</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H39" s="4"/>
       <c r="I39" s="4" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="J39" s="4"/>
     </row>
@@ -4263,7 +4276,7 @@
         <v>1708</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C40" s="3">
         <v>17</v>
@@ -4275,359 +4288,361 @@
       <c r="F40" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G40" s="4" t="s">
-        <v>102</v>
+      <c r="G40" s="11" t="s">
+        <v>188</v>
       </c>
       <c r="H40" s="4"/>
       <c r="I40" s="4" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="J40" s="4"/>
     </row>
     <row r="41" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="3">
-        <v>18</v>
+        <v>1709</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="C41" s="3">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="D41" s="3">
-        <v>18</v>
+        <v>1709</v>
       </c>
       <c r="E41" s="3"/>
       <c r="F41" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G41" s="4"/>
+        <v>35</v>
+      </c>
+      <c r="G41" s="4" t="s">
+        <v>101</v>
+      </c>
       <c r="H41" s="4"/>
       <c r="I41" s="4" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="J41" s="4"/>
     </row>
     <row r="42" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="3">
-        <v>1801</v>
+        <v>18</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C42" s="3">
+        <v>1</v>
+      </c>
+      <c r="D42" s="3">
         <v>18</v>
-      </c>
-      <c r="D42" s="3">
-        <v>1801</v>
       </c>
       <c r="E42" s="3"/>
       <c r="F42" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G42" s="4" t="s">
-        <v>105</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="G42" s="4"/>
       <c r="H42" s="4"/>
       <c r="I42" s="4" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="J42" s="4"/>
     </row>
     <row r="43" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="3">
-        <v>1802</v>
+        <v>1801</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="C43" s="3">
         <v>18</v>
       </c>
       <c r="D43" s="3">
-        <v>1802</v>
+        <v>1801</v>
       </c>
       <c r="E43" s="3"/>
       <c r="F43" s="3" t="s">
         <v>35</v>
       </c>
       <c r="G43" s="4" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="H43" s="4"/>
       <c r="I43" s="4" t="s">
-        <v>106</v>
+        <v>103</v>
       </c>
       <c r="J43" s="4"/>
     </row>
     <row r="44" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="3">
-        <v>1803</v>
+        <v>1802</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="C44" s="3">
         <v>18</v>
       </c>
       <c r="D44" s="3">
-        <v>1803</v>
+        <v>1802</v>
       </c>
       <c r="E44" s="3"/>
       <c r="F44" s="3" t="s">
         <v>35</v>
       </c>
       <c r="G44" s="4" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="H44" s="4"/>
       <c r="I44" s="4" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="J44" s="4"/>
     </row>
     <row r="45" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="3">
-        <v>1804</v>
+        <v>1803</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="C45" s="3">
         <v>18</v>
       </c>
       <c r="D45" s="3">
-        <v>1804</v>
+        <v>1803</v>
       </c>
       <c r="E45" s="3"/>
       <c r="F45" s="3" t="s">
         <v>35</v>
       </c>
       <c r="G45" s="4" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="H45" s="4"/>
       <c r="I45" s="4" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="J45" s="4"/>
     </row>
     <row r="46" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="3">
-        <v>1805</v>
+        <v>1804</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="C46" s="3">
         <v>18</v>
       </c>
       <c r="D46" s="3">
-        <v>1805</v>
+        <v>1804</v>
       </c>
       <c r="E46" s="3"/>
       <c r="F46" s="3" t="s">
         <v>35</v>
       </c>
       <c r="G46" s="4" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="H46" s="4"/>
       <c r="I46" s="4" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="J46" s="4"/>
     </row>
     <row r="47" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="3">
-        <v>19</v>
+        <v>1805</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C47" s="3">
-        <v>1</v>
+        <v>18</v>
       </c>
       <c r="D47" s="3">
-        <v>19</v>
+        <v>1805</v>
       </c>
       <c r="E47" s="3"/>
       <c r="F47" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G47" s="4"/>
+        <v>35</v>
+      </c>
+      <c r="G47" s="4" t="s">
+        <v>112</v>
+      </c>
       <c r="H47" s="4"/>
       <c r="I47" s="4" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="J47" s="4"/>
     </row>
     <row r="48" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="3">
-        <v>1901</v>
+        <v>19</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C48" s="3">
+        <v>1</v>
+      </c>
+      <c r="D48" s="3">
         <v>19</v>
-      </c>
-      <c r="D48" s="3">
-        <v>1901</v>
       </c>
       <c r="E48" s="3"/>
       <c r="F48" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G48" s="4" t="s">
-        <v>116</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="G48" s="4"/>
       <c r="H48" s="4"/>
       <c r="I48" s="4" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="J48" s="4"/>
     </row>
     <row r="49" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="3">
-        <v>1902</v>
+        <v>1901</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="C49" s="3">
         <v>19</v>
       </c>
       <c r="D49" s="3">
-        <v>1902</v>
+        <v>1901</v>
       </c>
       <c r="E49" s="3"/>
       <c r="F49" s="3" t="s">
         <v>35</v>
       </c>
       <c r="G49" s="4" t="s">
-        <v>118</v>
+        <v>115</v>
       </c>
       <c r="H49" s="4"/>
       <c r="I49" s="4" t="s">
-        <v>117</v>
+        <v>114</v>
       </c>
       <c r="J49" s="4"/>
     </row>
     <row r="50" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="3">
-        <v>1903</v>
+        <v>1902</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="C50" s="3">
         <v>19</v>
       </c>
       <c r="D50" s="3">
-        <v>1903</v>
+        <v>1902</v>
       </c>
       <c r="E50" s="3"/>
       <c r="F50" s="3" t="s">
         <v>35</v>
       </c>
       <c r="G50" s="4" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="H50" s="4"/>
       <c r="I50" s="4" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="J50" s="4"/>
     </row>
     <row r="51" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="3">
-        <v>1904</v>
+        <v>1903</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="C51" s="3">
         <v>19</v>
       </c>
       <c r="D51" s="3">
-        <v>1904</v>
+        <v>1903</v>
       </c>
       <c r="E51" s="3"/>
       <c r="F51" s="3" t="s">
         <v>35</v>
       </c>
       <c r="G51" s="4" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="H51" s="4"/>
       <c r="I51" s="4" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="J51" s="4"/>
     </row>
     <row r="52" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="3">
-        <v>1905</v>
+        <v>1904</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="C52" s="3">
         <v>19</v>
       </c>
       <c r="D52" s="3">
-        <v>1905</v>
+        <v>1904</v>
       </c>
       <c r="E52" s="3"/>
       <c r="F52" s="3" t="s">
         <v>35</v>
       </c>
       <c r="G52" s="4" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="H52" s="4"/>
       <c r="I52" s="4" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="J52" s="4"/>
     </row>
     <row r="53" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="3">
-        <v>2</v>
+        <v>1905</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="C53" s="3">
-        <v>-1</v>
+        <v>19</v>
       </c>
       <c r="D53" s="3">
-        <v>2</v>
+        <v>1905</v>
       </c>
       <c r="E53" s="3"/>
       <c r="F53" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G53" s="4"/>
+        <v>35</v>
+      </c>
+      <c r="G53" s="4" t="s">
+        <v>123</v>
+      </c>
       <c r="H53" s="4"/>
       <c r="I53" s="4" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="J53" s="4"/>
     </row>
     <row r="54" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="3">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C54" s="3">
+        <v>-1</v>
+      </c>
+      <c r="D54" s="3">
         <v>2</v>
-      </c>
-      <c r="D54" s="3">
-        <v>21</v>
       </c>
       <c r="E54" s="3"/>
       <c r="F54" s="3" t="s">
@@ -4636,953 +4651,977 @@
       <c r="G54" s="4"/>
       <c r="H54" s="4"/>
       <c r="I54" s="4" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="J54" s="4"/>
     </row>
     <row r="55" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="3">
-        <v>2110</v>
+        <v>21</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C55" s="3">
+        <v>2</v>
+      </c>
+      <c r="D55" s="3">
         <v>21</v>
-      </c>
-      <c r="D55" s="3">
-        <v>2110</v>
       </c>
       <c r="E55" s="3"/>
       <c r="F55" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G55" s="4" t="s">
-        <v>128</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="G55" s="4"/>
       <c r="H55" s="4"/>
       <c r="I55" s="4" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="J55" s="4"/>
     </row>
     <row r="56" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="3">
-        <v>2111</v>
+        <v>2110</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="C56" s="3">
         <v>21</v>
       </c>
       <c r="D56" s="3">
-        <v>2111</v>
+        <v>2110</v>
       </c>
       <c r="E56" s="3"/>
       <c r="F56" s="3" t="s">
         <v>35</v>
       </c>
       <c r="G56" s="4" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="H56" s="4"/>
       <c r="I56" s="4" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="J56" s="4"/>
     </row>
     <row r="57" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="3">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="C57" s="3">
         <v>21</v>
       </c>
       <c r="D57" s="3">
-        <v>2112</v>
+        <v>2111</v>
       </c>
       <c r="E57" s="3"/>
       <c r="F57" s="3" t="s">
         <v>35</v>
       </c>
       <c r="G57" s="4" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H57" s="4"/>
       <c r="I57" s="4" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="J57" s="4"/>
     </row>
     <row r="58" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="3">
-        <v>2113</v>
+        <v>2112</v>
       </c>
       <c r="B58" s="4" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C58" s="3">
         <v>21</v>
       </c>
       <c r="D58" s="3">
-        <v>2113</v>
+        <v>2112</v>
       </c>
       <c r="E58" s="3"/>
       <c r="F58" s="3" t="s">
         <v>35</v>
       </c>
       <c r="G58" s="4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="H58" s="4"/>
       <c r="I58" s="4" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="J58" s="4"/>
     </row>
     <row r="59" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="3">
-        <v>22</v>
+        <v>2113</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C59" s="3">
-        <v>2</v>
+        <v>21</v>
       </c>
       <c r="D59" s="3">
-        <v>22</v>
+        <v>2113</v>
       </c>
       <c r="E59" s="3"/>
       <c r="F59" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G59" s="4"/>
+        <v>35</v>
+      </c>
+      <c r="G59" s="4" t="s">
+        <v>127</v>
+      </c>
       <c r="H59" s="4"/>
       <c r="I59" s="4" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="J59" s="4"/>
     </row>
     <row r="60" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="3">
-        <v>2201</v>
+        <v>22</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C60" s="3">
+        <v>2</v>
+      </c>
+      <c r="D60" s="3">
         <v>22</v>
-      </c>
-      <c r="D60" s="3">
-        <v>2201</v>
       </c>
       <c r="E60" s="3"/>
       <c r="F60" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G60" s="4" t="s">
-        <v>135</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="G60" s="4"/>
       <c r="H60" s="4"/>
       <c r="I60" s="4" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="J60" s="4"/>
     </row>
     <row r="61" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="3">
-        <v>2202</v>
+        <v>2201</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="C61" s="3">
         <v>22</v>
       </c>
       <c r="D61" s="3">
-        <v>2202</v>
+        <v>2201</v>
       </c>
       <c r="E61" s="3"/>
       <c r="F61" s="3" t="s">
         <v>35</v>
       </c>
       <c r="G61" s="4" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="H61" s="4"/>
       <c r="I61" s="4" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="J61" s="4"/>
     </row>
     <row r="62" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="3">
-        <v>2203</v>
+        <v>2202</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="C62" s="3">
         <v>22</v>
       </c>
       <c r="D62" s="3">
-        <v>2203</v>
+        <v>2202</v>
       </c>
       <c r="E62" s="3"/>
       <c r="F62" s="3" t="s">
         <v>35</v>
       </c>
       <c r="G62" s="4" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="H62" s="4"/>
       <c r="I62" s="4" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="J62" s="4"/>
     </row>
     <row r="63" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="3">
-        <v>23</v>
+        <v>2203</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="C63" s="3">
-        <v>2</v>
+        <v>22</v>
       </c>
       <c r="D63" s="3">
-        <v>23</v>
+        <v>2203</v>
       </c>
       <c r="E63" s="3"/>
       <c r="F63" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G63" s="4"/>
+        <v>35</v>
+      </c>
+      <c r="G63" s="4" t="s">
+        <v>138</v>
+      </c>
       <c r="H63" s="4"/>
       <c r="I63" s="4" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="J63" s="4"/>
     </row>
     <row r="64" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="3">
-        <v>2301</v>
+        <v>23</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="C64" s="3">
+        <v>2</v>
+      </c>
+      <c r="D64" s="3">
         <v>23</v>
-      </c>
-      <c r="D64" s="3">
-        <v>2301</v>
       </c>
       <c r="E64" s="3"/>
       <c r="F64" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G64" s="4" t="s">
-        <v>142</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="G64" s="4"/>
       <c r="H64" s="4"/>
       <c r="I64" s="4" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="J64" s="4"/>
     </row>
     <row r="65" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="3">
-        <v>2302</v>
+        <v>2301</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>71</v>
+        <v>140</v>
       </c>
       <c r="C65" s="3">
         <v>23</v>
       </c>
       <c r="D65" s="3">
-        <v>2302</v>
+        <v>2301</v>
       </c>
       <c r="E65" s="3"/>
       <c r="F65" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G65" s="4"/>
+        <v>35</v>
+      </c>
+      <c r="G65" s="4" t="s">
+        <v>141</v>
+      </c>
       <c r="H65" s="4"/>
       <c r="I65" s="4" t="s">
-        <v>71</v>
+        <v>140</v>
       </c>
       <c r="J65" s="4"/>
     </row>
     <row r="66" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A66" s="3">
-        <v>23021</v>
+        <v>2302</v>
       </c>
       <c r="B66" s="4" t="s">
-        <v>143</v>
+        <v>71</v>
       </c>
       <c r="C66" s="3">
+        <v>23</v>
+      </c>
+      <c r="D66" s="3">
         <v>2302</v>
-      </c>
-      <c r="D66" s="3">
-        <v>23021</v>
       </c>
       <c r="E66" s="3"/>
       <c r="F66" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G66" s="4" t="s">
-        <v>144</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="G66" s="4"/>
       <c r="H66" s="4"/>
       <c r="I66" s="4" t="s">
-        <v>143</v>
+        <v>71</v>
       </c>
       <c r="J66" s="4"/>
     </row>
     <row r="67" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="3">
-        <v>23022</v>
+        <v>23021</v>
       </c>
       <c r="B67" s="4" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="C67" s="3">
         <v>2302</v>
       </c>
       <c r="D67" s="3">
-        <v>23022</v>
+        <v>23021</v>
       </c>
       <c r="E67" s="3"/>
       <c r="F67" s="3" t="s">
         <v>35</v>
       </c>
       <c r="G67" s="4" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="H67" s="4"/>
       <c r="I67" s="4" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="J67" s="4"/>
     </row>
     <row r="68" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A68" s="3">
-        <v>2303</v>
+        <v>23022</v>
       </c>
       <c r="B68" s="4" t="s">
-        <v>70</v>
+        <v>144</v>
       </c>
       <c r="C68" s="3">
-        <v>23</v>
+        <v>2302</v>
       </c>
       <c r="D68" s="3">
-        <v>2303</v>
+        <v>23022</v>
       </c>
       <c r="E68" s="3"/>
       <c r="F68" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G68" s="4"/>
+        <v>35</v>
+      </c>
+      <c r="G68" s="4" t="s">
+        <v>145</v>
+      </c>
       <c r="H68" s="4"/>
       <c r="I68" s="4" t="s">
-        <v>70</v>
+        <v>144</v>
       </c>
       <c r="J68" s="4"/>
     </row>
     <row r="69" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="3">
-        <v>23031</v>
+        <v>2303</v>
       </c>
       <c r="B69" s="4" t="s">
-        <v>147</v>
+        <v>70</v>
       </c>
       <c r="C69" s="3">
+        <v>23</v>
+      </c>
+      <c r="D69" s="3">
         <v>2303</v>
-      </c>
-      <c r="D69" s="3">
-        <v>23031</v>
       </c>
       <c r="E69" s="3"/>
       <c r="F69" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G69" s="4" t="s">
-        <v>148</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="G69" s="4"/>
       <c r="H69" s="4"/>
       <c r="I69" s="4" t="s">
-        <v>147</v>
+        <v>70</v>
       </c>
       <c r="J69" s="4"/>
     </row>
     <row r="70" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A70" s="3">
-        <v>23032</v>
+        <v>23031</v>
       </c>
       <c r="B70" s="4" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="C70" s="3">
         <v>2303</v>
       </c>
       <c r="D70" s="3">
-        <v>23032</v>
+        <v>23031</v>
       </c>
       <c r="E70" s="3"/>
       <c r="F70" s="3" t="s">
         <v>35</v>
       </c>
       <c r="G70" s="4" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="H70" s="4"/>
       <c r="I70" s="4" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="J70" s="4"/>
     </row>
     <row r="71" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="3">
-        <v>23033</v>
+        <v>23032</v>
       </c>
       <c r="B71" s="4" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="C71" s="3">
         <v>2303</v>
       </c>
       <c r="D71" s="3">
-        <v>23033</v>
+        <v>23032</v>
       </c>
       <c r="E71" s="3"/>
       <c r="F71" s="3" t="s">
         <v>35</v>
       </c>
       <c r="G71" s="4" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="H71" s="4"/>
       <c r="I71" s="4" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="J71" s="4"/>
     </row>
     <row r="72" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A72" s="3">
-        <v>23034</v>
+        <v>23033</v>
       </c>
       <c r="B72" s="4" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="C72" s="3">
         <v>2303</v>
       </c>
       <c r="D72" s="3">
-        <v>23034</v>
+        <v>23033</v>
       </c>
       <c r="E72" s="3"/>
       <c r="F72" s="3" t="s">
         <v>35</v>
       </c>
       <c r="G72" s="4" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
       <c r="H72" s="4"/>
       <c r="I72" s="4" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="J72" s="4"/>
     </row>
     <row r="73" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="3">
-        <v>23035</v>
+        <v>23034</v>
       </c>
       <c r="B73" s="4" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C73" s="3">
         <v>2303</v>
       </c>
       <c r="D73" s="3">
-        <v>23035</v>
+        <v>23034</v>
       </c>
       <c r="E73" s="3"/>
       <c r="F73" s="3" t="s">
         <v>35</v>
       </c>
       <c r="G73" s="4" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
       <c r="H73" s="4"/>
       <c r="I73" s="4" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="J73" s="4"/>
     </row>
     <row r="74" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A74" s="3">
-        <v>2304</v>
+        <v>23035</v>
       </c>
       <c r="B74" s="4" t="s">
-        <v>103</v>
+        <v>154</v>
       </c>
       <c r="C74" s="3">
-        <v>23</v>
+        <v>2303</v>
       </c>
       <c r="D74" s="3">
-        <v>2304</v>
+        <v>23035</v>
       </c>
       <c r="E74" s="3"/>
       <c r="F74" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G74" s="4"/>
+        <v>35</v>
+      </c>
+      <c r="G74" s="4" t="s">
+        <v>155</v>
+      </c>
       <c r="H74" s="4"/>
       <c r="I74" s="4" t="s">
-        <v>103</v>
+        <v>154</v>
       </c>
       <c r="J74" s="4"/>
     </row>
     <row r="75" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="3">
-        <v>23041</v>
-      </c>
-      <c r="B75" s="11" t="s">
-        <v>186</v>
+        <v>2304</v>
+      </c>
+      <c r="B75" s="4" t="s">
+        <v>102</v>
       </c>
       <c r="C75" s="3">
+        <v>23</v>
+      </c>
+      <c r="D75" s="3">
         <v>2304</v>
-      </c>
-      <c r="D75" s="3">
-        <v>23041</v>
       </c>
       <c r="E75" s="3"/>
       <c r="F75" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G75" s="4" t="s">
-        <v>158</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="G75" s="4"/>
       <c r="H75" s="4"/>
       <c r="I75" s="4" t="s">
-        <v>157</v>
+        <v>102</v>
       </c>
       <c r="J75" s="4"/>
     </row>
     <row r="76" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A76" s="3">
-        <v>23042</v>
-      </c>
-      <c r="B76" s="4" t="s">
-        <v>159</v>
+        <v>23041</v>
+      </c>
+      <c r="B76" s="11" t="s">
+        <v>185</v>
       </c>
       <c r="C76" s="3">
         <v>2304</v>
       </c>
       <c r="D76" s="3">
-        <v>23042</v>
+        <v>23041</v>
       </c>
       <c r="E76" s="3"/>
       <c r="F76" s="3" t="s">
         <v>35</v>
       </c>
       <c r="G76" s="4" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="H76" s="4"/>
       <c r="I76" s="4" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="J76" s="4"/>
     </row>
     <row r="77" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="3">
-        <v>23043</v>
+        <v>23042</v>
       </c>
       <c r="B77" s="4" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="C77" s="3">
         <v>2304</v>
       </c>
       <c r="D77" s="3">
-        <v>23043</v>
+        <v>23042</v>
       </c>
       <c r="E77" s="3"/>
       <c r="F77" s="3" t="s">
         <v>35</v>
       </c>
       <c r="G77" s="4" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="H77" s="4"/>
       <c r="I77" s="4" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="J77" s="4"/>
     </row>
     <row r="78" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A78" s="3">
-        <v>23044</v>
+        <v>23043</v>
       </c>
       <c r="B78" s="4" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="C78" s="3">
         <v>2304</v>
       </c>
       <c r="D78" s="3">
-        <v>23044</v>
+        <v>23043</v>
       </c>
       <c r="E78" s="3"/>
       <c r="F78" s="3" t="s">
         <v>35</v>
       </c>
       <c r="G78" s="4" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="H78" s="4"/>
       <c r="I78" s="4" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
       <c r="J78" s="4"/>
     </row>
     <row r="79" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A79" s="3">
-        <v>23045</v>
-      </c>
-      <c r="B79" s="11" t="s">
-        <v>185</v>
+        <v>23044</v>
+      </c>
+      <c r="B79" s="4" t="s">
+        <v>162</v>
       </c>
       <c r="C79" s="3">
         <v>2304</v>
       </c>
       <c r="D79" s="3">
-        <v>23045</v>
+        <v>23044</v>
       </c>
       <c r="E79" s="3"/>
       <c r="F79" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G79" s="6" t="s">
-        <v>165</v>
+      <c r="G79" s="4" t="s">
+        <v>163</v>
       </c>
       <c r="H79" s="4"/>
-      <c r="I79" s="11" t="s">
-        <v>185</v>
+      <c r="I79" s="4" t="s">
+        <v>162</v>
       </c>
       <c r="J79" s="4"/>
     </row>
     <row r="80" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A80" s="3">
-        <v>23046</v>
-      </c>
-      <c r="B80" s="4" t="s">
-        <v>166</v>
+        <v>23045</v>
+      </c>
+      <c r="B80" s="11" t="s">
+        <v>184</v>
       </c>
       <c r="C80" s="3">
         <v>2304</v>
       </c>
       <c r="D80" s="3">
-        <v>23046</v>
+        <v>23045</v>
       </c>
       <c r="E80" s="3"/>
       <c r="F80" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G80" s="4" t="s">
-        <v>167</v>
+      <c r="G80" s="6" t="s">
+        <v>164</v>
       </c>
       <c r="H80" s="4"/>
-      <c r="I80" s="4" t="s">
-        <v>166</v>
+      <c r="I80" s="11" t="s">
+        <v>184</v>
       </c>
       <c r="J80" s="4"/>
     </row>
     <row r="81" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A81" s="3">
-        <v>2307</v>
+        <v>23046</v>
       </c>
       <c r="B81" s="4" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="C81" s="3">
-        <v>23</v>
+        <v>2304</v>
       </c>
       <c r="D81" s="3">
-        <v>2307</v>
+        <v>23046</v>
       </c>
       <c r="E81" s="3"/>
       <c r="F81" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G81" s="3"/>
-      <c r="H81" s="3"/>
+        <v>35</v>
+      </c>
+      <c r="G81" s="4" t="s">
+        <v>166</v>
+      </c>
+      <c r="H81" s="4"/>
       <c r="I81" s="4" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="J81" s="4"/>
     </row>
     <row r="82" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="3">
-        <v>23071</v>
+        <v>2307</v>
       </c>
       <c r="B82" s="4" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="C82" s="3">
+        <v>23</v>
+      </c>
+      <c r="D82" s="3">
         <v>2307</v>
-      </c>
-      <c r="D82" s="3">
-        <v>23071</v>
       </c>
       <c r="E82" s="3"/>
       <c r="F82" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G82" s="4" t="s">
-        <v>170</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="G82" s="3"/>
       <c r="H82" s="3"/>
       <c r="I82" s="4" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="J82" s="4"/>
     </row>
     <row r="83" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="3">
-        <v>23072</v>
+        <v>23071</v>
       </c>
       <c r="B83" s="4" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="C83" s="3">
         <v>2307</v>
       </c>
       <c r="D83" s="3">
-        <v>23072</v>
+        <v>23071</v>
       </c>
       <c r="E83" s="3"/>
       <c r="F83" s="3" t="s">
         <v>35</v>
       </c>
       <c r="G83" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="H83" s="4"/>
+        <v>169</v>
+      </c>
+      <c r="H83" s="3"/>
       <c r="I83" s="4" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="J83" s="4"/>
     </row>
     <row r="84" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="3">
-        <v>23073</v>
+        <v>23072</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="C84" s="3">
         <v>2307</v>
       </c>
       <c r="D84" s="3">
-        <v>23073</v>
+        <v>23072</v>
       </c>
       <c r="E84" s="3"/>
       <c r="F84" s="3" t="s">
         <v>35</v>
       </c>
       <c r="G84" s="4" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="H84" s="4"/>
       <c r="I84" s="4" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="J84" s="4"/>
     </row>
     <row r="85" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="3">
-        <v>24</v>
+        <v>23073</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C85" s="3">
-        <v>2</v>
+        <v>2307</v>
       </c>
       <c r="D85" s="3">
-        <v>24</v>
-      </c>
-      <c r="E85" s="4"/>
+        <v>23073</v>
+      </c>
+      <c r="E85" s="3"/>
       <c r="F85" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G85" s="4"/>
+        <v>35</v>
+      </c>
+      <c r="G85" s="4" t="s">
+        <v>173</v>
+      </c>
       <c r="H85" s="4"/>
       <c r="I85" s="4" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="J85" s="4"/>
     </row>
     <row r="86" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="3">
-        <v>2401</v>
+        <v>24</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C86" s="3">
+        <v>2</v>
+      </c>
+      <c r="D86" s="3">
         <v>24</v>
-      </c>
-      <c r="D86" s="3">
-        <v>2401</v>
       </c>
       <c r="E86" s="4"/>
       <c r="F86" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G86" s="4" t="s">
-        <v>177</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="G86" s="4"/>
       <c r="H86" s="4"/>
       <c r="I86" s="4" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="J86" s="4"/>
     </row>
     <row r="87" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="3">
-        <v>25</v>
+        <v>2401</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="C87" s="3">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="D87" s="3">
-        <v>25</v>
+        <v>2401</v>
       </c>
       <c r="E87" s="4"/>
       <c r="F87" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G87" s="4"/>
+        <v>35</v>
+      </c>
+      <c r="G87" s="4" t="s">
+        <v>176</v>
+      </c>
       <c r="H87" s="4"/>
       <c r="I87" s="4" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="J87" s="4"/>
     </row>
     <row r="88" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="3">
-        <v>2501</v>
+        <v>25</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="C88" s="3">
+        <v>2</v>
+      </c>
+      <c r="D88" s="3">
         <v>25</v>
       </c>
-      <c r="D88" s="3">
-        <v>2501</v>
-      </c>
-      <c r="E88" s="3"/>
+      <c r="E88" s="4"/>
       <c r="F88" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G88" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="H88" s="3"/>
+        <v>32</v>
+      </c>
+      <c r="G88" s="4"/>
+      <c r="H88" s="4"/>
       <c r="I88" s="4" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
       <c r="J88" s="4"/>
     </row>
     <row r="89" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="3">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>180</v>
+        <v>174</v>
       </c>
       <c r="C89" s="3">
         <v>25</v>
       </c>
       <c r="D89" s="3">
-        <v>2502</v>
+        <v>2501</v>
       </c>
       <c r="E89" s="3"/>
       <c r="F89" s="3" t="s">
         <v>35</v>
       </c>
       <c r="G89" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="H89" s="5"/>
-      <c r="I89" s="5" t="s">
-        <v>180</v>
-      </c>
-      <c r="J89" s="5"/>
+        <v>178</v>
+      </c>
+      <c r="H89" s="3"/>
+      <c r="I89" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="J89" s="4"/>
     </row>
     <row r="90" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A90" s="3">
-        <v>26</v>
+        <v>2502</v>
       </c>
       <c r="B90" s="4" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="C90" s="3">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="D90" s="3">
-        <v>26</v>
+        <v>2502</v>
       </c>
       <c r="E90" s="3"/>
       <c r="F90" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G90" s="4"/>
-      <c r="H90" s="4"/>
-      <c r="I90" s="4" t="s">
-        <v>182</v>
-      </c>
-      <c r="J90" s="4"/>
+        <v>35</v>
+      </c>
+      <c r="G90" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="H90" s="5"/>
+      <c r="I90" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="J90" s="5"/>
     </row>
     <row r="91" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A91" s="3">
-        <v>2601</v>
+        <v>26</v>
       </c>
       <c r="B91" s="4" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="C91" s="3">
+        <v>2</v>
+      </c>
+      <c r="D91" s="3">
         <v>26</v>
       </c>
-      <c r="D91" s="3">
-        <v>2601</v>
-      </c>
-      <c r="E91" s="4"/>
+      <c r="E91" s="3"/>
       <c r="F91" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G91" s="4" t="s">
-        <v>184</v>
-      </c>
+        <v>32</v>
+      </c>
+      <c r="G91" s="4"/>
       <c r="H91" s="4"/>
       <c r="I91" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="J91" s="4"/>
+    </row>
+    <row r="92" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A92" s="3">
+        <v>2601</v>
+      </c>
+      <c r="B92" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="C92" s="3">
+        <v>26</v>
+      </c>
+      <c r="D92" s="3">
+        <v>2601</v>
+      </c>
+      <c r="E92" s="4"/>
+      <c r="F92" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G92" s="4" t="s">
         <v>183</v>
       </c>
-      <c r="J91" s="4"/>
+      <c r="H92" s="4"/>
+      <c r="I92" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="J92" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="6" type="noConversion"/>

</xml_diff>

<commit_message>
#176 CIB老化 1. CIB老化 2. 修改stage mock bf df center position, x y direction， bf <=> stage , df  <=> stage 3. aod delay bug fix 4. review保存日志的时候文件名架构设计OK
</commit_message>
<xml_diff>
--- a/Sources/Cuga-Calibration-Solution/Assets/Data/InitData.xlsx
+++ b/Sources/Cuga-Calibration-Solution/Assets/Data/InitData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\RiderProjects\semix\kaizhi.xuan\netcore_semix_cuga_calibration\Sources\Cuga-Calibration-Solution\Assets\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1EA6A74-647F-4886-9478-CA449C53CCA8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{551E876A-AFD7-4EAE-A534-2BABF1A44F2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="500" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="414" uniqueCount="184">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="421" uniqueCount="187">
   <si>
     <t>Id</t>
   </si>
@@ -646,12 +646,24 @@
   <si>
     <t>CugaCalibration.ViewModels.ApplicationAboutWindowViewModel</t>
   </si>
+  <si>
+    <t>CIB</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>Aging</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
+  <si>
+    <t>CugaCalibration.ViewModels.Common.Windows.Tools.CIB.CIBAgingWindowViewModel</t>
+    <phoneticPr fontId="5" type="noConversion"/>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -687,6 +699,13 @@
     </font>
     <font>
       <sz val="9"/>
+      <name val="等线"/>
+      <family val="3"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
       <name val="等线"/>
       <family val="3"/>
       <charset val="134"/>
@@ -763,7 +782,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -793,6 +812,9 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -3211,7 +3233,7 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
-  <dimension ref="A1:J89"/>
+  <dimension ref="A1:J91"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.625" style="1" customWidth="1"/>
@@ -5304,66 +5326,66 @@
     </row>
     <row r="82" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A82" s="3">
+        <v>2305</v>
+      </c>
+      <c r="B82" s="10" t="s">
+        <v>184</v>
+      </c>
+      <c r="C82" s="3">
         <v>23</v>
       </c>
-      <c r="B82" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="C82" s="3">
-        <v>2</v>
-      </c>
       <c r="D82" s="3">
-        <v>23</v>
-      </c>
-      <c r="E82" s="4"/>
+        <v>2305</v>
+      </c>
+      <c r="E82" s="3"/>
       <c r="F82" s="3" t="s">
         <v>32</v>
       </c>
       <c r="G82" s="4"/>
       <c r="H82" s="4"/>
-      <c r="I82" s="4" t="s">
-        <v>172</v>
+      <c r="I82" s="10" t="s">
+        <v>184</v>
       </c>
       <c r="J82" s="4"/>
     </row>
     <row r="83" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A83" s="3">
-        <v>2301</v>
-      </c>
-      <c r="B83" s="4" t="s">
-        <v>173</v>
+        <v>23051</v>
+      </c>
+      <c r="B83" s="10" t="s">
+        <v>185</v>
       </c>
       <c r="C83" s="3">
-        <v>23</v>
+        <v>2305</v>
       </c>
       <c r="D83" s="3">
-        <v>2301</v>
-      </c>
-      <c r="E83" s="4"/>
+        <v>23051</v>
+      </c>
+      <c r="E83" s="3"/>
       <c r="F83" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="G83" s="4" t="s">
-        <v>174</v>
+      <c r="G83" s="10" t="s">
+        <v>186</v>
       </c>
       <c r="H83" s="4"/>
-      <c r="I83" s="4" t="s">
-        <v>173</v>
+      <c r="I83" s="10" t="s">
+        <v>185</v>
       </c>
       <c r="J83" s="4"/>
     </row>
     <row r="84" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A84" s="3">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B84" s="4" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="C84" s="3">
         <v>2</v>
       </c>
       <c r="D84" s="3">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E84" s="4"/>
       <c r="F84" s="3" t="s">
@@ -5372,137 +5394,187 @@
       <c r="G84" s="4"/>
       <c r="H84" s="4"/>
       <c r="I84" s="4" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="J84" s="4"/>
     </row>
     <row r="85" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A85" s="3">
-        <v>2401</v>
+        <v>2301</v>
       </c>
       <c r="B85" s="4" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="C85" s="3">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D85" s="3">
-        <v>2401</v>
-      </c>
-      <c r="E85" s="3"/>
+        <v>2301</v>
+      </c>
+      <c r="E85" s="4"/>
       <c r="F85" s="3" t="s">
         <v>35</v>
       </c>
       <c r="G85" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="H85" s="3"/>
+        <v>174</v>
+      </c>
+      <c r="H85" s="4"/>
       <c r="I85" s="4" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="J85" s="4"/>
     </row>
     <row r="86" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A86" s="3">
-        <v>2402</v>
+        <v>24</v>
       </c>
       <c r="B86" s="4" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="C86" s="3">
+        <v>2</v>
+      </c>
+      <c r="D86" s="3">
         <v>24</v>
       </c>
-      <c r="D86" s="3">
-        <v>2402</v>
-      </c>
-      <c r="E86" s="3"/>
+      <c r="E86" s="4"/>
       <c r="F86" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="G86" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="H86" s="5"/>
-      <c r="I86" s="5" t="s">
-        <v>177</v>
-      </c>
-      <c r="J86" s="5"/>
+        <v>32</v>
+      </c>
+      <c r="G86" s="4"/>
+      <c r="H86" s="4"/>
+      <c r="I86" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="J86" s="4"/>
     </row>
     <row r="87" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A87" s="3">
-        <v>2403</v>
+        <v>2401</v>
       </c>
       <c r="B87" s="4" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="C87" s="3">
         <v>24</v>
       </c>
       <c r="D87" s="3">
-        <v>2403</v>
+        <v>2401</v>
       </c>
       <c r="E87" s="3"/>
       <c r="F87" s="3" t="s">
         <v>35</v>
       </c>
       <c r="G87" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="H87" s="4"/>
+        <v>176</v>
+      </c>
+      <c r="H87" s="3"/>
       <c r="I87" s="4" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="J87" s="4"/>
     </row>
     <row r="88" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A88" s="3">
-        <v>25</v>
+        <v>2402</v>
       </c>
       <c r="B88" s="4" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="C88" s="3">
-        <v>2</v>
+        <v>24</v>
       </c>
       <c r="D88" s="3">
-        <v>25</v>
+        <v>2402</v>
       </c>
       <c r="E88" s="3"/>
       <c r="F88" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="G88" s="4"/>
-      <c r="H88" s="4"/>
-      <c r="I88" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="J88" s="4"/>
+        <v>35</v>
+      </c>
+      <c r="G88" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="H88" s="5"/>
+      <c r="I88" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="J88" s="5"/>
     </row>
     <row r="89" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A89" s="3">
-        <v>2501</v>
+        <v>2403</v>
       </c>
       <c r="B89" s="4" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="C89" s="3">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D89" s="3">
-        <v>2501</v>
-      </c>
-      <c r="E89" s="4"/>
+        <v>2403</v>
+      </c>
+      <c r="E89" s="3"/>
       <c r="F89" s="3" t="s">
         <v>35</v>
       </c>
       <c r="G89" s="4" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="H89" s="4"/>
       <c r="I89" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="J89" s="4"/>
+    </row>
+    <row r="90" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A90" s="3">
+        <v>25</v>
+      </c>
+      <c r="B90" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="C90" s="3">
+        <v>2</v>
+      </c>
+      <c r="D90" s="3">
+        <v>25</v>
+      </c>
+      <c r="E90" s="3"/>
+      <c r="F90" s="3" t="s">
+        <v>32</v>
+      </c>
+      <c r="G90" s="4"/>
+      <c r="H90" s="4"/>
+      <c r="I90" s="4" t="s">
+        <v>181</v>
+      </c>
+      <c r="J90" s="4"/>
+    </row>
+    <row r="91" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A91" s="3">
+        <v>2501</v>
+      </c>
+      <c r="B91" s="4" t="s">
         <v>182</v>
       </c>
-      <c r="J89" s="4"/>
+      <c r="C91" s="3">
+        <v>25</v>
+      </c>
+      <c r="D91" s="3">
+        <v>2501</v>
+      </c>
+      <c r="E91" s="4"/>
+      <c r="F91" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="G91" s="4" t="s">
+        <v>183</v>
+      </c>
+      <c r="H91" s="4"/>
+      <c r="I91" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="J91" s="4"/>
     </row>
   </sheetData>
   <phoneticPr fontId="5" type="noConversion"/>

</xml_diff>